<commit_message>
feat: permanent champion-challenger lifecycle and evidence provenance
- Establish permanent champion-challenger production architecture across 21 supported markets
- Enforce evidence provenance (live_prospective, pit_replay, historical_backtest, synthetic)
- Introduce ChallengerBuildStatus and NextAction research control plane in qualification registry
- Implement fail-isolated prediction execution and atomic promotion / rollback pointers
- Add complete 90-test lifecycle, promotion, contract, and provenance verification suite
- Promote mlb-structural-v10-frozen to MLB Total production champion with totals-v3 rollback
</commit_message>
<xml_diff>
--- a/data/auto_buyer_picks.xlsx
+++ b/data/auto_buyer_picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DP54" headerRowCount="1">
-  <autoFilter ref="A1:DP54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DP51" headerRowCount="1">
+  <autoFilter ref="A1:DP51"/>
   <tableColumns count="120">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -779,19 +779,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$54)</f>
+        <f>COUNTA('Picks'!$A$2:$A$51)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$54,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$51,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$54,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$51,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$54,"settled",'Picks'!$V$2:$V$54,"win")+COUNTIFS('Picks'!$U$2:$U$54,"settled",'Picks'!$V$2:$V$54,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$51,"settled",'Picks'!$V$2:$V$51,"win")+COUNTIFS('Picks'!$U$2:$U$51,"settled",'Picks'!$V$2:$V$51,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -819,19 +819,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$54,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$51,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$54,"&gt;0",'Picks'!$V$2:$V$54,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$54,"&gt;0",'Picks'!$V$2:$V$54,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$51,"&gt;0",'Picks'!$V$2:$V$51,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$51,"&gt;0",'Picks'!$V$2:$V$51,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$54,"&gt;0",'Picks'!$V$2:$V$54,"win")/(COUNTIFS('Picks'!$BX$2:$BX$54,"&gt;0",'Picks'!$V$2:$V$54,"win")+COUNTIFS('Picks'!$BX$2:$BX$54,"&gt;0",'Picks'!$V$2:$V$54,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$51,"&gt;0",'Picks'!$V$2:$V$51,"win")/(COUNTIFS('Picks'!$BX$2:$BX$51,"&gt;0",'Picks'!$V$2:$V$51,"win")+COUNTIFS('Picks'!$BX$2:$BX$51,"&gt;0",'Picks'!$V$2:$V$51,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$54)/SUM('Picks'!$BX$2:$BX$54),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$51)/SUM('Picks'!$BX$2:$BX$51),0)</f>
         <v/>
       </c>
     </row>
@@ -859,19 +859,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$54)</f>
+        <f>SUM('Picks'!$BY$2:$BY$51)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$54,"&lt;&gt;",'Picks'!$AB$2:$AB$54),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$51,"&lt;&gt;",'Picks'!$AB$2:$AB$51),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$54,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$54,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$51,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$51,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$54,'Picks'!$AM$2:$AM$54,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$51,'Picks'!$AM$2:$AM$51,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -926,15 +926,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A14,'Picks'!$U$2:$U$54,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A14,'Picks'!$U$2:$U$51,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A14,'Picks'!$U$2:$U$54,"settled",'Picks'!$V$2:$V$54,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A14,'Picks'!$U$2:$U$51,"settled",'Picks'!$V$2:$V$51,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A14,'Picks'!$U$2:$U$54,"settled",'Picks'!$V$2:$V$54,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A14,'Picks'!$U$2:$U$51,"settled",'Picks'!$V$2:$V$51,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -942,11 +942,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$54,'Picks'!$H$2:$H$54,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$51,'Picks'!$H$2:$H$51,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$54,'Picks'!$H$2:$H$54,$A14,'Picks'!$U$2:$U$54,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$51,'Picks'!$H$2:$H$51,$A14,'Picks'!$U$2:$U$51,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -957,15 +957,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A15,'Picks'!$U$2:$U$54,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A15,'Picks'!$U$2:$U$51,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A15,'Picks'!$U$2:$U$54,"settled",'Picks'!$V$2:$V$54,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A15,'Picks'!$U$2:$U$51,"settled",'Picks'!$V$2:$V$51,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A15,'Picks'!$U$2:$U$54,"settled",'Picks'!$V$2:$V$54,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A15,'Picks'!$U$2:$U$51,"settled",'Picks'!$V$2:$V$51,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -973,11 +973,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$54,'Picks'!$H$2:$H$54,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$51,'Picks'!$H$2:$H$51,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$54,'Picks'!$H$2:$H$54,$A15,'Picks'!$U$2:$U$54,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$51,'Picks'!$H$2:$H$51,$A15,'Picks'!$U$2:$U$51,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -988,15 +988,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A16,'Picks'!$U$2:$U$54,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A16,'Picks'!$U$2:$U$51,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A16,'Picks'!$U$2:$U$54,"settled",'Picks'!$V$2:$V$54,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A16,'Picks'!$U$2:$U$51,"settled",'Picks'!$V$2:$V$51,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$54,$A16,'Picks'!$U$2:$U$54,"settled",'Picks'!$V$2:$V$54,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$51,$A16,'Picks'!$U$2:$U$51,"settled",'Picks'!$V$2:$V$51,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -1004,11 +1004,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$54,'Picks'!$H$2:$H$54,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$51,'Picks'!$H$2:$H$51,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$54,'Picks'!$H$2:$H$54,$A16,'Picks'!$U$2:$U$54,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$51,'Picks'!$H$2:$H$51,$A16,'Picks'!$U$2:$U$51,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DP54"/>
+  <dimension ref="A1:DP51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7069,7 +7069,7 @@
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>3514efbef314473c</t>
+          <t>6a99a099dcfa4a08</t>
         </is>
       </c>
       <c r="B27" s="24" t="inlineStr">
@@ -7079,37 +7079,37 @@
       </c>
       <c r="C27" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T00:05Z</t>
+          <t>2026-08-31T15:00Z</t>
         </is>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>tsc-mlb-ath-tex-2026-08-31-7pt5</t>
+          <t>aec-wta-mansaw-panudv-2026-08-30</t>
         </is>
       </c>
       <c r="E27" s="24" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>TENNIS</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Panna Udvardy</t>
         </is>
       </c>
       <c r="G27" s="24" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Mananchaya Sawangkaew</t>
         </is>
       </c>
       <c r="H27" s="24" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>moneyline</t>
         </is>
       </c>
       <c r="I27" s="24" t="inlineStr">
         <is>
-          <t>over</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J27" s="25" t="n"/>
@@ -7119,53 +7119,59 @@
         </is>
       </c>
       <c r="L27" s="26" t="n">
-        <v>104</v>
+        <v>156</v>
       </c>
       <c r="M27" s="27" t="n">
-        <v>2.04</v>
+        <v>2.56</v>
       </c>
       <c r="N27" s="28" t="n">
-        <v>0.495</v>
+        <v>0.3906</v>
       </c>
       <c r="O27" s="28" t="n">
-        <v>0.5393</v>
+        <v>0.5028</v>
       </c>
       <c r="P27" s="28" t="n"/>
       <c r="Q27" s="28" t="n">
-        <v>0.0443</v>
+        <v>0.1128</v>
       </c>
       <c r="R27" s="26" t="n"/>
       <c r="S27" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T27" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U27" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V27" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W27" s="26" t="n"/>
+      <c r="X27" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="T27" s="24" t="inlineStr">
-        <is>
-          <t>measured-edge-totals-v3</t>
-        </is>
-      </c>
-      <c r="U27" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V27" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="W27" s="26" t="n"/>
-      <c r="X27" s="26" t="n"/>
       <c r="Y27" s="25" t="n"/>
       <c r="Z27" s="26" t="n"/>
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
       <c r="AC27" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD27" s="24" t="n"/>
+        <v>-1.5</v>
+      </c>
+      <c r="AD27" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-31T18:41:38.707356Z</t>
+        </is>
+      </c>
       <c r="AE27" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VGABJQRKDK on tsc-mlb-ath-tex-2026-08-31-7pt5 (long)</t>
+          <t>Auto-Buyer order C6VFDE70CKDN on aec-wta-mansaw-panudv-2026-08-30 (short)</t>
         </is>
       </c>
       <c r="AF27" s="31" t="n"/>
@@ -7275,7 +7281,7 @@
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>1366137b9f7f4139</t>
+          <t>8b833b3bf6574b26</t>
         </is>
       </c>
       <c r="B28" s="24" t="inlineStr">
@@ -7285,37 +7291,37 @@
       </c>
       <c r="C28" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T00:40Z</t>
+          <t>2026-08-31T17:00Z</t>
         </is>
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>tsc-mlb-bal-col-2026-08-31-10pt5</t>
+          <t>aec-wta-tamzid-martim-2026-08-30</t>
         </is>
       </c>
       <c r="E28" s="24" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>TENNIS</t>
         </is>
       </c>
       <c r="F28" s="24" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Maria Timofeeva</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Tamara Zidansek</t>
         </is>
       </c>
       <c r="H28" s="24" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>moneyline</t>
         </is>
       </c>
       <c r="I28" s="24" t="inlineStr">
         <is>
-          <t>under</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J28" s="25" t="n"/>
@@ -7325,28 +7331,28 @@
         </is>
       </c>
       <c r="L28" s="26" t="n">
-        <v>113</v>
+        <v>194</v>
       </c>
       <c r="M28" s="27" t="n">
-        <v>2.13</v>
+        <v>2.94</v>
       </c>
       <c r="N28" s="28" t="n">
-        <v>0.4695</v>
+        <v>0.3401</v>
       </c>
       <c r="O28" s="28" t="n">
-        <v>0.5286</v>
+        <v>0.5261</v>
       </c>
       <c r="P28" s="28" t="n"/>
       <c r="Q28" s="28" t="n">
-        <v>0.0586</v>
+        <v>0.1861</v>
       </c>
       <c r="R28" s="26" t="n"/>
       <c r="S28" s="29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T28" s="24" t="inlineStr">
         <is>
-          <t>measured-edge-totals-v3</t>
+          <t>tennis-surface-elo-v1</t>
         </is>
       </c>
       <c r="U28" s="24" t="inlineStr">
@@ -7371,7 +7377,7 @@
       <c r="AD28" s="24" t="n"/>
       <c r="AE28" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFYJRFCKDF on tsc-mlb-bal-col-2026-08-31-10pt5 (short)</t>
+          <t>Auto-Buyer order C6VFNH8ZYKDJ on aec-wta-tamzid-martim-2026-08-30 (long)</t>
         </is>
       </c>
       <c r="AF28" s="31" t="n"/>
@@ -7481,7 +7487,7 @@
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>6a99a099dcfa4a08</t>
+          <t>55dfd65193ae4c3d</t>
         </is>
       </c>
       <c r="B29" s="24" t="inlineStr">
@@ -7496,7 +7502,7 @@
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>aec-wta-mansaw-panudv-2026-08-30</t>
+          <t>aec-atp-valvac-alekov-2026-08-30</t>
         </is>
       </c>
       <c r="E29" s="24" t="inlineStr">
@@ -7506,12 +7512,12 @@
       </c>
       <c r="F29" s="24" t="inlineStr">
         <is>
-          <t>Panna Udvardy</t>
+          <t>Aleksandar Kovacevic</t>
         </is>
       </c>
       <c r="G29" s="24" t="inlineStr">
         <is>
-          <t>Mananchaya Sawangkaew</t>
+          <t>Valentin Vacherot</t>
         </is>
       </c>
       <c r="H29" s="24" t="inlineStr">
@@ -7521,7 +7527,7 @@
       </c>
       <c r="I29" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J29" s="25" t="n"/>
@@ -7531,20 +7537,20 @@
         </is>
       </c>
       <c r="L29" s="26" t="n">
-        <v>156</v>
+        <v>-108</v>
       </c>
       <c r="M29" s="27" t="n">
-        <v>2.56</v>
+        <v>1.9259</v>
       </c>
       <c r="N29" s="28" t="n">
-        <v>0.3906</v>
+        <v>0.5192</v>
       </c>
       <c r="O29" s="28" t="n">
-        <v>0.5028</v>
+        <v>0.6385</v>
       </c>
       <c r="P29" s="28" t="n"/>
       <c r="Q29" s="28" t="n">
-        <v>0.1128</v>
+        <v>0.1185</v>
       </c>
       <c r="R29" s="26" t="n"/>
       <c r="S29" s="29" t="n">
@@ -7562,7 +7568,7 @@
       </c>
       <c r="V29" s="24" t="inlineStr">
         <is>
-          <t>loss</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W29" s="26" t="n"/>
@@ -7574,7 +7580,7 @@
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
       <c r="AC29" s="30" t="n">
-        <v>-1.5</v>
+        <v>1.38</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
         <is>
@@ -7583,7 +7589,7 @@
       </c>
       <c r="AE29" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFDE70CKDN on aec-wta-mansaw-panudv-2026-08-30 (short)</t>
+          <t>Auto-Buyer order C6VFNH9JYKDJ on aec-atp-valvac-alekov-2026-08-30 (long)</t>
         </is>
       </c>
       <c r="AF29" s="31" t="n"/>
@@ -7693,7 +7699,7 @@
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>8b833b3bf6574b26</t>
+          <t>525d5353a78b4b49</t>
         </is>
       </c>
       <c r="B30" s="24" t="inlineStr">
@@ -7708,7 +7714,7 @@
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>aec-wta-tamzid-martim-2026-08-30</t>
+          <t>aec-atp-matarn-jamduc-2026-08-30</t>
         </is>
       </c>
       <c r="E30" s="24" t="inlineStr">
@@ -7718,12 +7724,12 @@
       </c>
       <c r="F30" s="24" t="inlineStr">
         <is>
-          <t>Maria Timofeeva</t>
+          <t>James Duckworth</t>
         </is>
       </c>
       <c r="G30" s="24" t="inlineStr">
         <is>
-          <t>Tamara Zidansek</t>
+          <t>Matteo Arnaldi</t>
         </is>
       </c>
       <c r="H30" s="24" t="inlineStr">
@@ -7733,7 +7739,7 @@
       </c>
       <c r="I30" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J30" s="25" t="n"/>
@@ -7743,20 +7749,20 @@
         </is>
       </c>
       <c r="L30" s="26" t="n">
-        <v>194</v>
+        <v>156</v>
       </c>
       <c r="M30" s="27" t="n">
-        <v>2.94</v>
+        <v>2.56</v>
       </c>
       <c r="N30" s="28" t="n">
-        <v>0.3401</v>
+        <v>0.3906</v>
       </c>
       <c r="O30" s="28" t="n">
-        <v>0.5261</v>
+        <v>0.5743</v>
       </c>
       <c r="P30" s="28" t="n"/>
       <c r="Q30" s="28" t="n">
-        <v>0.1861</v>
+        <v>0.1843</v>
       </c>
       <c r="R30" s="26" t="n"/>
       <c r="S30" s="29" t="n">
@@ -7789,7 +7795,7 @@
       <c r="AD30" s="24" t="n"/>
       <c r="AE30" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFNH8ZYKDJ on aec-wta-tamzid-martim-2026-08-30 (long)</t>
+          <t>Auto-Buyer order C6VFCN0FYKDG on aec-atp-matarn-jamduc-2026-08-30 (short)</t>
         </is>
       </c>
       <c r="AF30" s="31" t="n"/>
@@ -7899,7 +7905,7 @@
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>55dfd65193ae4c3d</t>
+          <t>62563810a67a4509</t>
         </is>
       </c>
       <c r="B31" s="24" t="inlineStr">
@@ -7909,12 +7915,12 @@
       </c>
       <c r="C31" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T15:00Z</t>
+          <t>2026-08-31T17:00Z</t>
         </is>
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>aec-atp-valvac-alekov-2026-08-30</t>
+          <t>aec-atp-romsaf-caralc-2026-08-30</t>
         </is>
       </c>
       <c r="E31" s="24" t="inlineStr">
@@ -7924,12 +7930,12 @@
       </c>
       <c r="F31" s="24" t="inlineStr">
         <is>
-          <t>Aleksandar Kovacevic</t>
+          <t>Carlos Alcaraz</t>
         </is>
       </c>
       <c r="G31" s="24" t="inlineStr">
         <is>
-          <t>Valentin Vacherot</t>
+          <t>Roman Safiullin</t>
         </is>
       </c>
       <c r="H31" s="24" t="inlineStr">
@@ -7939,7 +7945,7 @@
       </c>
       <c r="I31" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J31" s="25" t="n"/>
@@ -7949,20 +7955,20 @@
         </is>
       </c>
       <c r="L31" s="26" t="n">
-        <v>-108</v>
+        <v>-488</v>
       </c>
       <c r="M31" s="27" t="n">
-        <v>1.9259</v>
+        <v>1.2049</v>
       </c>
       <c r="N31" s="28" t="n">
-        <v>0.5192</v>
+        <v>0.8299</v>
       </c>
       <c r="O31" s="28" t="n">
-        <v>0.6385</v>
+        <v>0.9435</v>
       </c>
       <c r="P31" s="28" t="n"/>
       <c r="Q31" s="28" t="n">
-        <v>0.1185</v>
+        <v>0.1135</v>
       </c>
       <c r="R31" s="26" t="n"/>
       <c r="S31" s="29" t="n">
@@ -7975,33 +7981,27 @@
       </c>
       <c r="U31" s="24" t="inlineStr">
         <is>
-          <t>settled</t>
+          <t>open</t>
         </is>
       </c>
       <c r="V31" s="24" t="inlineStr">
         <is>
-          <t>win</t>
+          <t>open</t>
         </is>
       </c>
       <c r="W31" s="26" t="n"/>
-      <c r="X31" s="26" t="n">
-        <v>1</v>
-      </c>
+      <c r="X31" s="26" t="n"/>
       <c r="Y31" s="25" t="n"/>
       <c r="Z31" s="26" t="n"/>
       <c r="AA31" s="28" t="n"/>
       <c r="AB31" s="28" t="n"/>
       <c r="AC31" s="30" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="AD31" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-31T18:41:38.707356Z</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AD31" s="24" t="n"/>
       <c r="AE31" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFNH9JYKDJ on aec-atp-valvac-alekov-2026-08-30 (long)</t>
+          <t>Auto-Buyer order C6VGABM5CKDK on aec-atp-romsaf-caralc-2026-08-30 (short)</t>
         </is>
       </c>
       <c r="AF31" s="31" t="n"/>
@@ -8111,7 +8111,7 @@
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>525d5353a78b4b49</t>
+          <t>a405afb6c6f7469b</t>
         </is>
       </c>
       <c r="B32" s="24" t="inlineStr">
@@ -8121,12 +8121,12 @@
       </c>
       <c r="C32" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T17:00Z</t>
+          <t>2026-08-31T18:00Z</t>
         </is>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>aec-atp-matarn-jamduc-2026-08-30</t>
+          <t>aec-atp-dalsvr-valroy-2026-08-30</t>
         </is>
       </c>
       <c r="E32" s="24" t="inlineStr">
@@ -8136,12 +8136,12 @@
       </c>
       <c r="F32" s="24" t="inlineStr">
         <is>
-          <t>James Duckworth</t>
+          <t>Valentin Royer</t>
         </is>
       </c>
       <c r="G32" s="24" t="inlineStr">
         <is>
-          <t>Matteo Arnaldi</t>
+          <t>Dalibor Svrcina</t>
         </is>
       </c>
       <c r="H32" s="24" t="inlineStr">
@@ -8151,7 +8151,7 @@
       </c>
       <c r="I32" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J32" s="25" t="n"/>
@@ -8161,24 +8161,24 @@
         </is>
       </c>
       <c r="L32" s="26" t="n">
-        <v>156</v>
+        <v>104</v>
       </c>
       <c r="M32" s="27" t="n">
-        <v>2.56</v>
+        <v>2.04</v>
       </c>
       <c r="N32" s="28" t="n">
-        <v>0.3906</v>
+        <v>0.4902</v>
       </c>
       <c r="O32" s="28" t="n">
-        <v>0.5743</v>
+        <v>0.5763</v>
       </c>
       <c r="P32" s="28" t="n"/>
       <c r="Q32" s="28" t="n">
-        <v>0.1843</v>
+        <v>0.0863</v>
       </c>
       <c r="R32" s="26" t="n"/>
       <c r="S32" s="29" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="T32" s="24" t="inlineStr">
         <is>
@@ -8207,7 +8207,7 @@
       <c r="AD32" s="24" t="n"/>
       <c r="AE32" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFCN0FYKDG on aec-atp-matarn-jamduc-2026-08-30 (short)</t>
+          <t>Auto-Buyer order C6VEZ2T7JKDC on aec-atp-dalsvr-valroy-2026-08-30 (long)</t>
         </is>
       </c>
       <c r="AF32" s="31" t="n"/>
@@ -8317,7 +8317,7 @@
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>62563810a67a4509</t>
+          <t>34d64f0e02e04343</t>
         </is>
       </c>
       <c r="B33" s="24" t="inlineStr">
@@ -8327,12 +8327,12 @@
       </c>
       <c r="C33" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T17:00Z</t>
+          <t>2026-08-31T18:30Z</t>
         </is>
       </c>
       <c r="D33" s="24" t="inlineStr">
         <is>
-          <t>aec-atp-romsaf-caralc-2026-08-30</t>
+          <t>aec-atp-jurrod-gioper-2026-08-30</t>
         </is>
       </c>
       <c r="E33" s="24" t="inlineStr">
@@ -8342,12 +8342,12 @@
       </c>
       <c r="F33" s="24" t="inlineStr">
         <is>
-          <t>Carlos Alcaraz</t>
+          <t>Giovanni Mpetshi Perricard</t>
         </is>
       </c>
       <c r="G33" s="24" t="inlineStr">
         <is>
-          <t>Roman Safiullin</t>
+          <t>Jurij Rodionov</t>
         </is>
       </c>
       <c r="H33" s="24" t="inlineStr">
@@ -8357,7 +8357,7 @@
       </c>
       <c r="I33" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J33" s="25" t="n"/>
@@ -8367,24 +8367,24 @@
         </is>
       </c>
       <c r="L33" s="26" t="n">
-        <v>-488</v>
+        <v>104</v>
       </c>
       <c r="M33" s="27" t="n">
-        <v>1.2049</v>
+        <v>2.04</v>
       </c>
       <c r="N33" s="28" t="n">
-        <v>0.8299</v>
+        <v>0.4902</v>
       </c>
       <c r="O33" s="28" t="n">
-        <v>0.9435</v>
+        <v>0.5453</v>
       </c>
       <c r="P33" s="28" t="n"/>
       <c r="Q33" s="28" t="n">
-        <v>0.1135</v>
+        <v>0.0553</v>
       </c>
       <c r="R33" s="26" t="n"/>
       <c r="S33" s="29" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="T33" s="24" t="inlineStr">
         <is>
@@ -8413,7 +8413,7 @@
       <c r="AD33" s="24" t="n"/>
       <c r="AE33" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VGABM5CKDK on aec-atp-romsaf-caralc-2026-08-30 (short)</t>
+          <t>Auto-Buyer order C6VF7S7KGKDM on aec-atp-jurrod-gioper-2026-08-30 (long)</t>
         </is>
       </c>
       <c r="AF33" s="31" t="n"/>
@@ -8523,7 +8523,7 @@
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>a405afb6c6f7469b</t>
+          <t>f138da48996b4c4e</t>
         </is>
       </c>
       <c r="B34" s="24" t="inlineStr">
@@ -8533,12 +8533,12 @@
       </c>
       <c r="C34" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T18:00Z</t>
+          <t>2026-08-31T20:30Z</t>
         </is>
       </c>
       <c r="D34" s="24" t="inlineStr">
         <is>
-          <t>aec-atp-dalsvr-valroy-2026-08-30</t>
+          <t>aec-atp-yanhan-aletab-2026-08-30</t>
         </is>
       </c>
       <c r="E34" s="24" t="inlineStr">
@@ -8548,12 +8548,12 @@
       </c>
       <c r="F34" s="24" t="inlineStr">
         <is>
-          <t>Valentin Royer</t>
+          <t>Alejandro Tabilo</t>
         </is>
       </c>
       <c r="G34" s="24" t="inlineStr">
         <is>
-          <t>Dalibor Svrcina</t>
+          <t>Yannick Hanfmann</t>
         </is>
       </c>
       <c r="H34" s="24" t="inlineStr">
@@ -8573,24 +8573,24 @@
         </is>
       </c>
       <c r="L34" s="26" t="n">
-        <v>104</v>
+        <v>133</v>
       </c>
       <c r="M34" s="27" t="n">
-        <v>2.04</v>
+        <v>2.33</v>
       </c>
       <c r="N34" s="28" t="n">
-        <v>0.4902</v>
+        <v>0.4292</v>
       </c>
       <c r="O34" s="28" t="n">
-        <v>0.5763</v>
+        <v>0.5565</v>
       </c>
       <c r="P34" s="28" t="n"/>
       <c r="Q34" s="28" t="n">
-        <v>0.0863</v>
+        <v>0.1265</v>
       </c>
       <c r="R34" s="26" t="n"/>
       <c r="S34" s="29" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="T34" s="24" t="inlineStr">
         <is>
@@ -8619,7 +8619,7 @@
       <c r="AD34" s="24" t="n"/>
       <c r="AE34" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VEZ2T7JKDC on aec-atp-dalsvr-valroy-2026-08-30 (long)</t>
+          <t>Auto-Buyer order C6VEZ2V6CKDC on aec-atp-yanhan-aletab-2026-08-30 (long)</t>
         </is>
       </c>
       <c r="AF34" s="31" t="n"/>
@@ -8729,7 +8729,7 @@
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>34d64f0e02e04343</t>
+          <t>87994ded7cbc49d8</t>
         </is>
       </c>
       <c r="B35" s="24" t="inlineStr">
@@ -8739,27 +8739,27 @@
       </c>
       <c r="C35" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T18:30Z</t>
+          <t>2026-08-31T08:00:00Z</t>
         </is>
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>aec-atp-jurrod-gioper-2026-08-30</t>
+          <t>aec-cs2-ssins-havu-2026-08-31</t>
         </is>
       </c>
       <c r="E35" s="24" t="inlineStr">
         <is>
-          <t>TENNIS</t>
+          <t>CS2</t>
         </is>
       </c>
       <c r="F35" s="24" t="inlineStr">
         <is>
-          <t>Giovanni Mpetshi Perricard</t>
+          <t>HAVU</t>
         </is>
       </c>
       <c r="G35" s="24" t="inlineStr">
         <is>
-          <t>Jurij Rodionov</t>
+          <t>Saint Sinners</t>
         </is>
       </c>
       <c r="H35" s="24" t="inlineStr">
@@ -8779,20 +8779,20 @@
         </is>
       </c>
       <c r="L35" s="26" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="M35" s="27" t="n">
-        <v>2.04</v>
+        <v>2.13</v>
       </c>
       <c r="N35" s="28" t="n">
-        <v>0.4902</v>
+        <v>0.4695</v>
       </c>
       <c r="O35" s="28" t="n">
-        <v>0.5453</v>
+        <v>0.5151</v>
       </c>
       <c r="P35" s="28" t="n"/>
       <c r="Q35" s="28" t="n">
-        <v>0.0553</v>
+        <v>0.0451</v>
       </c>
       <c r="R35" s="26" t="n"/>
       <c r="S35" s="29" t="n">
@@ -8800,17 +8800,17 @@
       </c>
       <c r="T35" s="24" t="inlineStr">
         <is>
-          <t>tennis-surface-elo-v1</t>
+          <t>cs2-tiered-elo-v6</t>
         </is>
       </c>
       <c r="U35" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V35" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W35" s="26" t="n"/>
@@ -8820,12 +8820,16 @@
       <c r="AA35" s="28" t="n"/>
       <c r="AB35" s="28" t="n"/>
       <c r="AC35" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD35" s="24" t="n"/>
+        <v>1.13</v>
+      </c>
+      <c r="AD35" s="24" t="inlineStr">
+        <is>
+          <t>2026-08-31T16:02:25.134027Z</t>
+        </is>
+      </c>
       <c r="AE35" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VF7S7KGKDM on aec-atp-jurrod-gioper-2026-08-30 (long)</t>
+          <t>Auto-Buyer order C6VFCN1GAKDG on aec-cs2-ssins-havu-2026-08-31 (long)</t>
         </is>
       </c>
       <c r="AF35" s="31" t="n"/>
@@ -8935,7 +8939,7 @@
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>f138da48996b4c4e</t>
+          <t>76d3b05a54a14e62</t>
         </is>
       </c>
       <c r="B36" s="24" t="inlineStr">
@@ -8945,27 +8949,27 @@
       </c>
       <c r="C36" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T20:30Z</t>
+          <t>2026-08-31T10:30:00Z</t>
         </is>
       </c>
       <c r="D36" s="24" t="inlineStr">
         <is>
-          <t>aec-atp-yanhan-aletab-2026-08-30</t>
+          <t>aec-cs2-ff-mel-2026-08-31</t>
         </is>
       </c>
       <c r="E36" s="24" t="inlineStr">
         <is>
-          <t>TENNIS</t>
+          <t>CS2</t>
         </is>
       </c>
       <c r="F36" s="24" t="inlineStr">
         <is>
-          <t>Alejandro Tabilo</t>
+          <t>mellren</t>
         </is>
       </c>
       <c r="G36" s="24" t="inlineStr">
         <is>
-          <t>Yannick Hanfmann</t>
+          <t>Fire Flux Esports</t>
         </is>
       </c>
       <c r="H36" s="24" t="inlineStr">
@@ -8975,7 +8979,7 @@
       </c>
       <c r="I36" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J36" s="25" t="n"/>
@@ -8985,28 +8989,28 @@
         </is>
       </c>
       <c r="L36" s="26" t="n">
-        <v>133</v>
+        <v>-113</v>
       </c>
       <c r="M36" s="27" t="n">
-        <v>2.33</v>
+        <v>1.885</v>
       </c>
       <c r="N36" s="28" t="n">
-        <v>0.4292</v>
+        <v>0.5305</v>
       </c>
       <c r="O36" s="28" t="n">
-        <v>0.5565</v>
+        <v>0.5667</v>
       </c>
       <c r="P36" s="28" t="n"/>
       <c r="Q36" s="28" t="n">
-        <v>0.1265</v>
+        <v>0.0367</v>
       </c>
       <c r="R36" s="26" t="n"/>
       <c r="S36" s="29" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="T36" s="24" t="inlineStr">
         <is>
-          <t>tennis-surface-elo-v1</t>
+          <t>cs2-tiered-elo-v6</t>
         </is>
       </c>
       <c r="U36" s="24" t="inlineStr">
@@ -9031,7 +9035,7 @@
       <c r="AD36" s="24" t="n"/>
       <c r="AE36" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VEZ2V6CKDC on aec-atp-yanhan-aletab-2026-08-30 (long)</t>
+          <t>Auto-Buyer order C6VGABNFWKDK on aec-cs2-ff-mel-2026-08-31 (short)</t>
         </is>
       </c>
       <c r="AF36" s="31" t="n"/>
@@ -9141,7 +9145,7 @@
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>87994ded7cbc49d8</t>
+          <t>6d6be9d1964a4439</t>
         </is>
       </c>
       <c r="B37" s="24" t="inlineStr">
@@ -9151,12 +9155,12 @@
       </c>
       <c r="C37" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T08:00:00Z</t>
+          <t>2026-08-31T11:30:00Z</t>
         </is>
       </c>
       <c r="D37" s="24" t="inlineStr">
         <is>
-          <t>aec-cs2-ssins-havu-2026-08-31</t>
+          <t>aec-cs2-g2-aur-2026-08-31</t>
         </is>
       </c>
       <c r="E37" s="24" t="inlineStr">
@@ -9166,12 +9170,12 @@
       </c>
       <c r="F37" s="24" t="inlineStr">
         <is>
-          <t>HAVU</t>
+          <t>Aurora Gaming</t>
         </is>
       </c>
       <c r="G37" s="24" t="inlineStr">
         <is>
-          <t>Saint Sinners</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="H37" s="24" t="inlineStr">
@@ -9191,20 +9195,20 @@
         </is>
       </c>
       <c r="L37" s="26" t="n">
-        <v>113</v>
+        <v>-122</v>
       </c>
       <c r="M37" s="27" t="n">
-        <v>2.13</v>
+        <v>1.8197</v>
       </c>
       <c r="N37" s="28" t="n">
-        <v>0.4695</v>
+        <v>0.5495</v>
       </c>
       <c r="O37" s="28" t="n">
-        <v>0.5151</v>
+        <v>0.6077</v>
       </c>
       <c r="P37" s="28" t="n"/>
       <c r="Q37" s="28" t="n">
-        <v>0.0451</v>
+        <v>0.0577</v>
       </c>
       <c r="R37" s="26" t="n"/>
       <c r="S37" s="29" t="n">
@@ -9232,7 +9236,7 @@
       <c r="AA37" s="28" t="n"/>
       <c r="AB37" s="28" t="n"/>
       <c r="AC37" s="30" t="n">
-        <v>1.13</v>
+        <v>0.82</v>
       </c>
       <c r="AD37" s="24" t="inlineStr">
         <is>
@@ -9241,7 +9245,7 @@
       </c>
       <c r="AE37" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFCN1GAKDG on aec-cs2-ssins-havu-2026-08-31 (long)</t>
+          <t>Auto-Buyer order C6VGABNP6KDK on aec-cs2-g2-aur-2026-08-31 (long)</t>
         </is>
       </c>
       <c r="AF37" s="31" t="n"/>
@@ -9351,7 +9355,7 @@
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>76d3b05a54a14e62</t>
+          <t>69301f19746a4d8d</t>
         </is>
       </c>
       <c r="B38" s="24" t="inlineStr">
@@ -9361,12 +9365,12 @@
       </c>
       <c r="C38" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T10:30:00Z</t>
+          <t>2026-08-31T12:00:00Z</t>
         </is>
       </c>
       <c r="D38" s="24" t="inlineStr">
         <is>
-          <t>aec-cs2-ff-mel-2026-08-31</t>
+          <t>aec-cs2-nem-ntr-2026-08-31</t>
         </is>
       </c>
       <c r="E38" s="24" t="inlineStr">
@@ -9376,12 +9380,12 @@
       </c>
       <c r="F38" s="24" t="inlineStr">
         <is>
-          <t>mellren</t>
+          <t>Nuclear TigeRES</t>
         </is>
       </c>
       <c r="G38" s="24" t="inlineStr">
         <is>
-          <t>Fire Flux Esports</t>
+          <t>Team Nemesis</t>
         </is>
       </c>
       <c r="H38" s="24" t="inlineStr">
@@ -9401,24 +9405,24 @@
         </is>
       </c>
       <c r="L38" s="26" t="n">
-        <v>-113</v>
+        <v>-100</v>
       </c>
       <c r="M38" s="27" t="n">
-        <v>1.885</v>
+        <v>2</v>
       </c>
       <c r="N38" s="28" t="n">
-        <v>0.5305</v>
+        <v>0.5</v>
       </c>
       <c r="O38" s="28" t="n">
-        <v>0.5667</v>
+        <v>0.6264999999999999</v>
       </c>
       <c r="P38" s="28" t="n"/>
       <c r="Q38" s="28" t="n">
-        <v>0.0367</v>
+        <v>0.1265</v>
       </c>
       <c r="R38" s="26" t="n"/>
       <c r="S38" s="29" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="T38" s="24" t="inlineStr">
         <is>
@@ -9447,7 +9451,7 @@
       <c r="AD38" s="24" t="n"/>
       <c r="AE38" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VGABNFWKDK on aec-cs2-ff-mel-2026-08-31 (short)</t>
+          <t>Auto-Buyer order C6VFCN23GKDG on aec-cs2-nem-ntr-2026-08-31 (short)</t>
         </is>
       </c>
       <c r="AF38" s="31" t="n"/>
@@ -9557,7 +9561,7 @@
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>6d6be9d1964a4439</t>
+          <t>08a9248313f04395</t>
         </is>
       </c>
       <c r="B39" s="24" t="inlineStr">
@@ -9567,12 +9571,12 @@
       </c>
       <c r="C39" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T11:30:00Z</t>
+          <t>2026-08-31T12:30:00Z</t>
         </is>
       </c>
       <c r="D39" s="24" t="inlineStr">
         <is>
-          <t>aec-cs2-g2-aur-2026-08-31</t>
+          <t>aec-cs2-cw-5s-2026-08-31</t>
         </is>
       </c>
       <c r="E39" s="24" t="inlineStr">
@@ -9582,12 +9586,12 @@
       </c>
       <c r="F39" s="24" t="inlineStr">
         <is>
-          <t>Aurora Gaming</t>
+          <t>5star</t>
         </is>
       </c>
       <c r="G39" s="24" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>Chinggis Warriors</t>
         </is>
       </c>
       <c r="H39" s="24" t="inlineStr">
@@ -9613,18 +9617,18 @@
         <v>1.8197</v>
       </c>
       <c r="N39" s="28" t="n">
-        <v>0.5495</v>
+        <v>0.5305</v>
       </c>
       <c r="O39" s="28" t="n">
-        <v>0.6077</v>
+        <v>0.6124000000000001</v>
       </c>
       <c r="P39" s="28" t="n"/>
       <c r="Q39" s="28" t="n">
-        <v>0.0577</v>
+        <v>0.0624</v>
       </c>
       <c r="R39" s="26" t="n"/>
       <c r="S39" s="29" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="T39" s="24" t="inlineStr">
         <is>
@@ -9638,7 +9642,7 @@
       </c>
       <c r="V39" s="24" t="inlineStr">
         <is>
-          <t>win</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="W39" s="26" t="n"/>
@@ -9648,7 +9652,7 @@
       <c r="AA39" s="28" t="n"/>
       <c r="AB39" s="28" t="n"/>
       <c r="AC39" s="30" t="n">
-        <v>0.82</v>
+        <v>-1.25</v>
       </c>
       <c r="AD39" s="24" t="inlineStr">
         <is>
@@ -9657,7 +9661,7 @@
       </c>
       <c r="AE39" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VGABNP6KDK on aec-cs2-g2-aur-2026-08-31 (long)</t>
+          <t>Auto-Buyer order C6VFNHBQEKDJ on aec-cs2-cw-5s-2026-08-31 (long)</t>
         </is>
       </c>
       <c r="AF39" s="31" t="n"/>
@@ -9767,7 +9771,7 @@
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>69301f19746a4d8d</t>
+          <t>10fe43507a894dff</t>
         </is>
       </c>
       <c r="B40" s="24" t="inlineStr">
@@ -9777,12 +9781,12 @@
       </c>
       <c r="C40" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T12:00:00Z</t>
+          <t>2026-08-31T14:00:00Z</t>
         </is>
       </c>
       <c r="D40" s="24" t="inlineStr">
         <is>
-          <t>aec-cs2-nem-ntr-2026-08-31</t>
+          <t>aec-cs2-mouz-fal-2026-08-31</t>
         </is>
       </c>
       <c r="E40" s="24" t="inlineStr">
@@ -9792,12 +9796,12 @@
       </c>
       <c r="F40" s="24" t="inlineStr">
         <is>
-          <t>Nuclear TigeRES</t>
+          <t>Team Falcons</t>
         </is>
       </c>
       <c r="G40" s="24" t="inlineStr">
         <is>
-          <t>Team Nemesis</t>
+          <t>MOUZ</t>
         </is>
       </c>
       <c r="H40" s="24" t="inlineStr">
@@ -9817,24 +9821,24 @@
         </is>
       </c>
       <c r="L40" s="26" t="n">
-        <v>-100</v>
+        <v>-122</v>
       </c>
       <c r="M40" s="27" t="n">
-        <v>2</v>
+        <v>1.8197</v>
       </c>
       <c r="N40" s="28" t="n">
-        <v>0.5</v>
+        <v>0.5495</v>
       </c>
       <c r="O40" s="28" t="n">
-        <v>0.6264999999999999</v>
+        <v>0.5978</v>
       </c>
       <c r="P40" s="28" t="n"/>
       <c r="Q40" s="28" t="n">
-        <v>0.1265</v>
+        <v>0.0478</v>
       </c>
       <c r="R40" s="26" t="n"/>
       <c r="S40" s="29" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="T40" s="24" t="inlineStr">
         <is>
@@ -9863,7 +9867,7 @@
       <c r="AD40" s="24" t="n"/>
       <c r="AE40" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFCN23GKDG on aec-cs2-nem-ntr-2026-08-31 (short)</t>
+          <t>Auto-Buyer order C6VFCN32YKDG on aec-cs2-mouz-fal-2026-08-31 (short)</t>
         </is>
       </c>
       <c r="AF40" s="31" t="n"/>
@@ -9973,7 +9977,7 @@
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>08a9248313f04395</t>
+          <t>2888a62dd3ba4d78</t>
         </is>
       </c>
       <c r="B41" s="24" t="inlineStr">
@@ -9983,12 +9987,12 @@
       </c>
       <c r="C41" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T12:30:00Z</t>
+          <t>2026-08-31T16:30:00Z</t>
         </is>
       </c>
       <c r="D41" s="24" t="inlineStr">
         <is>
-          <t>aec-cs2-cw-5s-2026-08-31</t>
+          <t>aec-cs2-fut-vit-2026-08-31</t>
         </is>
       </c>
       <c r="E41" s="24" t="inlineStr">
@@ -9998,12 +10002,12 @@
       </c>
       <c r="F41" s="24" t="inlineStr">
         <is>
-          <t>5star</t>
+          <t>Vitality</t>
         </is>
       </c>
       <c r="G41" s="24" t="inlineStr">
         <is>
-          <t>Chinggis Warriors</t>
+          <t>FUT Esports</t>
         </is>
       </c>
       <c r="H41" s="24" t="inlineStr">
@@ -10013,7 +10017,7 @@
       </c>
       <c r="I41" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J41" s="25" t="n"/>
@@ -10023,24 +10027,24 @@
         </is>
       </c>
       <c r="L41" s="26" t="n">
-        <v>-122</v>
+        <v>-213</v>
       </c>
       <c r="M41" s="27" t="n">
-        <v>1.8197</v>
+        <v>1.4695</v>
       </c>
       <c r="N41" s="28" t="n">
-        <v>0.5305</v>
+        <v>0.6805</v>
       </c>
       <c r="O41" s="28" t="n">
-        <v>0.6124000000000001</v>
+        <v>0.9538</v>
       </c>
       <c r="P41" s="28" t="n"/>
       <c r="Q41" s="28" t="n">
-        <v>0.0624</v>
+        <v>0.2738</v>
       </c>
       <c r="R41" s="26" t="n"/>
       <c r="S41" s="29" t="n">
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="T41" s="24" t="inlineStr">
         <is>
@@ -10049,12 +10053,12 @@
       </c>
       <c r="U41" s="24" t="inlineStr">
         <is>
-          <t>settled</t>
+          <t>open</t>
         </is>
       </c>
       <c r="V41" s="24" t="inlineStr">
         <is>
-          <t>loss</t>
+          <t>open</t>
         </is>
       </c>
       <c r="W41" s="26" t="n"/>
@@ -10064,16 +10068,12 @@
       <c r="AA41" s="28" t="n"/>
       <c r="AB41" s="28" t="n"/>
       <c r="AC41" s="30" t="n">
-        <v>-1.25</v>
-      </c>
-      <c r="AD41" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-31T16:02:25.134027Z</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AD41" s="24" t="n"/>
       <c r="AE41" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFNHBQEKDJ on aec-cs2-cw-5s-2026-08-31 (long)</t>
+          <t>Auto-Buyer order C6VGABPXTKDK on aec-cs2-fut-vit-2026-08-31 (short)</t>
         </is>
       </c>
       <c r="AF41" s="31" t="n"/>
@@ -10183,7 +10183,7 @@
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>10fe43507a894dff</t>
+          <t>7a9087c46a114e9c</t>
         </is>
       </c>
       <c r="B42" s="24" t="inlineStr">
@@ -10193,12 +10193,12 @@
       </c>
       <c r="C42" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T14:00:00Z</t>
+          <t>2026-08-31T17:00:00Z</t>
         </is>
       </c>
       <c r="D42" s="24" t="inlineStr">
         <is>
-          <t>aec-cs2-mouz-fal-2026-08-31</t>
+          <t>aec-cs2-hon-sawy-2026-08-31</t>
         </is>
       </c>
       <c r="E42" s="24" t="inlineStr">
@@ -10208,12 +10208,12 @@
       </c>
       <c r="F42" s="24" t="inlineStr">
         <is>
-          <t>Team Falcons</t>
+          <t>SAW Youngsters</t>
         </is>
       </c>
       <c r="G42" s="24" t="inlineStr">
         <is>
-          <t>MOUZ</t>
+          <t>Honvéd</t>
         </is>
       </c>
       <c r="H42" s="24" t="inlineStr">
@@ -10223,7 +10223,7 @@
       </c>
       <c r="I42" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J42" s="25" t="n"/>
@@ -10233,24 +10233,24 @@
         </is>
       </c>
       <c r="L42" s="26" t="n">
-        <v>-122</v>
+        <v>-100</v>
       </c>
       <c r="M42" s="27" t="n">
-        <v>1.8197</v>
+        <v>2</v>
       </c>
       <c r="N42" s="28" t="n">
-        <v>0.5495</v>
+        <v>0.5</v>
       </c>
       <c r="O42" s="28" t="n">
-        <v>0.5978</v>
+        <v>0.5755</v>
       </c>
       <c r="P42" s="28" t="n"/>
       <c r="Q42" s="28" t="n">
-        <v>0.0478</v>
+        <v>0.0755</v>
       </c>
       <c r="R42" s="26" t="n"/>
       <c r="S42" s="29" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="T42" s="24" t="inlineStr">
         <is>
@@ -10279,7 +10279,7 @@
       <c r="AD42" s="24" t="n"/>
       <c r="AE42" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VFCN32YKDG on aec-cs2-mouz-fal-2026-08-31 (short)</t>
+          <t>Auto-Buyer order C6VGABQ8AKDK on aec-cs2-hon-sawy-2026-08-31 (long)</t>
         </is>
       </c>
       <c r="AF42" s="31" t="n"/>
@@ -10389,37 +10389,37 @@
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="24" t="inlineStr">
         <is>
-          <t>2888a62dd3ba4d78</t>
+          <t>48cccc66566349ce</t>
         </is>
       </c>
       <c r="B43" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T04:52:35.718859Z</t>
+          <t>2026-08-31T05:28:12.217545Z</t>
         </is>
       </c>
       <c r="C43" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T16:30:00Z</t>
+          <t>2026-08-31T18:05:00-0400</t>
         </is>
       </c>
       <c r="D43" s="24" t="inlineStr">
         <is>
-          <t>aec-cs2-fut-vit-2026-08-31</t>
+          <t>aec-mlb-sf-atl-2026-08-31</t>
         </is>
       </c>
       <c r="E43" s="24" t="inlineStr">
         <is>
-          <t>CS2</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F43" s="24" t="inlineStr">
         <is>
-          <t>Vitality</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="G43" s="24" t="inlineStr">
         <is>
-          <t>FUT Esports</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="H43" s="24" t="inlineStr">
@@ -10429,7 +10429,7 @@
       </c>
       <c r="I43" s="24" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="J43" s="25" t="n"/>
@@ -10439,28 +10439,28 @@
         </is>
       </c>
       <c r="L43" s="26" t="n">
-        <v>-213</v>
+        <v>-150</v>
       </c>
       <c r="M43" s="27" t="n">
-        <v>1.4695</v>
+        <v>1.6667</v>
       </c>
       <c r="N43" s="28" t="n">
-        <v>0.6805</v>
+        <v>0.6</v>
       </c>
       <c r="O43" s="28" t="n">
-        <v>0.9538</v>
+        <v>0.6571</v>
       </c>
       <c r="P43" s="28" t="n"/>
       <c r="Q43" s="28" t="n">
-        <v>0.2738</v>
+        <v>0.0521</v>
       </c>
       <c r="R43" s="26" t="n"/>
       <c r="S43" s="29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T43" s="24" t="inlineStr">
         <is>
-          <t>cs2-tiered-elo-v6</t>
+          <t>mlb-elo-trend-lr-v8</t>
         </is>
       </c>
       <c r="U43" s="24" t="inlineStr">
@@ -10485,7 +10485,7 @@
       <c r="AD43" s="24" t="n"/>
       <c r="AE43" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VGABPXTKDK on aec-cs2-fut-vit-2026-08-31 (short)</t>
+          <t>Auto-Buyer order C6VZ1TQF4KDJ on aec-mlb-sf-atl-2026-08-31 (short)</t>
         </is>
       </c>
       <c r="AF43" s="31" t="n"/>
@@ -10595,37 +10595,37 @@
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t>7a9087c46a114e9c</t>
+          <t>d972531055904f04</t>
         </is>
       </c>
       <c r="B44" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T04:52:35.718859Z</t>
+          <t>2026-08-31T05:28:12.217545Z</t>
         </is>
       </c>
       <c r="C44" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T17:00:00Z</t>
+          <t>2026-08-31T19:40:00-0400</t>
         </is>
       </c>
       <c r="D44" s="24" t="inlineStr">
         <is>
-          <t>aec-cs2-hon-sawy-2026-08-31</t>
+          <t>aec-mlb-det-min-2026-08-31</t>
         </is>
       </c>
       <c r="E44" s="24" t="inlineStr">
         <is>
-          <t>CS2</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F44" s="24" t="inlineStr">
         <is>
-          <t>SAW Youngsters</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="G44" s="24" t="inlineStr">
         <is>
-          <t>Honvéd</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="H44" s="24" t="inlineStr">
@@ -10635,7 +10635,7 @@
       </c>
       <c r="I44" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J44" s="25" t="n"/>
@@ -10645,28 +10645,28 @@
         </is>
       </c>
       <c r="L44" s="26" t="n">
-        <v>-100</v>
+        <v>117</v>
       </c>
       <c r="M44" s="27" t="n">
-        <v>2</v>
+        <v>2.17</v>
       </c>
       <c r="N44" s="28" t="n">
-        <v>0.5</v>
+        <v>0.4545</v>
       </c>
       <c r="O44" s="28" t="n">
-        <v>0.5755</v>
+        <v>0.5224</v>
       </c>
       <c r="P44" s="28" t="n"/>
       <c r="Q44" s="28" t="n">
-        <v>0.0755</v>
+        <v>0.0674</v>
       </c>
       <c r="R44" s="26" t="n"/>
       <c r="S44" s="29" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="T44" s="24" t="inlineStr">
         <is>
-          <t>cs2-tiered-elo-v6</t>
+          <t>mlb-elo-trend-lr-v8</t>
         </is>
       </c>
       <c r="U44" s="24" t="inlineStr">
@@ -10691,7 +10691,7 @@
       <c r="AD44" s="24" t="n"/>
       <c r="AE44" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VGABQ8AKDK on aec-cs2-hon-sawy-2026-08-31 (long)</t>
+          <t>Auto-Buyer order C6W0RWB0MKDH on aec-mlb-det-min-2026-08-31 (long)</t>
         </is>
       </c>
       <c r="AF44" s="31" t="n"/>
@@ -10801,22 +10801,22 @@
     <row r="45" ht="36" customHeight="1">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>48cccc66566349ce</t>
+          <t>26a05e27c35344e1</t>
         </is>
       </c>
       <c r="B45" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T05:28:12.217545Z</t>
+          <t>2026-08-31T16:12:42.599391Z</t>
         </is>
       </c>
       <c r="C45" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T18:05:00-0400</t>
+          <t>2026-08-31T20:40:00-0400</t>
         </is>
       </c>
       <c r="D45" s="24" t="inlineStr">
         <is>
-          <t>aec-mlb-sf-atl-2026-08-31</t>
+          <t>aec-mlb-bal-col-2026-08-31</t>
         </is>
       </c>
       <c r="E45" s="24" t="inlineStr">
@@ -10826,12 +10826,12 @@
       </c>
       <c r="F45" s="24" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="G45" s="24" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="H45" s="24" t="inlineStr">
@@ -10841,7 +10841,7 @@
       </c>
       <c r="I45" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J45" s="25" t="n"/>
@@ -10851,20 +10851,20 @@
         </is>
       </c>
       <c r="L45" s="26" t="n">
-        <v>-150</v>
+        <v>-127</v>
       </c>
       <c r="M45" s="27" t="n">
-        <v>1.6667</v>
+        <v>1.7874</v>
       </c>
       <c r="N45" s="28" t="n">
-        <v>0.6</v>
+        <v>0.5595</v>
       </c>
       <c r="O45" s="28" t="n">
-        <v>0.6571</v>
+        <v>0.5982</v>
       </c>
       <c r="P45" s="28" t="n"/>
       <c r="Q45" s="28" t="n">
-        <v>0.0521</v>
+        <v>0.0382</v>
       </c>
       <c r="R45" s="26" t="n"/>
       <c r="S45" s="29" t="n">
@@ -10897,7 +10897,7 @@
       <c r="AD45" s="24" t="n"/>
       <c r="AE45" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6VZ1TQF4KDJ on aec-mlb-sf-atl-2026-08-31 (short)</t>
+          <t>Auto-Buyer order C75CWYPPPKDC on aec-mlb-bal-col-2026-08-31 (long)</t>
         </is>
       </c>
       <c r="AF45" s="31" t="n"/>
@@ -11007,22 +11007,22 @@
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="24" t="inlineStr">
         <is>
-          <t>d972531055904f04</t>
+          <t>7ee8b96d25fc46af</t>
         </is>
       </c>
       <c r="B46" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T05:28:12.217545Z</t>
+          <t>2026-08-31T19:34:36.451981Z</t>
         </is>
       </c>
       <c r="C46" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T19:40:00-0400</t>
+          <t>2026-08-31T22:05Z</t>
         </is>
       </c>
       <c r="D46" s="24" t="inlineStr">
         <is>
-          <t>aec-mlb-det-min-2026-08-31</t>
+          <t>401878657</t>
         </is>
       </c>
       <c r="E46" s="24" t="inlineStr">
@@ -11032,53 +11032,59 @@
       </c>
       <c r="F46" s="24" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="G46" s="24" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="H46" s="24" t="inlineStr">
         <is>
-          <t>moneyline</t>
+          <t>total</t>
         </is>
       </c>
       <c r="I46" s="24" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J46" s="25" t="n"/>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J46" s="25" t="n">
+        <v>8.5</v>
+      </c>
       <c r="K46" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L46" s="26" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="M46" s="27" t="n">
-        <v>2.17</v>
+        <v>2.22</v>
       </c>
       <c r="N46" s="28" t="n">
-        <v>0.4545</v>
+        <v>0.4505</v>
       </c>
       <c r="O46" s="28" t="n">
-        <v>0.5224</v>
-      </c>
-      <c r="P46" s="28" t="n"/>
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="P46" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="Q46" s="28" t="n">
-        <v>0.0674</v>
-      </c>
-      <c r="R46" s="26" t="n"/>
+        <v>0.1135</v>
+      </c>
+      <c r="R46" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="S46" s="29" t="n">
         <v>1</v>
       </c>
       <c r="T46" s="24" t="inlineStr">
         <is>
-          <t>mlb-elo-trend-lr-v8</t>
+          <t>mlb-structural-v10-frozen</t>
         </is>
       </c>
       <c r="U46" s="24" t="inlineStr">
@@ -11086,27 +11092,29 @@
           <t>open</t>
         </is>
       </c>
-      <c r="V46" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="V46" s="24" t="n"/>
       <c r="W46" s="26" t="n"/>
       <c r="X46" s="26" t="n"/>
       <c r="Y46" s="25" t="n"/>
       <c r="Z46" s="26" t="n"/>
       <c r="AA46" s="28" t="n"/>
-      <c r="AB46" s="28" t="n"/>
+      <c r="AB46" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="AC46" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AD46" s="24" t="n"/>
       <c r="AE46" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C6W0RWB0MKDH on aec-mlb-det-min-2026-08-31 (long)</t>
-        </is>
-      </c>
-      <c r="AF46" s="31" t="n"/>
+          <t>Auto-Buyer order V10D71C79953 (1.0 sh @ $0.45) on tsc-mlb-sf-atl-2026-08-31-8pt5 (short)</t>
+        </is>
+      </c>
+      <c r="AF46" s="31" t="inlineStr">
+        <is>
+          <t>Auto-executed Polymarket US order</t>
+        </is>
+      </c>
       <c r="AG46" s="24" t="n"/>
       <c r="AH46" s="24" t="n"/>
       <c r="AI46" s="31" t="n"/>
@@ -11213,22 +11221,22 @@
     <row r="47" ht="36" customHeight="1">
       <c r="A47" s="24" t="inlineStr">
         <is>
-          <t>26a05e27c35344e1</t>
+          <t>37aaf37c09f84e3f</t>
         </is>
       </c>
       <c r="B47" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T16:12:42.599391Z</t>
+          <t>2026-08-31T19:34:36.590960Z</t>
         </is>
       </c>
       <c r="C47" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T20:40:00-0400</t>
+          <t>2026-08-31T23:40Z</t>
         </is>
       </c>
       <c r="D47" s="24" t="inlineStr">
         <is>
-          <t>aec-mlb-bal-col-2026-08-31</t>
+          <t>401816754</t>
         </is>
       </c>
       <c r="E47" s="24" t="inlineStr">
@@ -11238,53 +11246,59 @@
       </c>
       <c r="F47" s="24" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G47" s="24" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="H47" s="24" t="inlineStr">
         <is>
-          <t>moneyline</t>
+          <t>total</t>
         </is>
       </c>
       <c r="I47" s="24" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J47" s="25" t="n"/>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J47" s="25" t="n">
+        <v>9.5</v>
+      </c>
       <c r="K47" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L47" s="26" t="n">
-        <v>-127</v>
+        <v>-102</v>
       </c>
       <c r="M47" s="27" t="n">
-        <v>1.7874</v>
+        <v>1.9804</v>
       </c>
       <c r="N47" s="28" t="n">
-        <v>0.5595</v>
+        <v>0.505</v>
       </c>
       <c r="O47" s="28" t="n">
-        <v>0.5982</v>
-      </c>
-      <c r="P47" s="28" t="n"/>
+        <v>0.5755</v>
+      </c>
+      <c r="P47" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="Q47" s="28" t="n">
-        <v>0.0382</v>
-      </c>
-      <c r="R47" s="26" t="n"/>
+        <v>0.0706</v>
+      </c>
+      <c r="R47" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="S47" s="29" t="n">
         <v>1</v>
       </c>
       <c r="T47" s="24" t="inlineStr">
         <is>
-          <t>mlb-elo-trend-lr-v8</t>
+          <t>mlb-structural-v10-frozen</t>
         </is>
       </c>
       <c r="U47" s="24" t="inlineStr">
@@ -11292,27 +11306,29 @@
           <t>open</t>
         </is>
       </c>
-      <c r="V47" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="V47" s="24" t="n"/>
       <c r="W47" s="26" t="n"/>
       <c r="X47" s="26" t="n"/>
       <c r="Y47" s="25" t="n"/>
       <c r="Z47" s="26" t="n"/>
       <c r="AA47" s="28" t="n"/>
-      <c r="AB47" s="28" t="n"/>
+      <c r="AB47" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="AC47" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AD47" s="24" t="n"/>
       <c r="AE47" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C75CWYPPPKDC on aec-mlb-bal-col-2026-08-31 (long)</t>
-        </is>
-      </c>
-      <c r="AF47" s="31" t="n"/>
+          <t>Auto-Buyer order V101066144C4 (1.0 sh @ $0.50) on tsc-mlb-mil-chc-2026-08-31-9pt5 (short)</t>
+        </is>
+      </c>
+      <c r="AF47" s="31" t="inlineStr">
+        <is>
+          <t>Auto-executed Polymarket US order</t>
+        </is>
+      </c>
       <c r="AG47" s="24" t="n"/>
       <c r="AH47" s="24" t="n"/>
       <c r="AI47" s="31" t="n"/>
@@ -11419,7 +11435,7 @@
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="24" t="inlineStr">
         <is>
-          <t>7ee8b96d25fc46af</t>
+          <t>816e58389cba4c61</t>
         </is>
       </c>
       <c r="B48" s="24" t="inlineStr">
@@ -11429,37 +11445,37 @@
       </c>
       <c r="C48" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T22:05Z</t>
+          <t>2026-08-31T19:00Z</t>
         </is>
       </c>
       <c r="D48" s="24" t="inlineStr">
         <is>
-          <t>tsc-mlb-sf-atl-2026-08-31-8pt5</t>
+          <t>aec-wta-vikgol-diapar-2026-08-30</t>
         </is>
       </c>
       <c r="E48" s="24" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>TENNIS</t>
         </is>
       </c>
       <c r="F48" s="24" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Diane Parry</t>
         </is>
       </c>
       <c r="G48" s="24" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Viktorija Golubic</t>
         </is>
       </c>
       <c r="H48" s="24" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>moneyline</t>
         </is>
       </c>
       <c r="I48" s="24" t="inlineStr">
         <is>
-          <t>under</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J48" s="25" t="n"/>
@@ -11469,20 +11485,20 @@
         </is>
       </c>
       <c r="L48" s="26" t="n">
-        <v>122</v>
+        <v>-108</v>
       </c>
       <c r="M48" s="27" t="n">
-        <v>2.22</v>
+        <v>1.9259</v>
       </c>
       <c r="N48" s="28" t="n">
-        <v>0.4505</v>
+        <v>0.5192</v>
       </c>
       <c r="O48" s="28" t="n">
-        <v>0.5076000000000001</v>
+        <v>0.5579</v>
       </c>
       <c r="P48" s="28" t="n"/>
       <c r="Q48" s="28" t="n">
-        <v>0.0576</v>
+        <v>0.0379</v>
       </c>
       <c r="R48" s="26" t="n"/>
       <c r="S48" s="29" t="n">
@@ -11490,7 +11506,7 @@
       </c>
       <c r="T48" s="24" t="inlineStr">
         <is>
-          <t>measured-edge-totals-v3</t>
+          <t>tennis-surface-elo-v1</t>
         </is>
       </c>
       <c r="U48" s="24" t="inlineStr">
@@ -11515,7 +11531,7 @@
       <c r="AD48" s="24" t="n"/>
       <c r="AE48" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C75E2V3VPKDH on tsc-mlb-sf-atl-2026-08-31-8pt5 (short)</t>
+          <t>Auto-Buyer order C75DSQ4KAKDM on aec-wta-vikgol-diapar-2026-08-30 (short)</t>
         </is>
       </c>
       <c r="AF48" s="31" t="n"/>
@@ -11625,7 +11641,7 @@
     <row r="49" ht="36" customHeight="1">
       <c r="A49" s="24" t="inlineStr">
         <is>
-          <t>8e234c9a1aa54341</t>
+          <t>b214bda284bc4f41</t>
         </is>
       </c>
       <c r="B49" s="24" t="inlineStr">
@@ -11635,37 +11651,37 @@
       </c>
       <c r="C49" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T22:40Z</t>
+          <t>2026-08-31T19:00:00Z</t>
         </is>
       </c>
       <c r="D49" s="24" t="inlineStr">
         <is>
-          <t>tsc-mlb-nym-tb-2026-08-31-8pt5</t>
+          <t>aec-cs2-dam-zge-2026-08-31</t>
         </is>
       </c>
       <c r="E49" s="24" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CS2</t>
         </is>
       </c>
       <c r="F49" s="24" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Zetta Games</t>
         </is>
       </c>
       <c r="G49" s="24" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Damajuana</t>
         </is>
       </c>
       <c r="H49" s="24" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>moneyline</t>
         </is>
       </c>
       <c r="I49" s="24" t="inlineStr">
         <is>
-          <t>over</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J49" s="25" t="n"/>
@@ -11675,28 +11691,28 @@
         </is>
       </c>
       <c r="L49" s="26" t="n">
-        <v>113</v>
+        <v>212</v>
       </c>
       <c r="M49" s="27" t="n">
-        <v>2.13</v>
+        <v>3.12</v>
       </c>
       <c r="N49" s="28" t="n">
-        <v>0.4695</v>
+        <v>0.3205</v>
       </c>
       <c r="O49" s="28" t="n">
-        <v>0.5185</v>
+        <v>0.5642</v>
       </c>
       <c r="P49" s="28" t="n"/>
       <c r="Q49" s="28" t="n">
-        <v>0.0485</v>
+        <v>0.2442</v>
       </c>
       <c r="R49" s="26" t="n"/>
       <c r="S49" s="29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T49" s="24" t="inlineStr">
         <is>
-          <t>measured-edge-totals-v3</t>
+          <t>cs2-tiered-elo-v6</t>
         </is>
       </c>
       <c r="U49" s="24" t="inlineStr">
@@ -11721,7 +11737,7 @@
       <c r="AD49" s="24" t="n"/>
       <c r="AE49" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C75E2V4FEKDH on tsc-mlb-nym-tb-2026-08-31-8pt5 (long)</t>
+          <t>Auto-Buyer order C75ED9T52KDF on aec-cs2-dam-zge-2026-08-31 (short)</t>
         </is>
       </c>
       <c r="AF49" s="31" t="n"/>
@@ -11831,7 +11847,7 @@
     <row r="50" ht="36" customHeight="1">
       <c r="A50" s="24" t="inlineStr">
         <is>
-          <t>37aaf37c09f84e3f</t>
+          <t>fd008ef45af2480d</t>
         </is>
       </c>
       <c r="B50" s="24" t="inlineStr">
@@ -11841,37 +11857,37 @@
       </c>
       <c r="C50" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T23:40Z</t>
+          <t>2026-08-31T22:00:00Z</t>
         </is>
       </c>
       <c r="D50" s="24" t="inlineStr">
         <is>
-          <t>tsc-mlb-mil-chc-2026-08-31-9pt5</t>
+          <t>aec-cs2-mm-sdm-2026-08-31</t>
         </is>
       </c>
       <c r="E50" s="24" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CS2</t>
         </is>
       </c>
       <c r="F50" s="24" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Semente do Mal</t>
         </is>
       </c>
       <c r="G50" s="24" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Mansão Maromba</t>
         </is>
       </c>
       <c r="H50" s="24" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>moneyline</t>
         </is>
       </c>
       <c r="I50" s="24" t="inlineStr">
         <is>
-          <t>under</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J50" s="25" t="n"/>
@@ -11881,28 +11897,28 @@
         </is>
       </c>
       <c r="L50" s="26" t="n">
-        <v>-104</v>
+        <v>212</v>
       </c>
       <c r="M50" s="27" t="n">
-        <v>1.9615</v>
+        <v>3.12</v>
       </c>
       <c r="N50" s="28" t="n">
-        <v>0.505</v>
+        <v>0.3205</v>
       </c>
       <c r="O50" s="28" t="n">
-        <v>0.5448</v>
+        <v>0.5066000000000001</v>
       </c>
       <c r="P50" s="28" t="n"/>
       <c r="Q50" s="28" t="n">
-        <v>0.0398</v>
+        <v>0.1866</v>
       </c>
       <c r="R50" s="26" t="n"/>
       <c r="S50" s="29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T50" s="24" t="inlineStr">
         <is>
-          <t>measured-edge-totals-v3</t>
+          <t>cs2-tiered-elo-v6</t>
         </is>
       </c>
       <c r="U50" s="24" t="inlineStr">
@@ -11927,7 +11943,7 @@
       <c r="AD50" s="24" t="n"/>
       <c r="AE50" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C75E1JWMRKDG on tsc-mlb-mil-chc-2026-08-31-9pt5 (short)</t>
+          <t>Auto-Buyer order C75CWYWSTKDC on aec-cs2-mm-sdm-2026-08-31 (short)</t>
         </is>
       </c>
       <c r="AF50" s="31" t="n"/>
@@ -12037,22 +12053,22 @@
     <row r="51" ht="36" customHeight="1">
       <c r="A51" s="24" t="inlineStr">
         <is>
-          <t>8651501eb94f43b2</t>
+          <t>970da3eec9e24614</t>
         </is>
       </c>
       <c r="B51" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T16:12:42.599391Z</t>
+          <t>2026-08-31T19:34:36.729957Z</t>
         </is>
       </c>
       <c r="C51" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T01:38Z</t>
+          <t>2026-09-01T00:40Z</t>
         </is>
       </c>
       <c r="D51" s="24" t="inlineStr">
         <is>
-          <t>tsc-mlb-nyy-laa-2026-08-31-8pt5</t>
+          <t>401816755</t>
         </is>
       </c>
       <c r="E51" s="24" t="inlineStr">
@@ -12062,12 +12078,12 @@
       </c>
       <c r="F51" s="24" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="G51" s="24" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="H51" s="24" t="inlineStr">
@@ -12077,10 +12093,12 @@
       </c>
       <c r="I51" s="24" t="inlineStr">
         <is>
-          <t>over</t>
-        </is>
-      </c>
-      <c r="J51" s="25" t="n"/>
+          <t>under</t>
+        </is>
+      </c>
+      <c r="J51" s="25" t="n">
+        <v>10.5</v>
+      </c>
       <c r="K51" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -12096,19 +12114,23 @@
         <v>0.4695</v>
       </c>
       <c r="O51" s="28" t="n">
-        <v>0.513</v>
-      </c>
-      <c r="P51" s="28" t="n"/>
+        <v>0.5296</v>
+      </c>
+      <c r="P51" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="Q51" s="28" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="R51" s="26" t="n"/>
+        <v>0.0601</v>
+      </c>
+      <c r="R51" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="S51" s="29" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="T51" s="24" t="inlineStr">
         <is>
-          <t>measured-edge-totals-v3</t>
+          <t>mlb-structural-v10-frozen</t>
         </is>
       </c>
       <c r="U51" s="24" t="inlineStr">
@@ -12116,27 +12138,29 @@
           <t>open</t>
         </is>
       </c>
-      <c r="V51" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="V51" s="24" t="n"/>
       <c r="W51" s="26" t="n"/>
       <c r="X51" s="26" t="n"/>
       <c r="Y51" s="25" t="n"/>
       <c r="Z51" s="26" t="n"/>
       <c r="AA51" s="28" t="n"/>
-      <c r="AB51" s="28" t="n"/>
+      <c r="AB51" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="AC51" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AD51" s="24" t="n"/>
       <c r="AE51" s="31" t="inlineStr">
         <is>
-          <t>Auto-Buyer order C75D7932RKDD on tsc-mlb-nyy-laa-2026-08-31-8pt5 (long)</t>
-        </is>
-      </c>
-      <c r="AF51" s="31" t="n"/>
+          <t>Auto-Buyer order V105A22EB006 (1.0 sh @ $0.47) on tsc-mlb-bal-col-2026-08-31-10pt5 (short)</t>
+        </is>
+      </c>
+      <c r="AF51" s="31" t="inlineStr">
+        <is>
+          <t>Auto-executed Polymarket US order</t>
+        </is>
+      </c>
       <c r="AG51" s="24" t="n"/>
       <c r="AH51" s="24" t="n"/>
       <c r="AI51" s="31" t="n"/>
@@ -12240,624 +12264,6 @@
       <c r="DO51" s="24" t="n"/>
       <c r="DP51" s="24" t="n"/>
     </row>
-    <row r="52" ht="36" customHeight="1">
-      <c r="A52" s="24" t="inlineStr">
-        <is>
-          <t>816e58389cba4c61</t>
-        </is>
-      </c>
-      <c r="B52" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-31T16:12:42.599391Z</t>
-        </is>
-      </c>
-      <c r="C52" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-31T19:00Z</t>
-        </is>
-      </c>
-      <c r="D52" s="24" t="inlineStr">
-        <is>
-          <t>aec-wta-vikgol-diapar-2026-08-30</t>
-        </is>
-      </c>
-      <c r="E52" s="24" t="inlineStr">
-        <is>
-          <t>TENNIS</t>
-        </is>
-      </c>
-      <c r="F52" s="24" t="inlineStr">
-        <is>
-          <t>Diane Parry</t>
-        </is>
-      </c>
-      <c r="G52" s="24" t="inlineStr">
-        <is>
-          <t>Viktorija Golubic</t>
-        </is>
-      </c>
-      <c r="H52" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I52" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J52" s="25" t="n"/>
-      <c r="K52" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L52" s="26" t="n">
-        <v>-108</v>
-      </c>
-      <c r="M52" s="27" t="n">
-        <v>1.9259</v>
-      </c>
-      <c r="N52" s="28" t="n">
-        <v>0.5192</v>
-      </c>
-      <c r="O52" s="28" t="n">
-        <v>0.5579</v>
-      </c>
-      <c r="P52" s="28" t="n"/>
-      <c r="Q52" s="28" t="n">
-        <v>0.0379</v>
-      </c>
-      <c r="R52" s="26" t="n"/>
-      <c r="S52" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="T52" s="24" t="inlineStr">
-        <is>
-          <t>tennis-surface-elo-v1</t>
-        </is>
-      </c>
-      <c r="U52" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V52" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="W52" s="26" t="n"/>
-      <c r="X52" s="26" t="n"/>
-      <c r="Y52" s="25" t="n"/>
-      <c r="Z52" s="26" t="n"/>
-      <c r="AA52" s="28" t="n"/>
-      <c r="AB52" s="28" t="n"/>
-      <c r="AC52" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD52" s="24" t="n"/>
-      <c r="AE52" s="31" t="inlineStr">
-        <is>
-          <t>Auto-Buyer order C75DSQ4KAKDM on aec-wta-vikgol-diapar-2026-08-30 (short)</t>
-        </is>
-      </c>
-      <c r="AF52" s="31" t="n"/>
-      <c r="AG52" s="24" t="n"/>
-      <c r="AH52" s="24" t="n"/>
-      <c r="AI52" s="31" t="n"/>
-      <c r="AJ52" s="31" t="n"/>
-      <c r="AK52" s="24" t="n"/>
-      <c r="AL52" s="26" t="n">
-        <v>4</v>
-      </c>
-      <c r="AM52" s="24" t="inlineStr">
-        <is>
-          <t>decision</t>
-        </is>
-      </c>
-      <c r="AN52" s="24" t="inlineStr">
-        <is>
-          <t>take</t>
-        </is>
-      </c>
-      <c r="AO52" s="24" t="inlineStr">
-        <is>
-          <t>AUTO_BUYER_EXECUTION</t>
-        </is>
-      </c>
-      <c r="AP52" s="24" t="n"/>
-      <c r="AQ52" s="24" t="n"/>
-      <c r="AR52" s="24" t="n"/>
-      <c r="AS52" s="24" t="n"/>
-      <c r="AT52" s="24" t="n"/>
-      <c r="AU52" s="24" t="n"/>
-      <c r="AV52" s="24" t="n"/>
-      <c r="AW52" s="24" t="n"/>
-      <c r="AX52" s="24" t="n"/>
-      <c r="AY52" s="24" t="n"/>
-      <c r="AZ52" s="24" t="n"/>
-      <c r="BA52" s="24" t="n"/>
-      <c r="BB52" s="24" t="n"/>
-      <c r="BC52" s="24" t="n"/>
-      <c r="BD52" s="24" t="n"/>
-      <c r="BE52" s="24" t="n"/>
-      <c r="BF52" s="24" t="n"/>
-      <c r="BG52" s="24" t="n"/>
-      <c r="BH52" s="24" t="n"/>
-      <c r="BI52" s="24" t="n"/>
-      <c r="BJ52" s="25" t="n"/>
-      <c r="BK52" s="26" t="n"/>
-      <c r="BL52" s="27" t="n"/>
-      <c r="BM52" s="28" t="n"/>
-      <c r="BN52" s="28" t="n"/>
-      <c r="BO52" s="28" t="n"/>
-      <c r="BP52" s="25" t="n"/>
-      <c r="BQ52" s="27" t="n"/>
-      <c r="BR52" s="28" t="n"/>
-      <c r="BS52" s="28" t="n"/>
-      <c r="BT52" s="28" t="n"/>
-      <c r="BU52" s="25" t="n"/>
-      <c r="BV52" s="29" t="n"/>
-      <c r="BW52" s="24" t="n"/>
-      <c r="BX52" s="30" t="n"/>
-      <c r="BY52" s="27" t="n"/>
-      <c r="BZ52" s="24" t="n"/>
-      <c r="CA52" s="31" t="n"/>
-      <c r="CB52" s="24" t="n"/>
-      <c r="CC52" s="24" t="n"/>
-      <c r="CD52" s="24" t="n"/>
-      <c r="CE52" s="24" t="n"/>
-      <c r="CF52" s="24" t="n"/>
-      <c r="CG52" s="24" t="n"/>
-      <c r="CH52" s="24" t="n"/>
-      <c r="CI52" s="24" t="n"/>
-      <c r="CJ52" s="24" t="n"/>
-      <c r="CK52" s="24" t="n"/>
-      <c r="CL52" s="24" t="n"/>
-      <c r="CM52" s="24" t="n"/>
-      <c r="CN52" s="24" t="n"/>
-      <c r="CO52" s="24" t="n"/>
-      <c r="CP52" s="24" t="n"/>
-      <c r="CQ52" s="24" t="n"/>
-      <c r="CR52" s="24" t="n"/>
-      <c r="CS52" s="24" t="n"/>
-      <c r="CT52" s="24" t="n"/>
-      <c r="CU52" s="24" t="n"/>
-      <c r="CV52" s="24" t="n"/>
-      <c r="CW52" s="24" t="n"/>
-      <c r="CX52" s="24" t="n"/>
-      <c r="CY52" s="24" t="n"/>
-      <c r="CZ52" s="24" t="n"/>
-      <c r="DA52" s="24" t="n"/>
-      <c r="DB52" s="24" t="n"/>
-      <c r="DC52" s="24" t="n"/>
-      <c r="DD52" s="24" t="n"/>
-      <c r="DE52" s="24" t="n"/>
-      <c r="DF52" s="24" t="n"/>
-      <c r="DG52" s="24" t="n"/>
-      <c r="DH52" s="24" t="n"/>
-      <c r="DI52" s="24" t="n"/>
-      <c r="DJ52" s="24" t="n"/>
-      <c r="DK52" s="24" t="n"/>
-      <c r="DL52" s="24" t="n"/>
-      <c r="DM52" s="24" t="n"/>
-      <c r="DN52" s="24" t="n"/>
-      <c r="DO52" s="24" t="n"/>
-      <c r="DP52" s="24" t="n"/>
-    </row>
-    <row r="53" ht="36" customHeight="1">
-      <c r="A53" s="24" t="inlineStr">
-        <is>
-          <t>b214bda284bc4f41</t>
-        </is>
-      </c>
-      <c r="B53" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-31T16:12:42.599391Z</t>
-        </is>
-      </c>
-      <c r="C53" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-31T19:00:00Z</t>
-        </is>
-      </c>
-      <c r="D53" s="24" t="inlineStr">
-        <is>
-          <t>aec-cs2-dam-zge-2026-08-31</t>
-        </is>
-      </c>
-      <c r="E53" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F53" s="24" t="inlineStr">
-        <is>
-          <t>Zetta Games</t>
-        </is>
-      </c>
-      <c r="G53" s="24" t="inlineStr">
-        <is>
-          <t>Damajuana</t>
-        </is>
-      </c>
-      <c r="H53" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I53" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J53" s="25" t="n"/>
-      <c r="K53" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L53" s="26" t="n">
-        <v>212</v>
-      </c>
-      <c r="M53" s="27" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="N53" s="28" t="n">
-        <v>0.3205</v>
-      </c>
-      <c r="O53" s="28" t="n">
-        <v>0.5642</v>
-      </c>
-      <c r="P53" s="28" t="n"/>
-      <c r="Q53" s="28" t="n">
-        <v>0.2442</v>
-      </c>
-      <c r="R53" s="26" t="n"/>
-      <c r="S53" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="T53" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v6</t>
-        </is>
-      </c>
-      <c r="U53" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V53" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="W53" s="26" t="n"/>
-      <c r="X53" s="26" t="n"/>
-      <c r="Y53" s="25" t="n"/>
-      <c r="Z53" s="26" t="n"/>
-      <c r="AA53" s="28" t="n"/>
-      <c r="AB53" s="28" t="n"/>
-      <c r="AC53" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD53" s="24" t="n"/>
-      <c r="AE53" s="31" t="inlineStr">
-        <is>
-          <t>Auto-Buyer order C75ED9T52KDF on aec-cs2-dam-zge-2026-08-31 (short)</t>
-        </is>
-      </c>
-      <c r="AF53" s="31" t="n"/>
-      <c r="AG53" s="24" t="n"/>
-      <c r="AH53" s="24" t="n"/>
-      <c r="AI53" s="31" t="n"/>
-      <c r="AJ53" s="31" t="n"/>
-      <c r="AK53" s="24" t="n"/>
-      <c r="AL53" s="26" t="n">
-        <v>4</v>
-      </c>
-      <c r="AM53" s="24" t="inlineStr">
-        <is>
-          <t>decision</t>
-        </is>
-      </c>
-      <c r="AN53" s="24" t="inlineStr">
-        <is>
-          <t>take</t>
-        </is>
-      </c>
-      <c r="AO53" s="24" t="inlineStr">
-        <is>
-          <t>AUTO_BUYER_EXECUTION</t>
-        </is>
-      </c>
-      <c r="AP53" s="24" t="n"/>
-      <c r="AQ53" s="24" t="n"/>
-      <c r="AR53" s="24" t="n"/>
-      <c r="AS53" s="24" t="n"/>
-      <c r="AT53" s="24" t="n"/>
-      <c r="AU53" s="24" t="n"/>
-      <c r="AV53" s="24" t="n"/>
-      <c r="AW53" s="24" t="n"/>
-      <c r="AX53" s="24" t="n"/>
-      <c r="AY53" s="24" t="n"/>
-      <c r="AZ53" s="24" t="n"/>
-      <c r="BA53" s="24" t="n"/>
-      <c r="BB53" s="24" t="n"/>
-      <c r="BC53" s="24" t="n"/>
-      <c r="BD53" s="24" t="n"/>
-      <c r="BE53" s="24" t="n"/>
-      <c r="BF53" s="24" t="n"/>
-      <c r="BG53" s="24" t="n"/>
-      <c r="BH53" s="24" t="n"/>
-      <c r="BI53" s="24" t="n"/>
-      <c r="BJ53" s="25" t="n"/>
-      <c r="BK53" s="26" t="n"/>
-      <c r="BL53" s="27" t="n"/>
-      <c r="BM53" s="28" t="n"/>
-      <c r="BN53" s="28" t="n"/>
-      <c r="BO53" s="28" t="n"/>
-      <c r="BP53" s="25" t="n"/>
-      <c r="BQ53" s="27" t="n"/>
-      <c r="BR53" s="28" t="n"/>
-      <c r="BS53" s="28" t="n"/>
-      <c r="BT53" s="28" t="n"/>
-      <c r="BU53" s="25" t="n"/>
-      <c r="BV53" s="29" t="n"/>
-      <c r="BW53" s="24" t="n"/>
-      <c r="BX53" s="30" t="n"/>
-      <c r="BY53" s="27" t="n"/>
-      <c r="BZ53" s="24" t="n"/>
-      <c r="CA53" s="31" t="n"/>
-      <c r="CB53" s="24" t="n"/>
-      <c r="CC53" s="24" t="n"/>
-      <c r="CD53" s="24" t="n"/>
-      <c r="CE53" s="24" t="n"/>
-      <c r="CF53" s="24" t="n"/>
-      <c r="CG53" s="24" t="n"/>
-      <c r="CH53" s="24" t="n"/>
-      <c r="CI53" s="24" t="n"/>
-      <c r="CJ53" s="24" t="n"/>
-      <c r="CK53" s="24" t="n"/>
-      <c r="CL53" s="24" t="n"/>
-      <c r="CM53" s="24" t="n"/>
-      <c r="CN53" s="24" t="n"/>
-      <c r="CO53" s="24" t="n"/>
-      <c r="CP53" s="24" t="n"/>
-      <c r="CQ53" s="24" t="n"/>
-      <c r="CR53" s="24" t="n"/>
-      <c r="CS53" s="24" t="n"/>
-      <c r="CT53" s="24" t="n"/>
-      <c r="CU53" s="24" t="n"/>
-      <c r="CV53" s="24" t="n"/>
-      <c r="CW53" s="24" t="n"/>
-      <c r="CX53" s="24" t="n"/>
-      <c r="CY53" s="24" t="n"/>
-      <c r="CZ53" s="24" t="n"/>
-      <c r="DA53" s="24" t="n"/>
-      <c r="DB53" s="24" t="n"/>
-      <c r="DC53" s="24" t="n"/>
-      <c r="DD53" s="24" t="n"/>
-      <c r="DE53" s="24" t="n"/>
-      <c r="DF53" s="24" t="n"/>
-      <c r="DG53" s="24" t="n"/>
-      <c r="DH53" s="24" t="n"/>
-      <c r="DI53" s="24" t="n"/>
-      <c r="DJ53" s="24" t="n"/>
-      <c r="DK53" s="24" t="n"/>
-      <c r="DL53" s="24" t="n"/>
-      <c r="DM53" s="24" t="n"/>
-      <c r="DN53" s="24" t="n"/>
-      <c r="DO53" s="24" t="n"/>
-      <c r="DP53" s="24" t="n"/>
-    </row>
-    <row r="54" ht="36" customHeight="1">
-      <c r="A54" s="24" t="inlineStr">
-        <is>
-          <t>fd008ef45af2480d</t>
-        </is>
-      </c>
-      <c r="B54" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-31T16:12:42.599391Z</t>
-        </is>
-      </c>
-      <c r="C54" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-31T22:00:00Z</t>
-        </is>
-      </c>
-      <c r="D54" s="24" t="inlineStr">
-        <is>
-          <t>aec-cs2-mm-sdm-2026-08-31</t>
-        </is>
-      </c>
-      <c r="E54" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F54" s="24" t="inlineStr">
-        <is>
-          <t>Semente do Mal</t>
-        </is>
-      </c>
-      <c r="G54" s="24" t="inlineStr">
-        <is>
-          <t>Mansão Maromba</t>
-        </is>
-      </c>
-      <c r="H54" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I54" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J54" s="25" t="n"/>
-      <c r="K54" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L54" s="26" t="n">
-        <v>212</v>
-      </c>
-      <c r="M54" s="27" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="N54" s="28" t="n">
-        <v>0.3205</v>
-      </c>
-      <c r="O54" s="28" t="n">
-        <v>0.5066000000000001</v>
-      </c>
-      <c r="P54" s="28" t="n"/>
-      <c r="Q54" s="28" t="n">
-        <v>0.1866</v>
-      </c>
-      <c r="R54" s="26" t="n"/>
-      <c r="S54" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="T54" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v6</t>
-        </is>
-      </c>
-      <c r="U54" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V54" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="W54" s="26" t="n"/>
-      <c r="X54" s="26" t="n"/>
-      <c r="Y54" s="25" t="n"/>
-      <c r="Z54" s="26" t="n"/>
-      <c r="AA54" s="28" t="n"/>
-      <c r="AB54" s="28" t="n"/>
-      <c r="AC54" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD54" s="24" t="n"/>
-      <c r="AE54" s="31" t="inlineStr">
-        <is>
-          <t>Auto-Buyer order C75CWYWSTKDC on aec-cs2-mm-sdm-2026-08-31 (short)</t>
-        </is>
-      </c>
-      <c r="AF54" s="31" t="n"/>
-      <c r="AG54" s="24" t="n"/>
-      <c r="AH54" s="24" t="n"/>
-      <c r="AI54" s="31" t="n"/>
-      <c r="AJ54" s="31" t="n"/>
-      <c r="AK54" s="24" t="n"/>
-      <c r="AL54" s="26" t="n">
-        <v>4</v>
-      </c>
-      <c r="AM54" s="24" t="inlineStr">
-        <is>
-          <t>decision</t>
-        </is>
-      </c>
-      <c r="AN54" s="24" t="inlineStr">
-        <is>
-          <t>take</t>
-        </is>
-      </c>
-      <c r="AO54" s="24" t="inlineStr">
-        <is>
-          <t>AUTO_BUYER_EXECUTION</t>
-        </is>
-      </c>
-      <c r="AP54" s="24" t="n"/>
-      <c r="AQ54" s="24" t="n"/>
-      <c r="AR54" s="24" t="n"/>
-      <c r="AS54" s="24" t="n"/>
-      <c r="AT54" s="24" t="n"/>
-      <c r="AU54" s="24" t="n"/>
-      <c r="AV54" s="24" t="n"/>
-      <c r="AW54" s="24" t="n"/>
-      <c r="AX54" s="24" t="n"/>
-      <c r="AY54" s="24" t="n"/>
-      <c r="AZ54" s="24" t="n"/>
-      <c r="BA54" s="24" t="n"/>
-      <c r="BB54" s="24" t="n"/>
-      <c r="BC54" s="24" t="n"/>
-      <c r="BD54" s="24" t="n"/>
-      <c r="BE54" s="24" t="n"/>
-      <c r="BF54" s="24" t="n"/>
-      <c r="BG54" s="24" t="n"/>
-      <c r="BH54" s="24" t="n"/>
-      <c r="BI54" s="24" t="n"/>
-      <c r="BJ54" s="25" t="n"/>
-      <c r="BK54" s="26" t="n"/>
-      <c r="BL54" s="27" t="n"/>
-      <c r="BM54" s="28" t="n"/>
-      <c r="BN54" s="28" t="n"/>
-      <c r="BO54" s="28" t="n"/>
-      <c r="BP54" s="25" t="n"/>
-      <c r="BQ54" s="27" t="n"/>
-      <c r="BR54" s="28" t="n"/>
-      <c r="BS54" s="28" t="n"/>
-      <c r="BT54" s="28" t="n"/>
-      <c r="BU54" s="25" t="n"/>
-      <c r="BV54" s="29" t="n"/>
-      <c r="BW54" s="24" t="n"/>
-      <c r="BX54" s="30" t="n"/>
-      <c r="BY54" s="27" t="n"/>
-      <c r="BZ54" s="24" t="n"/>
-      <c r="CA54" s="31" t="n"/>
-      <c r="CB54" s="24" t="n"/>
-      <c r="CC54" s="24" t="n"/>
-      <c r="CD54" s="24" t="n"/>
-      <c r="CE54" s="24" t="n"/>
-      <c r="CF54" s="24" t="n"/>
-      <c r="CG54" s="24" t="n"/>
-      <c r="CH54" s="24" t="n"/>
-      <c r="CI54" s="24" t="n"/>
-      <c r="CJ54" s="24" t="n"/>
-      <c r="CK54" s="24" t="n"/>
-      <c r="CL54" s="24" t="n"/>
-      <c r="CM54" s="24" t="n"/>
-      <c r="CN54" s="24" t="n"/>
-      <c r="CO54" s="24" t="n"/>
-      <c r="CP54" s="24" t="n"/>
-      <c r="CQ54" s="24" t="n"/>
-      <c r="CR54" s="24" t="n"/>
-      <c r="CS54" s="24" t="n"/>
-      <c r="CT54" s="24" t="n"/>
-      <c r="CU54" s="24" t="n"/>
-      <c r="CV54" s="24" t="n"/>
-      <c r="CW54" s="24" t="n"/>
-      <c r="CX54" s="24" t="n"/>
-      <c r="CY54" s="24" t="n"/>
-      <c r="CZ54" s="24" t="n"/>
-      <c r="DA54" s="24" t="n"/>
-      <c r="DB54" s="24" t="n"/>
-      <c r="DC54" s="24" t="n"/>
-      <c r="DD54" s="24" t="n"/>
-      <c r="DE54" s="24" t="n"/>
-      <c r="DF54" s="24" t="n"/>
-      <c r="DG54" s="24" t="n"/>
-      <c r="DH54" s="24" t="n"/>
-      <c r="DI54" s="24" t="n"/>
-      <c r="DJ54" s="24" t="n"/>
-      <c r="DK54" s="24" t="n"/>
-      <c r="DL54" s="24" t="n"/>
-      <c r="DM54" s="24" t="n"/>
-      <c r="DN54" s="24" t="n"/>
-      <c r="DO54" s="24" t="n"/>
-      <c r="DP54" s="24" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix(auto-buyer): reconcile IOC fills and rest unfilled remainder at same price
Auto-Buyer was recording requested quantity/cost as filled even when the
exchange only partially or fully failed to fill an IOC order, corrupting
ledger and daily-spend accounting. Reconcile against actual cumQuantity,
and place any unfilled remainder as a resting GTC order at the original
price instead of chasing the ask with a marketable order.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/auto_buyer_picks.xlsx
+++ b/data/auto_buyer_picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DP103" headerRowCount="1">
-  <autoFilter ref="A1:DP103"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DP122" headerRowCount="1">
+  <autoFilter ref="A1:DP122"/>
   <tableColumns count="120">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -779,19 +779,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$103)</f>
+        <f>COUNTA('Picks'!$A$2:$A$122)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$103,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$122,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$103,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$122,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$103,"settled",'Picks'!$V$2:$V$103,"win")+COUNTIFS('Picks'!$U$2:$U$103,"settled",'Picks'!$V$2:$V$103,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"win")+COUNTIFS('Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -819,19 +819,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$103,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$122,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$103,"&gt;0",'Picks'!$V$2:$V$103,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$103,"&gt;0",'Picks'!$V$2:$V$103,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$103,"&gt;0",'Picks'!$V$2:$V$103,"win")/(COUNTIFS('Picks'!$BX$2:$BX$103,"&gt;0",'Picks'!$V$2:$V$103,"win")+COUNTIFS('Picks'!$BX$2:$BX$103,"&gt;0",'Picks'!$V$2:$V$103,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"win")/(COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"win")+COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$103)/SUM('Picks'!$BX$2:$BX$103),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$122)/SUM('Picks'!$BX$2:$BX$122),0)</f>
         <v/>
       </c>
     </row>
@@ -859,19 +859,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$103)</f>
+        <f>SUM('Picks'!$BY$2:$BY$122)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$103,"&lt;&gt;",'Picks'!$AB$2:$AB$103),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$122,"&lt;&gt;",'Picks'!$AB$2:$AB$122),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$103,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$103,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$122,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$122,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$103,'Picks'!$AM$2:$AM$103,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$122,'Picks'!$AM$2:$AM$122,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -926,15 +926,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A14,'Picks'!$U$2:$U$103,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A14,'Picks'!$U$2:$U$122,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A14,'Picks'!$U$2:$U$103,"settled",'Picks'!$V$2:$V$103,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A14,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A14,'Picks'!$U$2:$U$103,"settled",'Picks'!$V$2:$V$103,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A14,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -942,11 +942,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$103,'Picks'!$H$2:$H$103,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$122,'Picks'!$H$2:$H$122,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$103,'Picks'!$H$2:$H$103,$A14,'Picks'!$U$2:$U$103,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$122,'Picks'!$H$2:$H$122,$A14,'Picks'!$U$2:$U$122,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -957,15 +957,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A15,'Picks'!$U$2:$U$103,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A15,'Picks'!$U$2:$U$122,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A15,'Picks'!$U$2:$U$103,"settled",'Picks'!$V$2:$V$103,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A15,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A15,'Picks'!$U$2:$U$103,"settled",'Picks'!$V$2:$V$103,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A15,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -973,11 +973,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$103,'Picks'!$H$2:$H$103,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$122,'Picks'!$H$2:$H$122,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$103,'Picks'!$H$2:$H$103,$A15,'Picks'!$U$2:$U$103,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$122,'Picks'!$H$2:$H$122,$A15,'Picks'!$U$2:$U$122,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -988,15 +988,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A16,'Picks'!$U$2:$U$103,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A16,'Picks'!$U$2:$U$122,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A16,'Picks'!$U$2:$U$103,"settled",'Picks'!$V$2:$V$103,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A16,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$103,$A16,'Picks'!$U$2:$U$103,"settled",'Picks'!$V$2:$V$103,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$122,$A16,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -1004,11 +1004,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$103,'Picks'!$H$2:$H$103,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$122,'Picks'!$H$2:$H$122,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$103,'Picks'!$H$2:$H$103,$A16,'Picks'!$U$2:$U$103,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$122,'Picks'!$H$2:$H$122,$A16,'Picks'!$U$2:$U$122,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DP103"/>
+  <dimension ref="A1:DP122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21467,12 +21467,12 @@
       </c>
       <c r="U95" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V95" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W95" s="26" t="n"/>
@@ -21482,9 +21482,13 @@
       <c r="AA95" s="28" t="n"/>
       <c r="AB95" s="28" t="n"/>
       <c r="AC95" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD95" s="24" t="n"/>
+        <v>1.22</v>
+      </c>
+      <c r="AD95" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:41:14.239238Z</t>
+        </is>
+      </c>
       <c r="AE95" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8EPAWWCYMVK on aec-cs2-is-nemi-2026-09-03 (short)</t>
@@ -23135,12 +23139,12 @@
       </c>
       <c r="U103" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V103" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="W103" s="26" t="n"/>
@@ -23150,9 +23154,13 @@
       <c r="AA103" s="28" t="n"/>
       <c r="AB103" s="28" t="n"/>
       <c r="AC103" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD103" s="24" t="n"/>
+        <v>-1.02</v>
+      </c>
+      <c r="AD103" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:41:14.239238Z</t>
+        </is>
+      </c>
       <c r="AE103" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8EQT1EM2MVG on aec-cs2-sin-fokus-2026-09-03 (long)</t>
@@ -23262,6 +23270,3944 @@
       <c r="DO103" s="24" t="n"/>
       <c r="DP103" s="24" t="n"/>
     </row>
+    <row r="104" ht="36" customHeight="1">
+      <c r="A104" s="24" t="inlineStr">
+        <is>
+          <t>12fa89f6e495470b</t>
+        </is>
+      </c>
+      <c r="B104" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C104" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T01:00Z</t>
+        </is>
+      </c>
+      <c r="D104" s="24" t="inlineStr">
+        <is>
+          <t>aec-wta-jesman-eleryb-2026-09-02</t>
+        </is>
+      </c>
+      <c r="E104" s="24" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+      <c r="F104" s="24" t="inlineStr">
+        <is>
+          <t>Elena Rybakina</t>
+        </is>
+      </c>
+      <c r="G104" s="24" t="inlineStr">
+        <is>
+          <t>Jessica Bouzas Maneiro</t>
+        </is>
+      </c>
+      <c r="H104" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I104" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J104" s="25" t="n"/>
+      <c r="K104" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L104" s="26" t="n">
+        <v>-525</v>
+      </c>
+      <c r="M104" s="27" t="n">
+        <v>1.1905</v>
+      </c>
+      <c r="N104" s="28" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="O104" s="28" t="n">
+        <v>0.9249000000000001</v>
+      </c>
+      <c r="P104" s="28" t="n"/>
+      <c r="Q104" s="28" t="n">
+        <v>0.0849</v>
+      </c>
+      <c r="R104" s="26" t="n"/>
+      <c r="S104" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T104" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U104" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V104" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W104" s="26" t="n"/>
+      <c r="X104" s="26" t="n"/>
+      <c r="Y104" s="25" t="n"/>
+      <c r="Z104" s="26" t="n"/>
+      <c r="AA104" s="28" t="n"/>
+      <c r="AB104" s="28" t="n"/>
+      <c r="AC104" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD104" s="24" t="n"/>
+      <c r="AE104" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SAC97KPMW0 on aec-wta-jesman-eleryb-2026-09-02 (short)</t>
+        </is>
+      </c>
+      <c r="AF104" s="31" t="n"/>
+      <c r="AG104" s="24" t="n"/>
+      <c r="AH104" s="24" t="n"/>
+      <c r="AI104" s="31" t="n"/>
+      <c r="AJ104" s="31" t="n"/>
+      <c r="AK104" s="24" t="n"/>
+      <c r="AL104" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM104" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN104" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO104" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP104" s="24" t="n"/>
+      <c r="AQ104" s="24" t="n"/>
+      <c r="AR104" s="24" t="n"/>
+      <c r="AS104" s="24" t="n"/>
+      <c r="AT104" s="24" t="n"/>
+      <c r="AU104" s="24" t="n"/>
+      <c r="AV104" s="24" t="n"/>
+      <c r="AW104" s="24" t="n"/>
+      <c r="AX104" s="24" t="n"/>
+      <c r="AY104" s="24" t="n"/>
+      <c r="AZ104" s="24" t="n"/>
+      <c r="BA104" s="24" t="n"/>
+      <c r="BB104" s="24" t="n"/>
+      <c r="BC104" s="24" t="n"/>
+      <c r="BD104" s="24" t="n"/>
+      <c r="BE104" s="24" t="n"/>
+      <c r="BF104" s="24" t="n"/>
+      <c r="BG104" s="24" t="n"/>
+      <c r="BH104" s="24" t="n"/>
+      <c r="BI104" s="24" t="n"/>
+      <c r="BJ104" s="25" t="n"/>
+      <c r="BK104" s="26" t="n"/>
+      <c r="BL104" s="27" t="n"/>
+      <c r="BM104" s="28" t="n"/>
+      <c r="BN104" s="28" t="n"/>
+      <c r="BO104" s="28" t="n"/>
+      <c r="BP104" s="25" t="n"/>
+      <c r="BQ104" s="27" t="n"/>
+      <c r="BR104" s="28" t="n"/>
+      <c r="BS104" s="28" t="n"/>
+      <c r="BT104" s="28" t="n"/>
+      <c r="BU104" s="25" t="n"/>
+      <c r="BV104" s="29" t="n"/>
+      <c r="BW104" s="24" t="n"/>
+      <c r="BX104" s="30" t="n"/>
+      <c r="BY104" s="27" t="n"/>
+      <c r="BZ104" s="24" t="n"/>
+      <c r="CA104" s="31" t="n"/>
+      <c r="CB104" s="24" t="n"/>
+      <c r="CC104" s="24" t="n"/>
+      <c r="CD104" s="24" t="n"/>
+      <c r="CE104" s="24" t="n"/>
+      <c r="CF104" s="24" t="n"/>
+      <c r="CG104" s="24" t="n"/>
+      <c r="CH104" s="24" t="n"/>
+      <c r="CI104" s="24" t="n"/>
+      <c r="CJ104" s="24" t="n"/>
+      <c r="CK104" s="24" t="n"/>
+      <c r="CL104" s="24" t="n"/>
+      <c r="CM104" s="24" t="n"/>
+      <c r="CN104" s="24" t="n"/>
+      <c r="CO104" s="24" t="n"/>
+      <c r="CP104" s="24" t="n"/>
+      <c r="CQ104" s="24" t="n"/>
+      <c r="CR104" s="24" t="n"/>
+      <c r="CS104" s="24" t="n"/>
+      <c r="CT104" s="24" t="n"/>
+      <c r="CU104" s="24" t="n"/>
+      <c r="CV104" s="24" t="n"/>
+      <c r="CW104" s="24" t="n"/>
+      <c r="CX104" s="24" t="n"/>
+      <c r="CY104" s="24" t="n"/>
+      <c r="CZ104" s="24" t="n"/>
+      <c r="DA104" s="24" t="n"/>
+      <c r="DB104" s="24" t="n"/>
+      <c r="DC104" s="24" t="n"/>
+      <c r="DD104" s="24" t="n"/>
+      <c r="DE104" s="24" t="n"/>
+      <c r="DF104" s="24" t="n"/>
+      <c r="DG104" s="24" t="n"/>
+      <c r="DH104" s="24" t="n"/>
+      <c r="DI104" s="24" t="n"/>
+      <c r="DJ104" s="24" t="n"/>
+      <c r="DK104" s="24" t="n"/>
+      <c r="DL104" s="24" t="n"/>
+      <c r="DM104" s="24" t="n"/>
+      <c r="DN104" s="24" t="n"/>
+      <c r="DO104" s="24" t="n"/>
+      <c r="DP104" s="24" t="n"/>
+    </row>
+    <row r="105" ht="36" customHeight="1">
+      <c r="A105" s="24" t="inlineStr">
+        <is>
+          <t>e9bef91be0644ef4</t>
+        </is>
+      </c>
+      <c r="B105" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C105" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:00Z</t>
+        </is>
+      </c>
+      <c r="D105" s="24" t="inlineStr">
+        <is>
+          <t>aec-atp-felaug-karkha-2026-09-02</t>
+        </is>
+      </c>
+      <c r="E105" s="24" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+      <c r="F105" s="24" t="inlineStr">
+        <is>
+          <t>Karen Khachanov</t>
+        </is>
+      </c>
+      <c r="G105" s="24" t="inlineStr">
+        <is>
+          <t>Felix Auger-Aliassime</t>
+        </is>
+      </c>
+      <c r="H105" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I105" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J105" s="25" t="n"/>
+      <c r="K105" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L105" s="26" t="n">
+        <v>-257</v>
+      </c>
+      <c r="M105" s="27" t="n">
+        <v>1.3891</v>
+      </c>
+      <c r="N105" s="28" t="n">
+        <v>0.7199</v>
+      </c>
+      <c r="O105" s="28" t="n">
+        <v>0.7754</v>
+      </c>
+      <c r="P105" s="28" t="n"/>
+      <c r="Q105" s="28" t="n">
+        <v>0.0554</v>
+      </c>
+      <c r="R105" s="26" t="n"/>
+      <c r="S105" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T105" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U105" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V105" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W105" s="26" t="n"/>
+      <c r="X105" s="26" t="n"/>
+      <c r="Y105" s="25" t="n"/>
+      <c r="Z105" s="26" t="n"/>
+      <c r="AA105" s="28" t="n"/>
+      <c r="AB105" s="28" t="n"/>
+      <c r="AC105" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD105" s="24" t="n"/>
+      <c r="AE105" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8S9JGNDPMVY on aec-atp-felaug-karkha-2026-09-02 (long)</t>
+        </is>
+      </c>
+      <c r="AF105" s="31" t="n"/>
+      <c r="AG105" s="24" t="n"/>
+      <c r="AH105" s="24" t="n"/>
+      <c r="AI105" s="31" t="n"/>
+      <c r="AJ105" s="31" t="n"/>
+      <c r="AK105" s="24" t="n"/>
+      <c r="AL105" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM105" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN105" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO105" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP105" s="24" t="n"/>
+      <c r="AQ105" s="24" t="n"/>
+      <c r="AR105" s="24" t="n"/>
+      <c r="AS105" s="24" t="n"/>
+      <c r="AT105" s="24" t="n"/>
+      <c r="AU105" s="24" t="n"/>
+      <c r="AV105" s="24" t="n"/>
+      <c r="AW105" s="24" t="n"/>
+      <c r="AX105" s="24" t="n"/>
+      <c r="AY105" s="24" t="n"/>
+      <c r="AZ105" s="24" t="n"/>
+      <c r="BA105" s="24" t="n"/>
+      <c r="BB105" s="24" t="n"/>
+      <c r="BC105" s="24" t="n"/>
+      <c r="BD105" s="24" t="n"/>
+      <c r="BE105" s="24" t="n"/>
+      <c r="BF105" s="24" t="n"/>
+      <c r="BG105" s="24" t="n"/>
+      <c r="BH105" s="24" t="n"/>
+      <c r="BI105" s="24" t="n"/>
+      <c r="BJ105" s="25" t="n"/>
+      <c r="BK105" s="26" t="n"/>
+      <c r="BL105" s="27" t="n"/>
+      <c r="BM105" s="28" t="n"/>
+      <c r="BN105" s="28" t="n"/>
+      <c r="BO105" s="28" t="n"/>
+      <c r="BP105" s="25" t="n"/>
+      <c r="BQ105" s="27" t="n"/>
+      <c r="BR105" s="28" t="n"/>
+      <c r="BS105" s="28" t="n"/>
+      <c r="BT105" s="28" t="n"/>
+      <c r="BU105" s="25" t="n"/>
+      <c r="BV105" s="29" t="n"/>
+      <c r="BW105" s="24" t="n"/>
+      <c r="BX105" s="30" t="n"/>
+      <c r="BY105" s="27" t="n"/>
+      <c r="BZ105" s="24" t="n"/>
+      <c r="CA105" s="31" t="n"/>
+      <c r="CB105" s="24" t="n"/>
+      <c r="CC105" s="24" t="n"/>
+      <c r="CD105" s="24" t="n"/>
+      <c r="CE105" s="24" t="n"/>
+      <c r="CF105" s="24" t="n"/>
+      <c r="CG105" s="24" t="n"/>
+      <c r="CH105" s="24" t="n"/>
+      <c r="CI105" s="24" t="n"/>
+      <c r="CJ105" s="24" t="n"/>
+      <c r="CK105" s="24" t="n"/>
+      <c r="CL105" s="24" t="n"/>
+      <c r="CM105" s="24" t="n"/>
+      <c r="CN105" s="24" t="n"/>
+      <c r="CO105" s="24" t="n"/>
+      <c r="CP105" s="24" t="n"/>
+      <c r="CQ105" s="24" t="n"/>
+      <c r="CR105" s="24" t="n"/>
+      <c r="CS105" s="24" t="n"/>
+      <c r="CT105" s="24" t="n"/>
+      <c r="CU105" s="24" t="n"/>
+      <c r="CV105" s="24" t="n"/>
+      <c r="CW105" s="24" t="n"/>
+      <c r="CX105" s="24" t="n"/>
+      <c r="CY105" s="24" t="n"/>
+      <c r="CZ105" s="24" t="n"/>
+      <c r="DA105" s="24" t="n"/>
+      <c r="DB105" s="24" t="n"/>
+      <c r="DC105" s="24" t="n"/>
+      <c r="DD105" s="24" t="n"/>
+      <c r="DE105" s="24" t="n"/>
+      <c r="DF105" s="24" t="n"/>
+      <c r="DG105" s="24" t="n"/>
+      <c r="DH105" s="24" t="n"/>
+      <c r="DI105" s="24" t="n"/>
+      <c r="DJ105" s="24" t="n"/>
+      <c r="DK105" s="24" t="n"/>
+      <c r="DL105" s="24" t="n"/>
+      <c r="DM105" s="24" t="n"/>
+      <c r="DN105" s="24" t="n"/>
+      <c r="DO105" s="24" t="n"/>
+      <c r="DP105" s="24" t="n"/>
+    </row>
+    <row r="106" ht="36" customHeight="1">
+      <c r="A106" s="24" t="inlineStr">
+        <is>
+          <t>ec2906bb14b24356</t>
+        </is>
+      </c>
+      <c r="B106" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C106" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:00Z</t>
+        </is>
+      </c>
+      <c r="D106" s="24" t="inlineStr">
+        <is>
+          <t>aec-atp-lucdar-dalsvr-2026-09-02</t>
+        </is>
+      </c>
+      <c r="E106" s="24" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+      <c r="F106" s="24" t="inlineStr">
+        <is>
+          <t>Dalibor Svrcina</t>
+        </is>
+      </c>
+      <c r="G106" s="24" t="inlineStr">
+        <is>
+          <t>Luciano Darderi</t>
+        </is>
+      </c>
+      <c r="H106" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I106" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J106" s="25" t="n"/>
+      <c r="K106" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L106" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="M106" s="27" t="n">
+        <v>1.7519</v>
+      </c>
+      <c r="N106" s="28" t="n">
+        <v>0.5708</v>
+      </c>
+      <c r="O106" s="28" t="n">
+        <v>0.6375999999999999</v>
+      </c>
+      <c r="P106" s="28" t="n"/>
+      <c r="Q106" s="28" t="n">
+        <v>0.06759999999999999</v>
+      </c>
+      <c r="R106" s="26" t="n"/>
+      <c r="S106" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T106" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U106" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V106" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W106" s="26" t="n"/>
+      <c r="X106" s="26" t="n"/>
+      <c r="Y106" s="25" t="n"/>
+      <c r="Z106" s="26" t="n"/>
+      <c r="AA106" s="28" t="n"/>
+      <c r="AB106" s="28" t="n"/>
+      <c r="AC106" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD106" s="24" t="n"/>
+      <c r="AE106" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SAJ717GMVR on aec-atp-lucdar-dalsvr-2026-09-02 (long)</t>
+        </is>
+      </c>
+      <c r="AF106" s="31" t="n"/>
+      <c r="AG106" s="24" t="n"/>
+      <c r="AH106" s="24" t="n"/>
+      <c r="AI106" s="31" t="n"/>
+      <c r="AJ106" s="31" t="n"/>
+      <c r="AK106" s="24" t="n"/>
+      <c r="AL106" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM106" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN106" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO106" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP106" s="24" t="n"/>
+      <c r="AQ106" s="24" t="n"/>
+      <c r="AR106" s="24" t="n"/>
+      <c r="AS106" s="24" t="n"/>
+      <c r="AT106" s="24" t="n"/>
+      <c r="AU106" s="24" t="n"/>
+      <c r="AV106" s="24" t="n"/>
+      <c r="AW106" s="24" t="n"/>
+      <c r="AX106" s="24" t="n"/>
+      <c r="AY106" s="24" t="n"/>
+      <c r="AZ106" s="24" t="n"/>
+      <c r="BA106" s="24" t="n"/>
+      <c r="BB106" s="24" t="n"/>
+      <c r="BC106" s="24" t="n"/>
+      <c r="BD106" s="24" t="n"/>
+      <c r="BE106" s="24" t="n"/>
+      <c r="BF106" s="24" t="n"/>
+      <c r="BG106" s="24" t="n"/>
+      <c r="BH106" s="24" t="n"/>
+      <c r="BI106" s="24" t="n"/>
+      <c r="BJ106" s="25" t="n"/>
+      <c r="BK106" s="26" t="n"/>
+      <c r="BL106" s="27" t="n"/>
+      <c r="BM106" s="28" t="n"/>
+      <c r="BN106" s="28" t="n"/>
+      <c r="BO106" s="28" t="n"/>
+      <c r="BP106" s="25" t="n"/>
+      <c r="BQ106" s="27" t="n"/>
+      <c r="BR106" s="28" t="n"/>
+      <c r="BS106" s="28" t="n"/>
+      <c r="BT106" s="28" t="n"/>
+      <c r="BU106" s="25" t="n"/>
+      <c r="BV106" s="29" t="n"/>
+      <c r="BW106" s="24" t="n"/>
+      <c r="BX106" s="30" t="n"/>
+      <c r="BY106" s="27" t="n"/>
+      <c r="BZ106" s="24" t="n"/>
+      <c r="CA106" s="31" t="n"/>
+      <c r="CB106" s="24" t="n"/>
+      <c r="CC106" s="24" t="n"/>
+      <c r="CD106" s="24" t="n"/>
+      <c r="CE106" s="24" t="n"/>
+      <c r="CF106" s="24" t="n"/>
+      <c r="CG106" s="24" t="n"/>
+      <c r="CH106" s="24" t="n"/>
+      <c r="CI106" s="24" t="n"/>
+      <c r="CJ106" s="24" t="n"/>
+      <c r="CK106" s="24" t="n"/>
+      <c r="CL106" s="24" t="n"/>
+      <c r="CM106" s="24" t="n"/>
+      <c r="CN106" s="24" t="n"/>
+      <c r="CO106" s="24" t="n"/>
+      <c r="CP106" s="24" t="n"/>
+      <c r="CQ106" s="24" t="n"/>
+      <c r="CR106" s="24" t="n"/>
+      <c r="CS106" s="24" t="n"/>
+      <c r="CT106" s="24" t="n"/>
+      <c r="CU106" s="24" t="n"/>
+      <c r="CV106" s="24" t="n"/>
+      <c r="CW106" s="24" t="n"/>
+      <c r="CX106" s="24" t="n"/>
+      <c r="CY106" s="24" t="n"/>
+      <c r="CZ106" s="24" t="n"/>
+      <c r="DA106" s="24" t="n"/>
+      <c r="DB106" s="24" t="n"/>
+      <c r="DC106" s="24" t="n"/>
+      <c r="DD106" s="24" t="n"/>
+      <c r="DE106" s="24" t="n"/>
+      <c r="DF106" s="24" t="n"/>
+      <c r="DG106" s="24" t="n"/>
+      <c r="DH106" s="24" t="n"/>
+      <c r="DI106" s="24" t="n"/>
+      <c r="DJ106" s="24" t="n"/>
+      <c r="DK106" s="24" t="n"/>
+      <c r="DL106" s="24" t="n"/>
+      <c r="DM106" s="24" t="n"/>
+      <c r="DN106" s="24" t="n"/>
+      <c r="DO106" s="24" t="n"/>
+      <c r="DP106" s="24" t="n"/>
+    </row>
+    <row r="107" ht="36" customHeight="1">
+      <c r="A107" s="24" t="inlineStr">
+        <is>
+          <t>ad4dfd69909b43b5</t>
+        </is>
+      </c>
+      <c r="B107" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C107" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:00Z</t>
+        </is>
+      </c>
+      <c r="D107" s="24" t="inlineStr">
+        <is>
+          <t>aec-atp-janstr-fracer-2026-09-02</t>
+        </is>
+      </c>
+      <c r="E107" s="24" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+      <c r="F107" s="24" t="inlineStr">
+        <is>
+          <t>Francisco Cerundolo</t>
+        </is>
+      </c>
+      <c r="G107" s="24" t="inlineStr">
+        <is>
+          <t>Jan-Lennard Struff</t>
+        </is>
+      </c>
+      <c r="H107" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I107" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J107" s="25" t="n"/>
+      <c r="K107" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L107" s="26" t="n">
+        <v>-156</v>
+      </c>
+      <c r="M107" s="27" t="n">
+        <v>1.641</v>
+      </c>
+      <c r="N107" s="28" t="n">
+        <v>0.6094000000000001</v>
+      </c>
+      <c r="O107" s="28" t="n">
+        <v>0.7209</v>
+      </c>
+      <c r="P107" s="28" t="n"/>
+      <c r="Q107" s="28" t="n">
+        <v>0.1109</v>
+      </c>
+      <c r="R107" s="26" t="n"/>
+      <c r="S107" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T107" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U107" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V107" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W107" s="26" t="n"/>
+      <c r="X107" s="26" t="n"/>
+      <c r="Y107" s="25" t="n"/>
+      <c r="Z107" s="26" t="n"/>
+      <c r="AA107" s="28" t="n"/>
+      <c r="AB107" s="28" t="n"/>
+      <c r="AC107" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD107" s="24" t="n"/>
+      <c r="AE107" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SA9KYNEMVF on aec-atp-janstr-fracer-2026-09-02 (short)</t>
+        </is>
+      </c>
+      <c r="AF107" s="31" t="n"/>
+      <c r="AG107" s="24" t="n"/>
+      <c r="AH107" s="24" t="n"/>
+      <c r="AI107" s="31" t="n"/>
+      <c r="AJ107" s="31" t="n"/>
+      <c r="AK107" s="24" t="n"/>
+      <c r="AL107" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM107" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN107" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO107" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP107" s="24" t="n"/>
+      <c r="AQ107" s="24" t="n"/>
+      <c r="AR107" s="24" t="n"/>
+      <c r="AS107" s="24" t="n"/>
+      <c r="AT107" s="24" t="n"/>
+      <c r="AU107" s="24" t="n"/>
+      <c r="AV107" s="24" t="n"/>
+      <c r="AW107" s="24" t="n"/>
+      <c r="AX107" s="24" t="n"/>
+      <c r="AY107" s="24" t="n"/>
+      <c r="AZ107" s="24" t="n"/>
+      <c r="BA107" s="24" t="n"/>
+      <c r="BB107" s="24" t="n"/>
+      <c r="BC107" s="24" t="n"/>
+      <c r="BD107" s="24" t="n"/>
+      <c r="BE107" s="24" t="n"/>
+      <c r="BF107" s="24" t="n"/>
+      <c r="BG107" s="24" t="n"/>
+      <c r="BH107" s="24" t="n"/>
+      <c r="BI107" s="24" t="n"/>
+      <c r="BJ107" s="25" t="n"/>
+      <c r="BK107" s="26" t="n"/>
+      <c r="BL107" s="27" t="n"/>
+      <c r="BM107" s="28" t="n"/>
+      <c r="BN107" s="28" t="n"/>
+      <c r="BO107" s="28" t="n"/>
+      <c r="BP107" s="25" t="n"/>
+      <c r="BQ107" s="27" t="n"/>
+      <c r="BR107" s="28" t="n"/>
+      <c r="BS107" s="28" t="n"/>
+      <c r="BT107" s="28" t="n"/>
+      <c r="BU107" s="25" t="n"/>
+      <c r="BV107" s="29" t="n"/>
+      <c r="BW107" s="24" t="n"/>
+      <c r="BX107" s="30" t="n"/>
+      <c r="BY107" s="27" t="n"/>
+      <c r="BZ107" s="24" t="n"/>
+      <c r="CA107" s="31" t="n"/>
+      <c r="CB107" s="24" t="n"/>
+      <c r="CC107" s="24" t="n"/>
+      <c r="CD107" s="24" t="n"/>
+      <c r="CE107" s="24" t="n"/>
+      <c r="CF107" s="24" t="n"/>
+      <c r="CG107" s="24" t="n"/>
+      <c r="CH107" s="24" t="n"/>
+      <c r="CI107" s="24" t="n"/>
+      <c r="CJ107" s="24" t="n"/>
+      <c r="CK107" s="24" t="n"/>
+      <c r="CL107" s="24" t="n"/>
+      <c r="CM107" s="24" t="n"/>
+      <c r="CN107" s="24" t="n"/>
+      <c r="CO107" s="24" t="n"/>
+      <c r="CP107" s="24" t="n"/>
+      <c r="CQ107" s="24" t="n"/>
+      <c r="CR107" s="24" t="n"/>
+      <c r="CS107" s="24" t="n"/>
+      <c r="CT107" s="24" t="n"/>
+      <c r="CU107" s="24" t="n"/>
+      <c r="CV107" s="24" t="n"/>
+      <c r="CW107" s="24" t="n"/>
+      <c r="CX107" s="24" t="n"/>
+      <c r="CY107" s="24" t="n"/>
+      <c r="CZ107" s="24" t="n"/>
+      <c r="DA107" s="24" t="n"/>
+      <c r="DB107" s="24" t="n"/>
+      <c r="DC107" s="24" t="n"/>
+      <c r="DD107" s="24" t="n"/>
+      <c r="DE107" s="24" t="n"/>
+      <c r="DF107" s="24" t="n"/>
+      <c r="DG107" s="24" t="n"/>
+      <c r="DH107" s="24" t="n"/>
+      <c r="DI107" s="24" t="n"/>
+      <c r="DJ107" s="24" t="n"/>
+      <c r="DK107" s="24" t="n"/>
+      <c r="DL107" s="24" t="n"/>
+      <c r="DM107" s="24" t="n"/>
+      <c r="DN107" s="24" t="n"/>
+      <c r="DO107" s="24" t="n"/>
+      <c r="DP107" s="24" t="n"/>
+    </row>
+    <row r="108" ht="36" customHeight="1">
+      <c r="A108" s="24" t="inlineStr">
+        <is>
+          <t>5eb9281023994c1d</t>
+        </is>
+      </c>
+      <c r="B108" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C108" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T20:00Z</t>
+        </is>
+      </c>
+      <c r="D108" s="24" t="inlineStr">
+        <is>
+          <t>aec-atp-benbon-ignbus-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E108" s="24" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+      <c r="F108" s="24" t="inlineStr">
+        <is>
+          <t>Ignacio Buse</t>
+        </is>
+      </c>
+      <c r="G108" s="24" t="inlineStr">
+        <is>
+          <t>Benjamin Bonzi</t>
+        </is>
+      </c>
+      <c r="H108" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I108" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J108" s="25" t="n"/>
+      <c r="K108" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L108" s="26" t="n">
+        <v>138</v>
+      </c>
+      <c r="M108" s="27" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="N108" s="28" t="n">
+        <v>0.4255</v>
+      </c>
+      <c r="O108" s="28" t="n">
+        <v>0.5246</v>
+      </c>
+      <c r="P108" s="28" t="n"/>
+      <c r="Q108" s="28" t="n">
+        <v>0.09959999999999999</v>
+      </c>
+      <c r="R108" s="26" t="n"/>
+      <c r="S108" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T108" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U108" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V108" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W108" s="26" t="n"/>
+      <c r="X108" s="26" t="n"/>
+      <c r="Y108" s="25" t="n"/>
+      <c r="Z108" s="26" t="n"/>
+      <c r="AA108" s="28" t="n"/>
+      <c r="AB108" s="28" t="n"/>
+      <c r="AC108" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD108" s="24" t="n"/>
+      <c r="AE108" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8S9RQ5K2MVZ on aec-atp-benbon-ignbus-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF108" s="31" t="n"/>
+      <c r="AG108" s="24" t="n"/>
+      <c r="AH108" s="24" t="n"/>
+      <c r="AI108" s="31" t="n"/>
+      <c r="AJ108" s="31" t="n"/>
+      <c r="AK108" s="24" t="n"/>
+      <c r="AL108" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM108" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN108" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO108" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP108" s="24" t="n"/>
+      <c r="AQ108" s="24" t="n"/>
+      <c r="AR108" s="24" t="n"/>
+      <c r="AS108" s="24" t="n"/>
+      <c r="AT108" s="24" t="n"/>
+      <c r="AU108" s="24" t="n"/>
+      <c r="AV108" s="24" t="n"/>
+      <c r="AW108" s="24" t="n"/>
+      <c r="AX108" s="24" t="n"/>
+      <c r="AY108" s="24" t="n"/>
+      <c r="AZ108" s="24" t="n"/>
+      <c r="BA108" s="24" t="n"/>
+      <c r="BB108" s="24" t="n"/>
+      <c r="BC108" s="24" t="n"/>
+      <c r="BD108" s="24" t="n"/>
+      <c r="BE108" s="24" t="n"/>
+      <c r="BF108" s="24" t="n"/>
+      <c r="BG108" s="24" t="n"/>
+      <c r="BH108" s="24" t="n"/>
+      <c r="BI108" s="24" t="n"/>
+      <c r="BJ108" s="25" t="n"/>
+      <c r="BK108" s="26" t="n"/>
+      <c r="BL108" s="27" t="n"/>
+      <c r="BM108" s="28" t="n"/>
+      <c r="BN108" s="28" t="n"/>
+      <c r="BO108" s="28" t="n"/>
+      <c r="BP108" s="25" t="n"/>
+      <c r="BQ108" s="27" t="n"/>
+      <c r="BR108" s="28" t="n"/>
+      <c r="BS108" s="28" t="n"/>
+      <c r="BT108" s="28" t="n"/>
+      <c r="BU108" s="25" t="n"/>
+      <c r="BV108" s="29" t="n"/>
+      <c r="BW108" s="24" t="n"/>
+      <c r="BX108" s="30" t="n"/>
+      <c r="BY108" s="27" t="n"/>
+      <c r="BZ108" s="24" t="n"/>
+      <c r="CA108" s="31" t="n"/>
+      <c r="CB108" s="24" t="n"/>
+      <c r="CC108" s="24" t="n"/>
+      <c r="CD108" s="24" t="n"/>
+      <c r="CE108" s="24" t="n"/>
+      <c r="CF108" s="24" t="n"/>
+      <c r="CG108" s="24" t="n"/>
+      <c r="CH108" s="24" t="n"/>
+      <c r="CI108" s="24" t="n"/>
+      <c r="CJ108" s="24" t="n"/>
+      <c r="CK108" s="24" t="n"/>
+      <c r="CL108" s="24" t="n"/>
+      <c r="CM108" s="24" t="n"/>
+      <c r="CN108" s="24" t="n"/>
+      <c r="CO108" s="24" t="n"/>
+      <c r="CP108" s="24" t="n"/>
+      <c r="CQ108" s="24" t="n"/>
+      <c r="CR108" s="24" t="n"/>
+      <c r="CS108" s="24" t="n"/>
+      <c r="CT108" s="24" t="n"/>
+      <c r="CU108" s="24" t="n"/>
+      <c r="CV108" s="24" t="n"/>
+      <c r="CW108" s="24" t="n"/>
+      <c r="CX108" s="24" t="n"/>
+      <c r="CY108" s="24" t="n"/>
+      <c r="CZ108" s="24" t="n"/>
+      <c r="DA108" s="24" t="n"/>
+      <c r="DB108" s="24" t="n"/>
+      <c r="DC108" s="24" t="n"/>
+      <c r="DD108" s="24" t="n"/>
+      <c r="DE108" s="24" t="n"/>
+      <c r="DF108" s="24" t="n"/>
+      <c r="DG108" s="24" t="n"/>
+      <c r="DH108" s="24" t="n"/>
+      <c r="DI108" s="24" t="n"/>
+      <c r="DJ108" s="24" t="n"/>
+      <c r="DK108" s="24" t="n"/>
+      <c r="DL108" s="24" t="n"/>
+      <c r="DM108" s="24" t="n"/>
+      <c r="DN108" s="24" t="n"/>
+      <c r="DO108" s="24" t="n"/>
+      <c r="DP108" s="24" t="n"/>
+    </row>
+    <row r="109" ht="36" customHeight="1">
+      <c r="A109" s="24" t="inlineStr">
+        <is>
+          <t>499f668b627b4948</t>
+        </is>
+      </c>
+      <c r="B109" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C109" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="D109" s="24" t="inlineStr">
+        <is>
+          <t>aec-lol-doc-bce-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E109" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F109" s="24" t="inlineStr">
+        <is>
+          <t>Barcząca Esports</t>
+        </is>
+      </c>
+      <c r="G109" s="24" t="inlineStr">
+        <is>
+          <t>DOCISK</t>
+        </is>
+      </c>
+      <c r="H109" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I109" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J109" s="25" t="n"/>
+      <c r="K109" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L109" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="M109" s="27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N109" s="28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O109" s="28" t="n">
+        <v>0.5107</v>
+      </c>
+      <c r="P109" s="28" t="n"/>
+      <c r="Q109" s="28" t="n">
+        <v>0.1107</v>
+      </c>
+      <c r="R109" s="26" t="n"/>
+      <c r="S109" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T109" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U109" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V109" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W109" s="26" t="n"/>
+      <c r="X109" s="26" t="n"/>
+      <c r="Y109" s="25" t="n"/>
+      <c r="Z109" s="26" t="n"/>
+      <c r="AA109" s="28" t="n"/>
+      <c r="AB109" s="28" t="n"/>
+      <c r="AC109" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD109" s="24" t="n"/>
+      <c r="AE109" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SA9KZAEMVF on aec-lol-doc-bce-2026-09-03 (short)</t>
+        </is>
+      </c>
+      <c r="AF109" s="31" t="n"/>
+      <c r="AG109" s="24" t="n"/>
+      <c r="AH109" s="24" t="n"/>
+      <c r="AI109" s="31" t="n"/>
+      <c r="AJ109" s="31" t="n"/>
+      <c r="AK109" s="24" t="n"/>
+      <c r="AL109" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM109" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN109" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO109" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP109" s="24" t="n"/>
+      <c r="AQ109" s="24" t="n"/>
+      <c r="AR109" s="24" t="n"/>
+      <c r="AS109" s="24" t="n"/>
+      <c r="AT109" s="24" t="n"/>
+      <c r="AU109" s="24" t="n"/>
+      <c r="AV109" s="24" t="n"/>
+      <c r="AW109" s="24" t="n"/>
+      <c r="AX109" s="24" t="n"/>
+      <c r="AY109" s="24" t="n"/>
+      <c r="AZ109" s="24" t="n"/>
+      <c r="BA109" s="24" t="n"/>
+      <c r="BB109" s="24" t="n"/>
+      <c r="BC109" s="24" t="n"/>
+      <c r="BD109" s="24" t="n"/>
+      <c r="BE109" s="24" t="n"/>
+      <c r="BF109" s="24" t="n"/>
+      <c r="BG109" s="24" t="n"/>
+      <c r="BH109" s="24" t="n"/>
+      <c r="BI109" s="24" t="n"/>
+      <c r="BJ109" s="25" t="n"/>
+      <c r="BK109" s="26" t="n"/>
+      <c r="BL109" s="27" t="n"/>
+      <c r="BM109" s="28" t="n"/>
+      <c r="BN109" s="28" t="n"/>
+      <c r="BO109" s="28" t="n"/>
+      <c r="BP109" s="25" t="n"/>
+      <c r="BQ109" s="27" t="n"/>
+      <c r="BR109" s="28" t="n"/>
+      <c r="BS109" s="28" t="n"/>
+      <c r="BT109" s="28" t="n"/>
+      <c r="BU109" s="25" t="n"/>
+      <c r="BV109" s="29" t="n"/>
+      <c r="BW109" s="24" t="n"/>
+      <c r="BX109" s="30" t="n"/>
+      <c r="BY109" s="27" t="n"/>
+      <c r="BZ109" s="24" t="n"/>
+      <c r="CA109" s="31" t="n"/>
+      <c r="CB109" s="24" t="n"/>
+      <c r="CC109" s="24" t="n"/>
+      <c r="CD109" s="24" t="n"/>
+      <c r="CE109" s="24" t="n"/>
+      <c r="CF109" s="24" t="n"/>
+      <c r="CG109" s="24" t="n"/>
+      <c r="CH109" s="24" t="n"/>
+      <c r="CI109" s="24" t="n"/>
+      <c r="CJ109" s="24" t="n"/>
+      <c r="CK109" s="24" t="n"/>
+      <c r="CL109" s="24" t="n"/>
+      <c r="CM109" s="24" t="n"/>
+      <c r="CN109" s="24" t="n"/>
+      <c r="CO109" s="24" t="n"/>
+      <c r="CP109" s="24" t="n"/>
+      <c r="CQ109" s="24" t="n"/>
+      <c r="CR109" s="24" t="n"/>
+      <c r="CS109" s="24" t="n"/>
+      <c r="CT109" s="24" t="n"/>
+      <c r="CU109" s="24" t="n"/>
+      <c r="CV109" s="24" t="n"/>
+      <c r="CW109" s="24" t="n"/>
+      <c r="CX109" s="24" t="n"/>
+      <c r="CY109" s="24" t="n"/>
+      <c r="CZ109" s="24" t="n"/>
+      <c r="DA109" s="24" t="n"/>
+      <c r="DB109" s="24" t="n"/>
+      <c r="DC109" s="24" t="n"/>
+      <c r="DD109" s="24" t="n"/>
+      <c r="DE109" s="24" t="n"/>
+      <c r="DF109" s="24" t="n"/>
+      <c r="DG109" s="24" t="n"/>
+      <c r="DH109" s="24" t="n"/>
+      <c r="DI109" s="24" t="n"/>
+      <c r="DJ109" s="24" t="n"/>
+      <c r="DK109" s="24" t="n"/>
+      <c r="DL109" s="24" t="n"/>
+      <c r="DM109" s="24" t="n"/>
+      <c r="DN109" s="24" t="n"/>
+      <c r="DO109" s="24" t="n"/>
+      <c r="DP109" s="24" t="n"/>
+    </row>
+    <row r="110" ht="36" customHeight="1">
+      <c r="A110" s="24" t="inlineStr">
+        <is>
+          <t>1afb1ec1d9d340e5</t>
+        </is>
+      </c>
+      <c r="B110" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C110" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="D110" s="24" t="inlineStr">
+        <is>
+          <t>aec-lol-pcific-su-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E110" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F110" s="24" t="inlineStr">
+        <is>
+          <t>SU Esports</t>
+        </is>
+      </c>
+      <c r="G110" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCIFIC </t>
+        </is>
+      </c>
+      <c r="H110" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I110" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J110" s="25" t="n"/>
+      <c r="K110" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L110" s="26" t="n">
+        <v>138</v>
+      </c>
+      <c r="M110" s="27" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="N110" s="28" t="n">
+        <v>0.4202</v>
+      </c>
+      <c r="O110" s="28" t="n">
+        <v>0.5492</v>
+      </c>
+      <c r="P110" s="28" t="n"/>
+      <c r="Q110" s="28" t="n">
+        <v>0.1292</v>
+      </c>
+      <c r="R110" s="26" t="n"/>
+      <c r="S110" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T110" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U110" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V110" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W110" s="26" t="n"/>
+      <c r="X110" s="26" t="n"/>
+      <c r="Y110" s="25" t="n"/>
+      <c r="Z110" s="26" t="n"/>
+      <c r="AA110" s="28" t="n"/>
+      <c r="AB110" s="28" t="n"/>
+      <c r="AC110" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD110" s="24" t="n"/>
+      <c r="AE110" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SAKWMYRMVG on aec-lol-pcific-su-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF110" s="31" t="n"/>
+      <c r="AG110" s="24" t="n"/>
+      <c r="AH110" s="24" t="n"/>
+      <c r="AI110" s="31" t="n"/>
+      <c r="AJ110" s="31" t="n"/>
+      <c r="AK110" s="24" t="n"/>
+      <c r="AL110" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM110" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN110" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO110" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP110" s="24" t="n"/>
+      <c r="AQ110" s="24" t="n"/>
+      <c r="AR110" s="24" t="n"/>
+      <c r="AS110" s="24" t="n"/>
+      <c r="AT110" s="24" t="n"/>
+      <c r="AU110" s="24" t="n"/>
+      <c r="AV110" s="24" t="n"/>
+      <c r="AW110" s="24" t="n"/>
+      <c r="AX110" s="24" t="n"/>
+      <c r="AY110" s="24" t="n"/>
+      <c r="AZ110" s="24" t="n"/>
+      <c r="BA110" s="24" t="n"/>
+      <c r="BB110" s="24" t="n"/>
+      <c r="BC110" s="24" t="n"/>
+      <c r="BD110" s="24" t="n"/>
+      <c r="BE110" s="24" t="n"/>
+      <c r="BF110" s="24" t="n"/>
+      <c r="BG110" s="24" t="n"/>
+      <c r="BH110" s="24" t="n"/>
+      <c r="BI110" s="24" t="n"/>
+      <c r="BJ110" s="25" t="n"/>
+      <c r="BK110" s="26" t="n"/>
+      <c r="BL110" s="27" t="n"/>
+      <c r="BM110" s="28" t="n"/>
+      <c r="BN110" s="28" t="n"/>
+      <c r="BO110" s="28" t="n"/>
+      <c r="BP110" s="25" t="n"/>
+      <c r="BQ110" s="27" t="n"/>
+      <c r="BR110" s="28" t="n"/>
+      <c r="BS110" s="28" t="n"/>
+      <c r="BT110" s="28" t="n"/>
+      <c r="BU110" s="25" t="n"/>
+      <c r="BV110" s="29" t="n"/>
+      <c r="BW110" s="24" t="n"/>
+      <c r="BX110" s="30" t="n"/>
+      <c r="BY110" s="27" t="n"/>
+      <c r="BZ110" s="24" t="n"/>
+      <c r="CA110" s="31" t="n"/>
+      <c r="CB110" s="24" t="n"/>
+      <c r="CC110" s="24" t="n"/>
+      <c r="CD110" s="24" t="n"/>
+      <c r="CE110" s="24" t="n"/>
+      <c r="CF110" s="24" t="n"/>
+      <c r="CG110" s="24" t="n"/>
+      <c r="CH110" s="24" t="n"/>
+      <c r="CI110" s="24" t="n"/>
+      <c r="CJ110" s="24" t="n"/>
+      <c r="CK110" s="24" t="n"/>
+      <c r="CL110" s="24" t="n"/>
+      <c r="CM110" s="24" t="n"/>
+      <c r="CN110" s="24" t="n"/>
+      <c r="CO110" s="24" t="n"/>
+      <c r="CP110" s="24" t="n"/>
+      <c r="CQ110" s="24" t="n"/>
+      <c r="CR110" s="24" t="n"/>
+      <c r="CS110" s="24" t="n"/>
+      <c r="CT110" s="24" t="n"/>
+      <c r="CU110" s="24" t="n"/>
+      <c r="CV110" s="24" t="n"/>
+      <c r="CW110" s="24" t="n"/>
+      <c r="CX110" s="24" t="n"/>
+      <c r="CY110" s="24" t="n"/>
+      <c r="CZ110" s="24" t="n"/>
+      <c r="DA110" s="24" t="n"/>
+      <c r="DB110" s="24" t="n"/>
+      <c r="DC110" s="24" t="n"/>
+      <c r="DD110" s="24" t="n"/>
+      <c r="DE110" s="24" t="n"/>
+      <c r="DF110" s="24" t="n"/>
+      <c r="DG110" s="24" t="n"/>
+      <c r="DH110" s="24" t="n"/>
+      <c r="DI110" s="24" t="n"/>
+      <c r="DJ110" s="24" t="n"/>
+      <c r="DK110" s="24" t="n"/>
+      <c r="DL110" s="24" t="n"/>
+      <c r="DM110" s="24" t="n"/>
+      <c r="DN110" s="24" t="n"/>
+      <c r="DO110" s="24" t="n"/>
+      <c r="DP110" s="24" t="n"/>
+    </row>
+    <row r="111" ht="36" customHeight="1">
+      <c r="A111" s="24" t="inlineStr">
+        <is>
+          <t>5ea53b60e25a46ef</t>
+        </is>
+      </c>
+      <c r="B111" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C111" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T16:00:00Z</t>
+        </is>
+      </c>
+      <c r="D111" s="24" t="inlineStr">
+        <is>
+          <t>aec-lol-sec-myth-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E111" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F111" s="24" t="inlineStr">
+        <is>
+          <t>Myth Esports</t>
+        </is>
+      </c>
+      <c r="G111" s="24" t="inlineStr">
+        <is>
+          <t>Senshi Esports</t>
+        </is>
+      </c>
+      <c r="H111" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I111" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J111" s="25" t="n"/>
+      <c r="K111" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L111" s="26" t="n">
+        <v>108</v>
+      </c>
+      <c r="M111" s="27" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="N111" s="28" t="n">
+        <v>0.4808</v>
+      </c>
+      <c r="O111" s="28" t="n">
+        <v>0.5535</v>
+      </c>
+      <c r="P111" s="28" t="n"/>
+      <c r="Q111" s="28" t="n">
+        <v>0.0735</v>
+      </c>
+      <c r="R111" s="26" t="n"/>
+      <c r="S111" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T111" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U111" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V111" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W111" s="26" t="n"/>
+      <c r="X111" s="26" t="n"/>
+      <c r="Y111" s="25" t="n"/>
+      <c r="Z111" s="26" t="n"/>
+      <c r="AA111" s="28" t="n"/>
+      <c r="AB111" s="28" t="n"/>
+      <c r="AC111" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD111" s="24" t="n"/>
+      <c r="AE111" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SADETDWMVK on aec-lol-sec-myth-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF111" s="31" t="n"/>
+      <c r="AG111" s="24" t="n"/>
+      <c r="AH111" s="24" t="n"/>
+      <c r="AI111" s="31" t="n"/>
+      <c r="AJ111" s="31" t="n"/>
+      <c r="AK111" s="24" t="n"/>
+      <c r="AL111" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM111" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN111" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO111" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP111" s="24" t="n"/>
+      <c r="AQ111" s="24" t="n"/>
+      <c r="AR111" s="24" t="n"/>
+      <c r="AS111" s="24" t="n"/>
+      <c r="AT111" s="24" t="n"/>
+      <c r="AU111" s="24" t="n"/>
+      <c r="AV111" s="24" t="n"/>
+      <c r="AW111" s="24" t="n"/>
+      <c r="AX111" s="24" t="n"/>
+      <c r="AY111" s="24" t="n"/>
+      <c r="AZ111" s="24" t="n"/>
+      <c r="BA111" s="24" t="n"/>
+      <c r="BB111" s="24" t="n"/>
+      <c r="BC111" s="24" t="n"/>
+      <c r="BD111" s="24" t="n"/>
+      <c r="BE111" s="24" t="n"/>
+      <c r="BF111" s="24" t="n"/>
+      <c r="BG111" s="24" t="n"/>
+      <c r="BH111" s="24" t="n"/>
+      <c r="BI111" s="24" t="n"/>
+      <c r="BJ111" s="25" t="n"/>
+      <c r="BK111" s="26" t="n"/>
+      <c r="BL111" s="27" t="n"/>
+      <c r="BM111" s="28" t="n"/>
+      <c r="BN111" s="28" t="n"/>
+      <c r="BO111" s="28" t="n"/>
+      <c r="BP111" s="25" t="n"/>
+      <c r="BQ111" s="27" t="n"/>
+      <c r="BR111" s="28" t="n"/>
+      <c r="BS111" s="28" t="n"/>
+      <c r="BT111" s="28" t="n"/>
+      <c r="BU111" s="25" t="n"/>
+      <c r="BV111" s="29" t="n"/>
+      <c r="BW111" s="24" t="n"/>
+      <c r="BX111" s="30" t="n"/>
+      <c r="BY111" s="27" t="n"/>
+      <c r="BZ111" s="24" t="n"/>
+      <c r="CA111" s="31" t="n"/>
+      <c r="CB111" s="24" t="n"/>
+      <c r="CC111" s="24" t="n"/>
+      <c r="CD111" s="24" t="n"/>
+      <c r="CE111" s="24" t="n"/>
+      <c r="CF111" s="24" t="n"/>
+      <c r="CG111" s="24" t="n"/>
+      <c r="CH111" s="24" t="n"/>
+      <c r="CI111" s="24" t="n"/>
+      <c r="CJ111" s="24" t="n"/>
+      <c r="CK111" s="24" t="n"/>
+      <c r="CL111" s="24" t="n"/>
+      <c r="CM111" s="24" t="n"/>
+      <c r="CN111" s="24" t="n"/>
+      <c r="CO111" s="24" t="n"/>
+      <c r="CP111" s="24" t="n"/>
+      <c r="CQ111" s="24" t="n"/>
+      <c r="CR111" s="24" t="n"/>
+      <c r="CS111" s="24" t="n"/>
+      <c r="CT111" s="24" t="n"/>
+      <c r="CU111" s="24" t="n"/>
+      <c r="CV111" s="24" t="n"/>
+      <c r="CW111" s="24" t="n"/>
+      <c r="CX111" s="24" t="n"/>
+      <c r="CY111" s="24" t="n"/>
+      <c r="CZ111" s="24" t="n"/>
+      <c r="DA111" s="24" t="n"/>
+      <c r="DB111" s="24" t="n"/>
+      <c r="DC111" s="24" t="n"/>
+      <c r="DD111" s="24" t="n"/>
+      <c r="DE111" s="24" t="n"/>
+      <c r="DF111" s="24" t="n"/>
+      <c r="DG111" s="24" t="n"/>
+      <c r="DH111" s="24" t="n"/>
+      <c r="DI111" s="24" t="n"/>
+      <c r="DJ111" s="24" t="n"/>
+      <c r="DK111" s="24" t="n"/>
+      <c r="DL111" s="24" t="n"/>
+      <c r="DM111" s="24" t="n"/>
+      <c r="DN111" s="24" t="n"/>
+      <c r="DO111" s="24" t="n"/>
+      <c r="DP111" s="24" t="n"/>
+    </row>
+    <row r="112" ht="36" customHeight="1">
+      <c r="A112" s="24" t="inlineStr">
+        <is>
+          <t>b8c313dca7364d0e</t>
+        </is>
+      </c>
+      <c r="B112" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C112" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T17:30:00Z</t>
+        </is>
+      </c>
+      <c r="D112" s="24" t="inlineStr">
+        <is>
+          <t>aec-lol-lds-dv1-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E112" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F112" s="24" t="inlineStr">
+        <is>
+          <t>devils.one inStreamly</t>
+        </is>
+      </c>
+      <c r="G112" s="24" t="inlineStr">
+        <is>
+          <t>Lodis</t>
+        </is>
+      </c>
+      <c r="H112" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I112" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J112" s="25" t="n"/>
+      <c r="K112" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L112" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="M112" s="27" t="n">
+        <v>1.9615</v>
+      </c>
+      <c r="N112" s="28" t="n">
+        <v>0.5098</v>
+      </c>
+      <c r="O112" s="28" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="P112" s="28" t="n"/>
+      <c r="Q112" s="28" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="R112" s="26" t="n"/>
+      <c r="S112" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T112" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U112" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V112" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W112" s="26" t="n"/>
+      <c r="X112" s="26" t="n"/>
+      <c r="Y112" s="25" t="n"/>
+      <c r="Z112" s="26" t="n"/>
+      <c r="AA112" s="28" t="n"/>
+      <c r="AB112" s="28" t="n"/>
+      <c r="AC112" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD112" s="24" t="n"/>
+      <c r="AE112" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SAMAA24MVP on aec-lol-lds-dv1-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF112" s="31" t="n"/>
+      <c r="AG112" s="24" t="n"/>
+      <c r="AH112" s="24" t="n"/>
+      <c r="AI112" s="31" t="n"/>
+      <c r="AJ112" s="31" t="n"/>
+      <c r="AK112" s="24" t="n"/>
+      <c r="AL112" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM112" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN112" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO112" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP112" s="24" t="n"/>
+      <c r="AQ112" s="24" t="n"/>
+      <c r="AR112" s="24" t="n"/>
+      <c r="AS112" s="24" t="n"/>
+      <c r="AT112" s="24" t="n"/>
+      <c r="AU112" s="24" t="n"/>
+      <c r="AV112" s="24" t="n"/>
+      <c r="AW112" s="24" t="n"/>
+      <c r="AX112" s="24" t="n"/>
+      <c r="AY112" s="24" t="n"/>
+      <c r="AZ112" s="24" t="n"/>
+      <c r="BA112" s="24" t="n"/>
+      <c r="BB112" s="24" t="n"/>
+      <c r="BC112" s="24" t="n"/>
+      <c r="BD112" s="24" t="n"/>
+      <c r="BE112" s="24" t="n"/>
+      <c r="BF112" s="24" t="n"/>
+      <c r="BG112" s="24" t="n"/>
+      <c r="BH112" s="24" t="n"/>
+      <c r="BI112" s="24" t="n"/>
+      <c r="BJ112" s="25" t="n"/>
+      <c r="BK112" s="26" t="n"/>
+      <c r="BL112" s="27" t="n"/>
+      <c r="BM112" s="28" t="n"/>
+      <c r="BN112" s="28" t="n"/>
+      <c r="BO112" s="28" t="n"/>
+      <c r="BP112" s="25" t="n"/>
+      <c r="BQ112" s="27" t="n"/>
+      <c r="BR112" s="28" t="n"/>
+      <c r="BS112" s="28" t="n"/>
+      <c r="BT112" s="28" t="n"/>
+      <c r="BU112" s="25" t="n"/>
+      <c r="BV112" s="29" t="n"/>
+      <c r="BW112" s="24" t="n"/>
+      <c r="BX112" s="30" t="n"/>
+      <c r="BY112" s="27" t="n"/>
+      <c r="BZ112" s="24" t="n"/>
+      <c r="CA112" s="31" t="n"/>
+      <c r="CB112" s="24" t="n"/>
+      <c r="CC112" s="24" t="n"/>
+      <c r="CD112" s="24" t="n"/>
+      <c r="CE112" s="24" t="n"/>
+      <c r="CF112" s="24" t="n"/>
+      <c r="CG112" s="24" t="n"/>
+      <c r="CH112" s="24" t="n"/>
+      <c r="CI112" s="24" t="n"/>
+      <c r="CJ112" s="24" t="n"/>
+      <c r="CK112" s="24" t="n"/>
+      <c r="CL112" s="24" t="n"/>
+      <c r="CM112" s="24" t="n"/>
+      <c r="CN112" s="24" t="n"/>
+      <c r="CO112" s="24" t="n"/>
+      <c r="CP112" s="24" t="n"/>
+      <c r="CQ112" s="24" t="n"/>
+      <c r="CR112" s="24" t="n"/>
+      <c r="CS112" s="24" t="n"/>
+      <c r="CT112" s="24" t="n"/>
+      <c r="CU112" s="24" t="n"/>
+      <c r="CV112" s="24" t="n"/>
+      <c r="CW112" s="24" t="n"/>
+      <c r="CX112" s="24" t="n"/>
+      <c r="CY112" s="24" t="n"/>
+      <c r="CZ112" s="24" t="n"/>
+      <c r="DA112" s="24" t="n"/>
+      <c r="DB112" s="24" t="n"/>
+      <c r="DC112" s="24" t="n"/>
+      <c r="DD112" s="24" t="n"/>
+      <c r="DE112" s="24" t="n"/>
+      <c r="DF112" s="24" t="n"/>
+      <c r="DG112" s="24" t="n"/>
+      <c r="DH112" s="24" t="n"/>
+      <c r="DI112" s="24" t="n"/>
+      <c r="DJ112" s="24" t="n"/>
+      <c r="DK112" s="24" t="n"/>
+      <c r="DL112" s="24" t="n"/>
+      <c r="DM112" s="24" t="n"/>
+      <c r="DN112" s="24" t="n"/>
+      <c r="DO112" s="24" t="n"/>
+      <c r="DP112" s="24" t="n"/>
+    </row>
+    <row r="113" ht="36" customHeight="1">
+      <c r="A113" s="24" t="inlineStr">
+        <is>
+          <t>b7e3c094952e47cb</t>
+        </is>
+      </c>
+      <c r="B113" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C113" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="D113" s="24" t="inlineStr">
+        <is>
+          <t>aec-lol-domi-drm-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E113" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F113" s="24" t="inlineStr">
+        <is>
+          <t>Dream Esports</t>
+        </is>
+      </c>
+      <c r="G113" s="24" t="inlineStr">
+        <is>
+          <t>Dominion Goblins</t>
+        </is>
+      </c>
+      <c r="H113" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I113" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J113" s="25" t="n"/>
+      <c r="K113" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L113" s="26" t="n">
+        <v>144</v>
+      </c>
+      <c r="M113" s="27" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="N113" s="28" t="n">
+        <v>0.4098</v>
+      </c>
+      <c r="O113" s="28" t="n">
+        <v>0.5159</v>
+      </c>
+      <c r="P113" s="28" t="n"/>
+      <c r="Q113" s="28" t="n">
+        <v>0.1059</v>
+      </c>
+      <c r="R113" s="26" t="n"/>
+      <c r="S113" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T113" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U113" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V113" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W113" s="26" t="n"/>
+      <c r="X113" s="26" t="n"/>
+      <c r="Y113" s="25" t="n"/>
+      <c r="Z113" s="26" t="n"/>
+      <c r="AA113" s="28" t="n"/>
+      <c r="AB113" s="28" t="n"/>
+      <c r="AC113" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD113" s="24" t="n"/>
+      <c r="AE113" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SAC9AMPMW0 on aec-lol-domi-drm-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF113" s="31" t="n"/>
+      <c r="AG113" s="24" t="n"/>
+      <c r="AH113" s="24" t="n"/>
+      <c r="AI113" s="31" t="n"/>
+      <c r="AJ113" s="31" t="n"/>
+      <c r="AK113" s="24" t="n"/>
+      <c r="AL113" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM113" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN113" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO113" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP113" s="24" t="n"/>
+      <c r="AQ113" s="24" t="n"/>
+      <c r="AR113" s="24" t="n"/>
+      <c r="AS113" s="24" t="n"/>
+      <c r="AT113" s="24" t="n"/>
+      <c r="AU113" s="24" t="n"/>
+      <c r="AV113" s="24" t="n"/>
+      <c r="AW113" s="24" t="n"/>
+      <c r="AX113" s="24" t="n"/>
+      <c r="AY113" s="24" t="n"/>
+      <c r="AZ113" s="24" t="n"/>
+      <c r="BA113" s="24" t="n"/>
+      <c r="BB113" s="24" t="n"/>
+      <c r="BC113" s="24" t="n"/>
+      <c r="BD113" s="24" t="n"/>
+      <c r="BE113" s="24" t="n"/>
+      <c r="BF113" s="24" t="n"/>
+      <c r="BG113" s="24" t="n"/>
+      <c r="BH113" s="24" t="n"/>
+      <c r="BI113" s="24" t="n"/>
+      <c r="BJ113" s="25" t="n"/>
+      <c r="BK113" s="26" t="n"/>
+      <c r="BL113" s="27" t="n"/>
+      <c r="BM113" s="28" t="n"/>
+      <c r="BN113" s="28" t="n"/>
+      <c r="BO113" s="28" t="n"/>
+      <c r="BP113" s="25" t="n"/>
+      <c r="BQ113" s="27" t="n"/>
+      <c r="BR113" s="28" t="n"/>
+      <c r="BS113" s="28" t="n"/>
+      <c r="BT113" s="28" t="n"/>
+      <c r="BU113" s="25" t="n"/>
+      <c r="BV113" s="29" t="n"/>
+      <c r="BW113" s="24" t="n"/>
+      <c r="BX113" s="30" t="n"/>
+      <c r="BY113" s="27" t="n"/>
+      <c r="BZ113" s="24" t="n"/>
+      <c r="CA113" s="31" t="n"/>
+      <c r="CB113" s="24" t="n"/>
+      <c r="CC113" s="24" t="n"/>
+      <c r="CD113" s="24" t="n"/>
+      <c r="CE113" s="24" t="n"/>
+      <c r="CF113" s="24" t="n"/>
+      <c r="CG113" s="24" t="n"/>
+      <c r="CH113" s="24" t="n"/>
+      <c r="CI113" s="24" t="n"/>
+      <c r="CJ113" s="24" t="n"/>
+      <c r="CK113" s="24" t="n"/>
+      <c r="CL113" s="24" t="n"/>
+      <c r="CM113" s="24" t="n"/>
+      <c r="CN113" s="24" t="n"/>
+      <c r="CO113" s="24" t="n"/>
+      <c r="CP113" s="24" t="n"/>
+      <c r="CQ113" s="24" t="n"/>
+      <c r="CR113" s="24" t="n"/>
+      <c r="CS113" s="24" t="n"/>
+      <c r="CT113" s="24" t="n"/>
+      <c r="CU113" s="24" t="n"/>
+      <c r="CV113" s="24" t="n"/>
+      <c r="CW113" s="24" t="n"/>
+      <c r="CX113" s="24" t="n"/>
+      <c r="CY113" s="24" t="n"/>
+      <c r="CZ113" s="24" t="n"/>
+      <c r="DA113" s="24" t="n"/>
+      <c r="DB113" s="24" t="n"/>
+      <c r="DC113" s="24" t="n"/>
+      <c r="DD113" s="24" t="n"/>
+      <c r="DE113" s="24" t="n"/>
+      <c r="DF113" s="24" t="n"/>
+      <c r="DG113" s="24" t="n"/>
+      <c r="DH113" s="24" t="n"/>
+      <c r="DI113" s="24" t="n"/>
+      <c r="DJ113" s="24" t="n"/>
+      <c r="DK113" s="24" t="n"/>
+      <c r="DL113" s="24" t="n"/>
+      <c r="DM113" s="24" t="n"/>
+      <c r="DN113" s="24" t="n"/>
+      <c r="DO113" s="24" t="n"/>
+      <c r="DP113" s="24" t="n"/>
+    </row>
+    <row r="114" ht="36" customHeight="1">
+      <c r="A114" s="24" t="inlineStr">
+        <is>
+          <t>8ae128177f5b440c</t>
+        </is>
+      </c>
+      <c r="B114" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C114" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="D114" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-g2a-pf-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E114" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F114" s="24" t="inlineStr">
+        <is>
+          <t>PsychoFace</t>
+        </is>
+      </c>
+      <c r="G114" s="24" t="inlineStr">
+        <is>
+          <t>G2 Ares</t>
+        </is>
+      </c>
+      <c r="H114" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I114" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J114" s="25" t="n"/>
+      <c r="K114" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L114" s="26" t="n">
+        <v>-108</v>
+      </c>
+      <c r="M114" s="27" t="n">
+        <v>1.9259</v>
+      </c>
+      <c r="N114" s="28" t="n">
+        <v>0.5192</v>
+      </c>
+      <c r="O114" s="28" t="n">
+        <v>0.6032999999999999</v>
+      </c>
+      <c r="P114" s="28" t="n"/>
+      <c r="Q114" s="28" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="R114" s="26" t="n"/>
+      <c r="S114" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T114" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U114" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V114" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W114" s="26" t="n"/>
+      <c r="X114" s="26" t="n"/>
+      <c r="Y114" s="25" t="n"/>
+      <c r="Z114" s="26" t="n"/>
+      <c r="AA114" s="28" t="n"/>
+      <c r="AB114" s="28" t="n"/>
+      <c r="AC114" s="30" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="AD114" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:41:14.239238Z</t>
+        </is>
+      </c>
+      <c r="AE114" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8S9RQ7WYMVZ on aec-cs2-g2a-pf-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF114" s="31" t="n"/>
+      <c r="AG114" s="24" t="n"/>
+      <c r="AH114" s="24" t="n"/>
+      <c r="AI114" s="31" t="n"/>
+      <c r="AJ114" s="31" t="n"/>
+      <c r="AK114" s="24" t="n"/>
+      <c r="AL114" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM114" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN114" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO114" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP114" s="24" t="n"/>
+      <c r="AQ114" s="24" t="n"/>
+      <c r="AR114" s="24" t="n"/>
+      <c r="AS114" s="24" t="n"/>
+      <c r="AT114" s="24" t="n"/>
+      <c r="AU114" s="24" t="n"/>
+      <c r="AV114" s="24" t="n"/>
+      <c r="AW114" s="24" t="n"/>
+      <c r="AX114" s="24" t="n"/>
+      <c r="AY114" s="24" t="n"/>
+      <c r="AZ114" s="24" t="n"/>
+      <c r="BA114" s="24" t="n"/>
+      <c r="BB114" s="24" t="n"/>
+      <c r="BC114" s="24" t="n"/>
+      <c r="BD114" s="24" t="n"/>
+      <c r="BE114" s="24" t="n"/>
+      <c r="BF114" s="24" t="n"/>
+      <c r="BG114" s="24" t="n"/>
+      <c r="BH114" s="24" t="n"/>
+      <c r="BI114" s="24" t="n"/>
+      <c r="BJ114" s="25" t="n"/>
+      <c r="BK114" s="26" t="n"/>
+      <c r="BL114" s="27" t="n"/>
+      <c r="BM114" s="28" t="n"/>
+      <c r="BN114" s="28" t="n"/>
+      <c r="BO114" s="28" t="n"/>
+      <c r="BP114" s="25" t="n"/>
+      <c r="BQ114" s="27" t="n"/>
+      <c r="BR114" s="28" t="n"/>
+      <c r="BS114" s="28" t="n"/>
+      <c r="BT114" s="28" t="n"/>
+      <c r="BU114" s="25" t="n"/>
+      <c r="BV114" s="29" t="n"/>
+      <c r="BW114" s="24" t="n"/>
+      <c r="BX114" s="30" t="n"/>
+      <c r="BY114" s="27" t="n"/>
+      <c r="BZ114" s="24" t="n"/>
+      <c r="CA114" s="31" t="n"/>
+      <c r="CB114" s="24" t="n"/>
+      <c r="CC114" s="24" t="n"/>
+      <c r="CD114" s="24" t="n"/>
+      <c r="CE114" s="24" t="n"/>
+      <c r="CF114" s="24" t="n"/>
+      <c r="CG114" s="24" t="n"/>
+      <c r="CH114" s="24" t="n"/>
+      <c r="CI114" s="24" t="n"/>
+      <c r="CJ114" s="24" t="n"/>
+      <c r="CK114" s="24" t="n"/>
+      <c r="CL114" s="24" t="n"/>
+      <c r="CM114" s="24" t="n"/>
+      <c r="CN114" s="24" t="n"/>
+      <c r="CO114" s="24" t="n"/>
+      <c r="CP114" s="24" t="n"/>
+      <c r="CQ114" s="24" t="n"/>
+      <c r="CR114" s="24" t="n"/>
+      <c r="CS114" s="24" t="n"/>
+      <c r="CT114" s="24" t="n"/>
+      <c r="CU114" s="24" t="n"/>
+      <c r="CV114" s="24" t="n"/>
+      <c r="CW114" s="24" t="n"/>
+      <c r="CX114" s="24" t="n"/>
+      <c r="CY114" s="24" t="n"/>
+      <c r="CZ114" s="24" t="n"/>
+      <c r="DA114" s="24" t="n"/>
+      <c r="DB114" s="24" t="n"/>
+      <c r="DC114" s="24" t="n"/>
+      <c r="DD114" s="24" t="n"/>
+      <c r="DE114" s="24" t="n"/>
+      <c r="DF114" s="24" t="n"/>
+      <c r="DG114" s="24" t="n"/>
+      <c r="DH114" s="24" t="n"/>
+      <c r="DI114" s="24" t="n"/>
+      <c r="DJ114" s="24" t="n"/>
+      <c r="DK114" s="24" t="n"/>
+      <c r="DL114" s="24" t="n"/>
+      <c r="DM114" s="24" t="n"/>
+      <c r="DN114" s="24" t="n"/>
+      <c r="DO114" s="24" t="n"/>
+      <c r="DP114" s="24" t="n"/>
+    </row>
+    <row r="115" ht="36" customHeight="1">
+      <c r="A115" s="24" t="inlineStr">
+        <is>
+          <t>98602be4e1d84939</t>
+        </is>
+      </c>
+      <c r="B115" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C115" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="D115" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-vexar-bge-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E115" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F115" s="24" t="inlineStr">
+        <is>
+          <t>Benched gods</t>
+        </is>
+      </c>
+      <c r="G115" s="24" t="inlineStr">
+        <is>
+          <t>Vexar</t>
+        </is>
+      </c>
+      <c r="H115" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I115" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J115" s="25" t="n"/>
+      <c r="K115" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L115" s="26" t="n">
+        <v>117</v>
+      </c>
+      <c r="M115" s="27" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="N115" s="28" t="n">
+        <v>0.4608</v>
+      </c>
+      <c r="O115" s="28" t="n">
+        <v>0.5564</v>
+      </c>
+      <c r="P115" s="28" t="n"/>
+      <c r="Q115" s="28" t="n">
+        <v>0.0964</v>
+      </c>
+      <c r="R115" s="26" t="n"/>
+      <c r="S115" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T115" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U115" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V115" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W115" s="26" t="n"/>
+      <c r="X115" s="26" t="n"/>
+      <c r="Y115" s="25" t="n"/>
+      <c r="Z115" s="26" t="n"/>
+      <c r="AA115" s="28" t="n"/>
+      <c r="AB115" s="28" t="n"/>
+      <c r="AC115" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD115" s="24" t="n"/>
+      <c r="AE115" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8S9GE15EMVV on aec-cs2-vexar-bge-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF115" s="31" t="n"/>
+      <c r="AG115" s="24" t="n"/>
+      <c r="AH115" s="24" t="n"/>
+      <c r="AI115" s="31" t="n"/>
+      <c r="AJ115" s="31" t="n"/>
+      <c r="AK115" s="24" t="n"/>
+      <c r="AL115" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM115" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN115" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO115" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP115" s="24" t="n"/>
+      <c r="AQ115" s="24" t="n"/>
+      <c r="AR115" s="24" t="n"/>
+      <c r="AS115" s="24" t="n"/>
+      <c r="AT115" s="24" t="n"/>
+      <c r="AU115" s="24" t="n"/>
+      <c r="AV115" s="24" t="n"/>
+      <c r="AW115" s="24" t="n"/>
+      <c r="AX115" s="24" t="n"/>
+      <c r="AY115" s="24" t="n"/>
+      <c r="AZ115" s="24" t="n"/>
+      <c r="BA115" s="24" t="n"/>
+      <c r="BB115" s="24" t="n"/>
+      <c r="BC115" s="24" t="n"/>
+      <c r="BD115" s="24" t="n"/>
+      <c r="BE115" s="24" t="n"/>
+      <c r="BF115" s="24" t="n"/>
+      <c r="BG115" s="24" t="n"/>
+      <c r="BH115" s="24" t="n"/>
+      <c r="BI115" s="24" t="n"/>
+      <c r="BJ115" s="25" t="n"/>
+      <c r="BK115" s="26" t="n"/>
+      <c r="BL115" s="27" t="n"/>
+      <c r="BM115" s="28" t="n"/>
+      <c r="BN115" s="28" t="n"/>
+      <c r="BO115" s="28" t="n"/>
+      <c r="BP115" s="25" t="n"/>
+      <c r="BQ115" s="27" t="n"/>
+      <c r="BR115" s="28" t="n"/>
+      <c r="BS115" s="28" t="n"/>
+      <c r="BT115" s="28" t="n"/>
+      <c r="BU115" s="25" t="n"/>
+      <c r="BV115" s="29" t="n"/>
+      <c r="BW115" s="24" t="n"/>
+      <c r="BX115" s="30" t="n"/>
+      <c r="BY115" s="27" t="n"/>
+      <c r="BZ115" s="24" t="n"/>
+      <c r="CA115" s="31" t="n"/>
+      <c r="CB115" s="24" t="n"/>
+      <c r="CC115" s="24" t="n"/>
+      <c r="CD115" s="24" t="n"/>
+      <c r="CE115" s="24" t="n"/>
+      <c r="CF115" s="24" t="n"/>
+      <c r="CG115" s="24" t="n"/>
+      <c r="CH115" s="24" t="n"/>
+      <c r="CI115" s="24" t="n"/>
+      <c r="CJ115" s="24" t="n"/>
+      <c r="CK115" s="24" t="n"/>
+      <c r="CL115" s="24" t="n"/>
+      <c r="CM115" s="24" t="n"/>
+      <c r="CN115" s="24" t="n"/>
+      <c r="CO115" s="24" t="n"/>
+      <c r="CP115" s="24" t="n"/>
+      <c r="CQ115" s="24" t="n"/>
+      <c r="CR115" s="24" t="n"/>
+      <c r="CS115" s="24" t="n"/>
+      <c r="CT115" s="24" t="n"/>
+      <c r="CU115" s="24" t="n"/>
+      <c r="CV115" s="24" t="n"/>
+      <c r="CW115" s="24" t="n"/>
+      <c r="CX115" s="24" t="n"/>
+      <c r="CY115" s="24" t="n"/>
+      <c r="CZ115" s="24" t="n"/>
+      <c r="DA115" s="24" t="n"/>
+      <c r="DB115" s="24" t="n"/>
+      <c r="DC115" s="24" t="n"/>
+      <c r="DD115" s="24" t="n"/>
+      <c r="DE115" s="24" t="n"/>
+      <c r="DF115" s="24" t="n"/>
+      <c r="DG115" s="24" t="n"/>
+      <c r="DH115" s="24" t="n"/>
+      <c r="DI115" s="24" t="n"/>
+      <c r="DJ115" s="24" t="n"/>
+      <c r="DK115" s="24" t="n"/>
+      <c r="DL115" s="24" t="n"/>
+      <c r="DM115" s="24" t="n"/>
+      <c r="DN115" s="24" t="n"/>
+      <c r="DO115" s="24" t="n"/>
+      <c r="DP115" s="24" t="n"/>
+    </row>
+    <row r="116" ht="36" customHeight="1">
+      <c r="A116" s="24" t="inlineStr">
+        <is>
+          <t>59d5f8dca13249d0</t>
+        </is>
+      </c>
+      <c r="B116" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C116" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T09:00:00Z</t>
+        </is>
+      </c>
+      <c r="D116" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-is-nemi-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E116" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F116" s="24" t="inlineStr">
+        <is>
+          <t>Nemiga</t>
+        </is>
+      </c>
+      <c r="G116" s="24" t="inlineStr">
+        <is>
+          <t>Iberian Soul</t>
+        </is>
+      </c>
+      <c r="H116" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I116" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J116" s="25" t="n"/>
+      <c r="K116" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L116" s="26" t="n">
+        <v>133</v>
+      </c>
+      <c r="M116" s="27" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="N116" s="28" t="n">
+        <v>0.4292</v>
+      </c>
+      <c r="O116" s="28" t="n">
+        <v>0.5028</v>
+      </c>
+      <c r="P116" s="28" t="n"/>
+      <c r="Q116" s="28" t="n">
+        <v>0.0728</v>
+      </c>
+      <c r="R116" s="26" t="n"/>
+      <c r="S116" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T116" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U116" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V116" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W116" s="26" t="n"/>
+      <c r="X116" s="26" t="n"/>
+      <c r="Y116" s="25" t="n"/>
+      <c r="Z116" s="26" t="n"/>
+      <c r="AA116" s="28" t="n"/>
+      <c r="AB116" s="28" t="n"/>
+      <c r="AC116" s="30" t="n">
+        <v>-1.25</v>
+      </c>
+      <c r="AD116" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:41:14.239238Z</t>
+        </is>
+      </c>
+      <c r="AE116" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SAPZXQGMW0 on aec-cs2-is-nemi-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF116" s="31" t="n"/>
+      <c r="AG116" s="24" t="n"/>
+      <c r="AH116" s="24" t="n"/>
+      <c r="AI116" s="31" t="n"/>
+      <c r="AJ116" s="31" t="n"/>
+      <c r="AK116" s="24" t="n"/>
+      <c r="AL116" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM116" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN116" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO116" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP116" s="24" t="n"/>
+      <c r="AQ116" s="24" t="n"/>
+      <c r="AR116" s="24" t="n"/>
+      <c r="AS116" s="24" t="n"/>
+      <c r="AT116" s="24" t="n"/>
+      <c r="AU116" s="24" t="n"/>
+      <c r="AV116" s="24" t="n"/>
+      <c r="AW116" s="24" t="n"/>
+      <c r="AX116" s="24" t="n"/>
+      <c r="AY116" s="24" t="n"/>
+      <c r="AZ116" s="24" t="n"/>
+      <c r="BA116" s="24" t="n"/>
+      <c r="BB116" s="24" t="n"/>
+      <c r="BC116" s="24" t="n"/>
+      <c r="BD116" s="24" t="n"/>
+      <c r="BE116" s="24" t="n"/>
+      <c r="BF116" s="24" t="n"/>
+      <c r="BG116" s="24" t="n"/>
+      <c r="BH116" s="24" t="n"/>
+      <c r="BI116" s="24" t="n"/>
+      <c r="BJ116" s="25" t="n"/>
+      <c r="BK116" s="26" t="n"/>
+      <c r="BL116" s="27" t="n"/>
+      <c r="BM116" s="28" t="n"/>
+      <c r="BN116" s="28" t="n"/>
+      <c r="BO116" s="28" t="n"/>
+      <c r="BP116" s="25" t="n"/>
+      <c r="BQ116" s="27" t="n"/>
+      <c r="BR116" s="28" t="n"/>
+      <c r="BS116" s="28" t="n"/>
+      <c r="BT116" s="28" t="n"/>
+      <c r="BU116" s="25" t="n"/>
+      <c r="BV116" s="29" t="n"/>
+      <c r="BW116" s="24" t="n"/>
+      <c r="BX116" s="30" t="n"/>
+      <c r="BY116" s="27" t="n"/>
+      <c r="BZ116" s="24" t="n"/>
+      <c r="CA116" s="31" t="n"/>
+      <c r="CB116" s="24" t="n"/>
+      <c r="CC116" s="24" t="n"/>
+      <c r="CD116" s="24" t="n"/>
+      <c r="CE116" s="24" t="n"/>
+      <c r="CF116" s="24" t="n"/>
+      <c r="CG116" s="24" t="n"/>
+      <c r="CH116" s="24" t="n"/>
+      <c r="CI116" s="24" t="n"/>
+      <c r="CJ116" s="24" t="n"/>
+      <c r="CK116" s="24" t="n"/>
+      <c r="CL116" s="24" t="n"/>
+      <c r="CM116" s="24" t="n"/>
+      <c r="CN116" s="24" t="n"/>
+      <c r="CO116" s="24" t="n"/>
+      <c r="CP116" s="24" t="n"/>
+      <c r="CQ116" s="24" t="n"/>
+      <c r="CR116" s="24" t="n"/>
+      <c r="CS116" s="24" t="n"/>
+      <c r="CT116" s="24" t="n"/>
+      <c r="CU116" s="24" t="n"/>
+      <c r="CV116" s="24" t="n"/>
+      <c r="CW116" s="24" t="n"/>
+      <c r="CX116" s="24" t="n"/>
+      <c r="CY116" s="24" t="n"/>
+      <c r="CZ116" s="24" t="n"/>
+      <c r="DA116" s="24" t="n"/>
+      <c r="DB116" s="24" t="n"/>
+      <c r="DC116" s="24" t="n"/>
+      <c r="DD116" s="24" t="n"/>
+      <c r="DE116" s="24" t="n"/>
+      <c r="DF116" s="24" t="n"/>
+      <c r="DG116" s="24" t="n"/>
+      <c r="DH116" s="24" t="n"/>
+      <c r="DI116" s="24" t="n"/>
+      <c r="DJ116" s="24" t="n"/>
+      <c r="DK116" s="24" t="n"/>
+      <c r="DL116" s="24" t="n"/>
+      <c r="DM116" s="24" t="n"/>
+      <c r="DN116" s="24" t="n"/>
+      <c r="DO116" s="24" t="n"/>
+      <c r="DP116" s="24" t="n"/>
+    </row>
+    <row r="117" ht="36" customHeight="1">
+      <c r="A117" s="24" t="inlineStr">
+        <is>
+          <t>c3b52dee2e854cfa</t>
+        </is>
+      </c>
+      <c r="B117" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C117" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T10:30:00Z</t>
+        </is>
+      </c>
+      <c r="D117" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-for-biga-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E117" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F117" s="24" t="inlineStr">
+        <is>
+          <t>BIG Academy</t>
+        </is>
+      </c>
+      <c r="G117" s="24" t="inlineStr">
+        <is>
+          <t>Fortress</t>
+        </is>
+      </c>
+      <c r="H117" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I117" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J117" s="25" t="n"/>
+      <c r="K117" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L117" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="M117" s="27" t="n">
+        <v>1.8547</v>
+      </c>
+      <c r="N117" s="28" t="n">
+        <v>0.5392</v>
+      </c>
+      <c r="O117" s="28" t="n">
+        <v>0.8525</v>
+      </c>
+      <c r="P117" s="28" t="n"/>
+      <c r="Q117" s="28" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="R117" s="26" t="n"/>
+      <c r="S117" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T117" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U117" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V117" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W117" s="26" t="n"/>
+      <c r="X117" s="26" t="n"/>
+      <c r="Y117" s="25" t="n"/>
+      <c r="Z117" s="26" t="n"/>
+      <c r="AA117" s="28" t="n"/>
+      <c r="AB117" s="28" t="n"/>
+      <c r="AC117" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD117" s="24" t="n"/>
+      <c r="AE117" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8S9JDN66MW1 on aec-cs2-for-biga-2026-09-03 (short)</t>
+        </is>
+      </c>
+      <c r="AF117" s="31" t="n"/>
+      <c r="AG117" s="24" t="n"/>
+      <c r="AH117" s="24" t="n"/>
+      <c r="AI117" s="31" t="n"/>
+      <c r="AJ117" s="31" t="n"/>
+      <c r="AK117" s="24" t="n"/>
+      <c r="AL117" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM117" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN117" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO117" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP117" s="24" t="n"/>
+      <c r="AQ117" s="24" t="n"/>
+      <c r="AR117" s="24" t="n"/>
+      <c r="AS117" s="24" t="n"/>
+      <c r="AT117" s="24" t="n"/>
+      <c r="AU117" s="24" t="n"/>
+      <c r="AV117" s="24" t="n"/>
+      <c r="AW117" s="24" t="n"/>
+      <c r="AX117" s="24" t="n"/>
+      <c r="AY117" s="24" t="n"/>
+      <c r="AZ117" s="24" t="n"/>
+      <c r="BA117" s="24" t="n"/>
+      <c r="BB117" s="24" t="n"/>
+      <c r="BC117" s="24" t="n"/>
+      <c r="BD117" s="24" t="n"/>
+      <c r="BE117" s="24" t="n"/>
+      <c r="BF117" s="24" t="n"/>
+      <c r="BG117" s="24" t="n"/>
+      <c r="BH117" s="24" t="n"/>
+      <c r="BI117" s="24" t="n"/>
+      <c r="BJ117" s="25" t="n"/>
+      <c r="BK117" s="26" t="n"/>
+      <c r="BL117" s="27" t="n"/>
+      <c r="BM117" s="28" t="n"/>
+      <c r="BN117" s="28" t="n"/>
+      <c r="BO117" s="28" t="n"/>
+      <c r="BP117" s="25" t="n"/>
+      <c r="BQ117" s="27" t="n"/>
+      <c r="BR117" s="28" t="n"/>
+      <c r="BS117" s="28" t="n"/>
+      <c r="BT117" s="28" t="n"/>
+      <c r="BU117" s="25" t="n"/>
+      <c r="BV117" s="29" t="n"/>
+      <c r="BW117" s="24" t="n"/>
+      <c r="BX117" s="30" t="n"/>
+      <c r="BY117" s="27" t="n"/>
+      <c r="BZ117" s="24" t="n"/>
+      <c r="CA117" s="31" t="n"/>
+      <c r="CB117" s="24" t="n"/>
+      <c r="CC117" s="24" t="n"/>
+      <c r="CD117" s="24" t="n"/>
+      <c r="CE117" s="24" t="n"/>
+      <c r="CF117" s="24" t="n"/>
+      <c r="CG117" s="24" t="n"/>
+      <c r="CH117" s="24" t="n"/>
+      <c r="CI117" s="24" t="n"/>
+      <c r="CJ117" s="24" t="n"/>
+      <c r="CK117" s="24" t="n"/>
+      <c r="CL117" s="24" t="n"/>
+      <c r="CM117" s="24" t="n"/>
+      <c r="CN117" s="24" t="n"/>
+      <c r="CO117" s="24" t="n"/>
+      <c r="CP117" s="24" t="n"/>
+      <c r="CQ117" s="24" t="n"/>
+      <c r="CR117" s="24" t="n"/>
+      <c r="CS117" s="24" t="n"/>
+      <c r="CT117" s="24" t="n"/>
+      <c r="CU117" s="24" t="n"/>
+      <c r="CV117" s="24" t="n"/>
+      <c r="CW117" s="24" t="n"/>
+      <c r="CX117" s="24" t="n"/>
+      <c r="CY117" s="24" t="n"/>
+      <c r="CZ117" s="24" t="n"/>
+      <c r="DA117" s="24" t="n"/>
+      <c r="DB117" s="24" t="n"/>
+      <c r="DC117" s="24" t="n"/>
+      <c r="DD117" s="24" t="n"/>
+      <c r="DE117" s="24" t="n"/>
+      <c r="DF117" s="24" t="n"/>
+      <c r="DG117" s="24" t="n"/>
+      <c r="DH117" s="24" t="n"/>
+      <c r="DI117" s="24" t="n"/>
+      <c r="DJ117" s="24" t="n"/>
+      <c r="DK117" s="24" t="n"/>
+      <c r="DL117" s="24" t="n"/>
+      <c r="DM117" s="24" t="n"/>
+      <c r="DN117" s="24" t="n"/>
+      <c r="DO117" s="24" t="n"/>
+      <c r="DP117" s="24" t="n"/>
+    </row>
+    <row r="118" ht="36" customHeight="1">
+      <c r="A118" s="24" t="inlineStr">
+        <is>
+          <t>fe6312d3e15e40dd</t>
+        </is>
+      </c>
+      <c r="B118" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C118" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T11:00:00Z</t>
+        </is>
+      </c>
+      <c r="D118" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-leo-tlr-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E118" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F118" s="24" t="inlineStr">
+        <is>
+          <t>The Last Resort</t>
+        </is>
+      </c>
+      <c r="G118" s="24" t="inlineStr">
+        <is>
+          <t>Leo Team</t>
+        </is>
+      </c>
+      <c r="H118" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I118" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J118" s="25" t="n"/>
+      <c r="K118" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L118" s="26" t="n">
+        <v>178</v>
+      </c>
+      <c r="M118" s="27" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="N118" s="28" t="n">
+        <v>0.3597</v>
+      </c>
+      <c r="O118" s="28" t="n">
+        <v>0.5026</v>
+      </c>
+      <c r="P118" s="28" t="n"/>
+      <c r="Q118" s="28" t="n">
+        <v>0.1426</v>
+      </c>
+      <c r="R118" s="26" t="n"/>
+      <c r="S118" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T118" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U118" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V118" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W118" s="26" t="n"/>
+      <c r="X118" s="26" t="n"/>
+      <c r="Y118" s="25" t="n"/>
+      <c r="Z118" s="26" t="n"/>
+      <c r="AA118" s="28" t="n"/>
+      <c r="AB118" s="28" t="n"/>
+      <c r="AC118" s="30" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="AD118" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:41:14.239238Z</t>
+        </is>
+      </c>
+      <c r="AE118" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SAJ759CMVR on aec-cs2-leo-tlr-2026-09-03 (short)</t>
+        </is>
+      </c>
+      <c r="AF118" s="31" t="n"/>
+      <c r="AG118" s="24" t="n"/>
+      <c r="AH118" s="24" t="n"/>
+      <c r="AI118" s="31" t="n"/>
+      <c r="AJ118" s="31" t="n"/>
+      <c r="AK118" s="24" t="n"/>
+      <c r="AL118" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM118" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN118" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO118" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP118" s="24" t="n"/>
+      <c r="AQ118" s="24" t="n"/>
+      <c r="AR118" s="24" t="n"/>
+      <c r="AS118" s="24" t="n"/>
+      <c r="AT118" s="24" t="n"/>
+      <c r="AU118" s="24" t="n"/>
+      <c r="AV118" s="24" t="n"/>
+      <c r="AW118" s="24" t="n"/>
+      <c r="AX118" s="24" t="n"/>
+      <c r="AY118" s="24" t="n"/>
+      <c r="AZ118" s="24" t="n"/>
+      <c r="BA118" s="24" t="n"/>
+      <c r="BB118" s="24" t="n"/>
+      <c r="BC118" s="24" t="n"/>
+      <c r="BD118" s="24" t="n"/>
+      <c r="BE118" s="24" t="n"/>
+      <c r="BF118" s="24" t="n"/>
+      <c r="BG118" s="24" t="n"/>
+      <c r="BH118" s="24" t="n"/>
+      <c r="BI118" s="24" t="n"/>
+      <c r="BJ118" s="25" t="n"/>
+      <c r="BK118" s="26" t="n"/>
+      <c r="BL118" s="27" t="n"/>
+      <c r="BM118" s="28" t="n"/>
+      <c r="BN118" s="28" t="n"/>
+      <c r="BO118" s="28" t="n"/>
+      <c r="BP118" s="25" t="n"/>
+      <c r="BQ118" s="27" t="n"/>
+      <c r="BR118" s="28" t="n"/>
+      <c r="BS118" s="28" t="n"/>
+      <c r="BT118" s="28" t="n"/>
+      <c r="BU118" s="25" t="n"/>
+      <c r="BV118" s="29" t="n"/>
+      <c r="BW118" s="24" t="n"/>
+      <c r="BX118" s="30" t="n"/>
+      <c r="BY118" s="27" t="n"/>
+      <c r="BZ118" s="24" t="n"/>
+      <c r="CA118" s="31" t="n"/>
+      <c r="CB118" s="24" t="n"/>
+      <c r="CC118" s="24" t="n"/>
+      <c r="CD118" s="24" t="n"/>
+      <c r="CE118" s="24" t="n"/>
+      <c r="CF118" s="24" t="n"/>
+      <c r="CG118" s="24" t="n"/>
+      <c r="CH118" s="24" t="n"/>
+      <c r="CI118" s="24" t="n"/>
+      <c r="CJ118" s="24" t="n"/>
+      <c r="CK118" s="24" t="n"/>
+      <c r="CL118" s="24" t="n"/>
+      <c r="CM118" s="24" t="n"/>
+      <c r="CN118" s="24" t="n"/>
+      <c r="CO118" s="24" t="n"/>
+      <c r="CP118" s="24" t="n"/>
+      <c r="CQ118" s="24" t="n"/>
+      <c r="CR118" s="24" t="n"/>
+      <c r="CS118" s="24" t="n"/>
+      <c r="CT118" s="24" t="n"/>
+      <c r="CU118" s="24" t="n"/>
+      <c r="CV118" s="24" t="n"/>
+      <c r="CW118" s="24" t="n"/>
+      <c r="CX118" s="24" t="n"/>
+      <c r="CY118" s="24" t="n"/>
+      <c r="CZ118" s="24" t="n"/>
+      <c r="DA118" s="24" t="n"/>
+      <c r="DB118" s="24" t="n"/>
+      <c r="DC118" s="24" t="n"/>
+      <c r="DD118" s="24" t="n"/>
+      <c r="DE118" s="24" t="n"/>
+      <c r="DF118" s="24" t="n"/>
+      <c r="DG118" s="24" t="n"/>
+      <c r="DH118" s="24" t="n"/>
+      <c r="DI118" s="24" t="n"/>
+      <c r="DJ118" s="24" t="n"/>
+      <c r="DK118" s="24" t="n"/>
+      <c r="DL118" s="24" t="n"/>
+      <c r="DM118" s="24" t="n"/>
+      <c r="DN118" s="24" t="n"/>
+      <c r="DO118" s="24" t="n"/>
+      <c r="DP118" s="24" t="n"/>
+    </row>
+    <row r="119" ht="36" customHeight="1">
+      <c r="A119" s="24" t="inlineStr">
+        <is>
+          <t>b0078c89886b41a1</t>
+        </is>
+      </c>
+      <c r="B119" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C119" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T11:00:00Z</t>
+        </is>
+      </c>
+      <c r="D119" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-hotu-nem-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E119" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F119" s="24" t="inlineStr">
+        <is>
+          <t>Team Nemesis</t>
+        </is>
+      </c>
+      <c r="G119" s="24" t="inlineStr">
+        <is>
+          <t>HOTU</t>
+        </is>
+      </c>
+      <c r="H119" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I119" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J119" s="25" t="n"/>
+      <c r="K119" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L119" s="26" t="n">
+        <v>113</v>
+      </c>
+      <c r="M119" s="27" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="N119" s="28" t="n">
+        <v>0.4695</v>
+      </c>
+      <c r="O119" s="28" t="n">
+        <v>0.5232</v>
+      </c>
+      <c r="P119" s="28" t="n"/>
+      <c r="Q119" s="28" t="n">
+        <v>0.0532</v>
+      </c>
+      <c r="R119" s="26" t="n"/>
+      <c r="S119" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T119" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U119" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V119" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W119" s="26" t="n"/>
+      <c r="X119" s="26" t="n"/>
+      <c r="Y119" s="25" t="n"/>
+      <c r="Z119" s="26" t="n"/>
+      <c r="AA119" s="28" t="n"/>
+      <c r="AB119" s="28" t="n"/>
+      <c r="AC119" s="30" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AD119" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:41:14.239238Z</t>
+        </is>
+      </c>
+      <c r="AE119" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SADEXSEMVK on aec-cs2-hotu-nem-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF119" s="31" t="n"/>
+      <c r="AG119" s="24" t="n"/>
+      <c r="AH119" s="24" t="n"/>
+      <c r="AI119" s="31" t="n"/>
+      <c r="AJ119" s="31" t="n"/>
+      <c r="AK119" s="24" t="n"/>
+      <c r="AL119" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM119" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN119" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO119" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP119" s="24" t="n"/>
+      <c r="AQ119" s="24" t="n"/>
+      <c r="AR119" s="24" t="n"/>
+      <c r="AS119" s="24" t="n"/>
+      <c r="AT119" s="24" t="n"/>
+      <c r="AU119" s="24" t="n"/>
+      <c r="AV119" s="24" t="n"/>
+      <c r="AW119" s="24" t="n"/>
+      <c r="AX119" s="24" t="n"/>
+      <c r="AY119" s="24" t="n"/>
+      <c r="AZ119" s="24" t="n"/>
+      <c r="BA119" s="24" t="n"/>
+      <c r="BB119" s="24" t="n"/>
+      <c r="BC119" s="24" t="n"/>
+      <c r="BD119" s="24" t="n"/>
+      <c r="BE119" s="24" t="n"/>
+      <c r="BF119" s="24" t="n"/>
+      <c r="BG119" s="24" t="n"/>
+      <c r="BH119" s="24" t="n"/>
+      <c r="BI119" s="24" t="n"/>
+      <c r="BJ119" s="25" t="n"/>
+      <c r="BK119" s="26" t="n"/>
+      <c r="BL119" s="27" t="n"/>
+      <c r="BM119" s="28" t="n"/>
+      <c r="BN119" s="28" t="n"/>
+      <c r="BO119" s="28" t="n"/>
+      <c r="BP119" s="25" t="n"/>
+      <c r="BQ119" s="27" t="n"/>
+      <c r="BR119" s="28" t="n"/>
+      <c r="BS119" s="28" t="n"/>
+      <c r="BT119" s="28" t="n"/>
+      <c r="BU119" s="25" t="n"/>
+      <c r="BV119" s="29" t="n"/>
+      <c r="BW119" s="24" t="n"/>
+      <c r="BX119" s="30" t="n"/>
+      <c r="BY119" s="27" t="n"/>
+      <c r="BZ119" s="24" t="n"/>
+      <c r="CA119" s="31" t="n"/>
+      <c r="CB119" s="24" t="n"/>
+      <c r="CC119" s="24" t="n"/>
+      <c r="CD119" s="24" t="n"/>
+      <c r="CE119" s="24" t="n"/>
+      <c r="CF119" s="24" t="n"/>
+      <c r="CG119" s="24" t="n"/>
+      <c r="CH119" s="24" t="n"/>
+      <c r="CI119" s="24" t="n"/>
+      <c r="CJ119" s="24" t="n"/>
+      <c r="CK119" s="24" t="n"/>
+      <c r="CL119" s="24" t="n"/>
+      <c r="CM119" s="24" t="n"/>
+      <c r="CN119" s="24" t="n"/>
+      <c r="CO119" s="24" t="n"/>
+      <c r="CP119" s="24" t="n"/>
+      <c r="CQ119" s="24" t="n"/>
+      <c r="CR119" s="24" t="n"/>
+      <c r="CS119" s="24" t="n"/>
+      <c r="CT119" s="24" t="n"/>
+      <c r="CU119" s="24" t="n"/>
+      <c r="CV119" s="24" t="n"/>
+      <c r="CW119" s="24" t="n"/>
+      <c r="CX119" s="24" t="n"/>
+      <c r="CY119" s="24" t="n"/>
+      <c r="CZ119" s="24" t="n"/>
+      <c r="DA119" s="24" t="n"/>
+      <c r="DB119" s="24" t="n"/>
+      <c r="DC119" s="24" t="n"/>
+      <c r="DD119" s="24" t="n"/>
+      <c r="DE119" s="24" t="n"/>
+      <c r="DF119" s="24" t="n"/>
+      <c r="DG119" s="24" t="n"/>
+      <c r="DH119" s="24" t="n"/>
+      <c r="DI119" s="24" t="n"/>
+      <c r="DJ119" s="24" t="n"/>
+      <c r="DK119" s="24" t="n"/>
+      <c r="DL119" s="24" t="n"/>
+      <c r="DM119" s="24" t="n"/>
+      <c r="DN119" s="24" t="n"/>
+      <c r="DO119" s="24" t="n"/>
+      <c r="DP119" s="24" t="n"/>
+    </row>
+    <row r="120" ht="36" customHeight="1">
+      <c r="A120" s="24" t="inlineStr">
+        <is>
+          <t>008720233ab74009</t>
+        </is>
+      </c>
+      <c r="B120" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C120" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T12:00:00Z</t>
+        </is>
+      </c>
+      <c r="D120" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-k27-nemi-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E120" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F120" s="24" t="inlineStr">
+        <is>
+          <t>Nemiga</t>
+        </is>
+      </c>
+      <c r="G120" s="24" t="inlineStr">
+        <is>
+          <t>K27</t>
+        </is>
+      </c>
+      <c r="H120" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I120" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J120" s="25" t="n"/>
+      <c r="K120" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L120" s="26" t="n">
+        <v>-100</v>
+      </c>
+      <c r="M120" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="N120" s="28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O120" s="28" t="n">
+        <v>0.5435</v>
+      </c>
+      <c r="P120" s="28" t="n"/>
+      <c r="Q120" s="28" t="n">
+        <v>0.0435</v>
+      </c>
+      <c r="R120" s="26" t="n"/>
+      <c r="S120" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T120" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U120" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V120" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W120" s="26" t="n"/>
+      <c r="X120" s="26" t="n"/>
+      <c r="Y120" s="25" t="n"/>
+      <c r="Z120" s="26" t="n"/>
+      <c r="AA120" s="28" t="n"/>
+      <c r="AB120" s="28" t="n"/>
+      <c r="AC120" s="30" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AD120" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:41:14.239238Z</t>
+        </is>
+      </c>
+      <c r="AE120" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8S9ZJRFWMVY on aec-cs2-k27-nemi-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF120" s="31" t="n"/>
+      <c r="AG120" s="24" t="n"/>
+      <c r="AH120" s="24" t="n"/>
+      <c r="AI120" s="31" t="n"/>
+      <c r="AJ120" s="31" t="n"/>
+      <c r="AK120" s="24" t="n"/>
+      <c r="AL120" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM120" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN120" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO120" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP120" s="24" t="n"/>
+      <c r="AQ120" s="24" t="n"/>
+      <c r="AR120" s="24" t="n"/>
+      <c r="AS120" s="24" t="n"/>
+      <c r="AT120" s="24" t="n"/>
+      <c r="AU120" s="24" t="n"/>
+      <c r="AV120" s="24" t="n"/>
+      <c r="AW120" s="24" t="n"/>
+      <c r="AX120" s="24" t="n"/>
+      <c r="AY120" s="24" t="n"/>
+      <c r="AZ120" s="24" t="n"/>
+      <c r="BA120" s="24" t="n"/>
+      <c r="BB120" s="24" t="n"/>
+      <c r="BC120" s="24" t="n"/>
+      <c r="BD120" s="24" t="n"/>
+      <c r="BE120" s="24" t="n"/>
+      <c r="BF120" s="24" t="n"/>
+      <c r="BG120" s="24" t="n"/>
+      <c r="BH120" s="24" t="n"/>
+      <c r="BI120" s="24" t="n"/>
+      <c r="BJ120" s="25" t="n"/>
+      <c r="BK120" s="26" t="n"/>
+      <c r="BL120" s="27" t="n"/>
+      <c r="BM120" s="28" t="n"/>
+      <c r="BN120" s="28" t="n"/>
+      <c r="BO120" s="28" t="n"/>
+      <c r="BP120" s="25" t="n"/>
+      <c r="BQ120" s="27" t="n"/>
+      <c r="BR120" s="28" t="n"/>
+      <c r="BS120" s="28" t="n"/>
+      <c r="BT120" s="28" t="n"/>
+      <c r="BU120" s="25" t="n"/>
+      <c r="BV120" s="29" t="n"/>
+      <c r="BW120" s="24" t="n"/>
+      <c r="BX120" s="30" t="n"/>
+      <c r="BY120" s="27" t="n"/>
+      <c r="BZ120" s="24" t="n"/>
+      <c r="CA120" s="31" t="n"/>
+      <c r="CB120" s="24" t="n"/>
+      <c r="CC120" s="24" t="n"/>
+      <c r="CD120" s="24" t="n"/>
+      <c r="CE120" s="24" t="n"/>
+      <c r="CF120" s="24" t="n"/>
+      <c r="CG120" s="24" t="n"/>
+      <c r="CH120" s="24" t="n"/>
+      <c r="CI120" s="24" t="n"/>
+      <c r="CJ120" s="24" t="n"/>
+      <c r="CK120" s="24" t="n"/>
+      <c r="CL120" s="24" t="n"/>
+      <c r="CM120" s="24" t="n"/>
+      <c r="CN120" s="24" t="n"/>
+      <c r="CO120" s="24" t="n"/>
+      <c r="CP120" s="24" t="n"/>
+      <c r="CQ120" s="24" t="n"/>
+      <c r="CR120" s="24" t="n"/>
+      <c r="CS120" s="24" t="n"/>
+      <c r="CT120" s="24" t="n"/>
+      <c r="CU120" s="24" t="n"/>
+      <c r="CV120" s="24" t="n"/>
+      <c r="CW120" s="24" t="n"/>
+      <c r="CX120" s="24" t="n"/>
+      <c r="CY120" s="24" t="n"/>
+      <c r="CZ120" s="24" t="n"/>
+      <c r="DA120" s="24" t="n"/>
+      <c r="DB120" s="24" t="n"/>
+      <c r="DC120" s="24" t="n"/>
+      <c r="DD120" s="24" t="n"/>
+      <c r="DE120" s="24" t="n"/>
+      <c r="DF120" s="24" t="n"/>
+      <c r="DG120" s="24" t="n"/>
+      <c r="DH120" s="24" t="n"/>
+      <c r="DI120" s="24" t="n"/>
+      <c r="DJ120" s="24" t="n"/>
+      <c r="DK120" s="24" t="n"/>
+      <c r="DL120" s="24" t="n"/>
+      <c r="DM120" s="24" t="n"/>
+      <c r="DN120" s="24" t="n"/>
+      <c r="DO120" s="24" t="n"/>
+      <c r="DP120" s="24" t="n"/>
+    </row>
+    <row r="121" ht="36" customHeight="1">
+      <c r="A121" s="24" t="inlineStr">
+        <is>
+          <t>13e14aa86506432f</t>
+        </is>
+      </c>
+      <c r="B121" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C121" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T12:00:00Z</t>
+        </is>
+      </c>
+      <c r="D121" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-mgc-big-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E121" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F121" s="24" t="inlineStr">
+        <is>
+          <t>BIG</t>
+        </is>
+      </c>
+      <c r="G121" s="24" t="inlineStr">
+        <is>
+          <t>magic</t>
+        </is>
+      </c>
+      <c r="H121" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I121" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J121" s="25" t="n"/>
+      <c r="K121" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L121" s="26" t="n">
+        <v>133</v>
+      </c>
+      <c r="M121" s="27" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="N121" s="28" t="n">
+        <v>0.4292</v>
+      </c>
+      <c r="O121" s="28" t="n">
+        <v>0.5151</v>
+      </c>
+      <c r="P121" s="28" t="n"/>
+      <c r="Q121" s="28" t="n">
+        <v>0.0851</v>
+      </c>
+      <c r="R121" s="26" t="n"/>
+      <c r="S121" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T121" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U121" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V121" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W121" s="26" t="n"/>
+      <c r="X121" s="26" t="n"/>
+      <c r="Y121" s="25" t="n"/>
+      <c r="Z121" s="26" t="n"/>
+      <c r="AA121" s="28" t="n"/>
+      <c r="AB121" s="28" t="n"/>
+      <c r="AC121" s="30" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="AD121" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:41:14.239238Z</t>
+        </is>
+      </c>
+      <c r="AE121" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8S9JDPXWMW1 on aec-cs2-mgc-big-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF121" s="31" t="n"/>
+      <c r="AG121" s="24" t="n"/>
+      <c r="AH121" s="24" t="n"/>
+      <c r="AI121" s="31" t="n"/>
+      <c r="AJ121" s="31" t="n"/>
+      <c r="AK121" s="24" t="n"/>
+      <c r="AL121" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM121" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN121" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO121" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP121" s="24" t="n"/>
+      <c r="AQ121" s="24" t="n"/>
+      <c r="AR121" s="24" t="n"/>
+      <c r="AS121" s="24" t="n"/>
+      <c r="AT121" s="24" t="n"/>
+      <c r="AU121" s="24" t="n"/>
+      <c r="AV121" s="24" t="n"/>
+      <c r="AW121" s="24" t="n"/>
+      <c r="AX121" s="24" t="n"/>
+      <c r="AY121" s="24" t="n"/>
+      <c r="AZ121" s="24" t="n"/>
+      <c r="BA121" s="24" t="n"/>
+      <c r="BB121" s="24" t="n"/>
+      <c r="BC121" s="24" t="n"/>
+      <c r="BD121" s="24" t="n"/>
+      <c r="BE121" s="24" t="n"/>
+      <c r="BF121" s="24" t="n"/>
+      <c r="BG121" s="24" t="n"/>
+      <c r="BH121" s="24" t="n"/>
+      <c r="BI121" s="24" t="n"/>
+      <c r="BJ121" s="25" t="n"/>
+      <c r="BK121" s="26" t="n"/>
+      <c r="BL121" s="27" t="n"/>
+      <c r="BM121" s="28" t="n"/>
+      <c r="BN121" s="28" t="n"/>
+      <c r="BO121" s="28" t="n"/>
+      <c r="BP121" s="25" t="n"/>
+      <c r="BQ121" s="27" t="n"/>
+      <c r="BR121" s="28" t="n"/>
+      <c r="BS121" s="28" t="n"/>
+      <c r="BT121" s="28" t="n"/>
+      <c r="BU121" s="25" t="n"/>
+      <c r="BV121" s="29" t="n"/>
+      <c r="BW121" s="24" t="n"/>
+      <c r="BX121" s="30" t="n"/>
+      <c r="BY121" s="27" t="n"/>
+      <c r="BZ121" s="24" t="n"/>
+      <c r="CA121" s="31" t="n"/>
+      <c r="CB121" s="24" t="n"/>
+      <c r="CC121" s="24" t="n"/>
+      <c r="CD121" s="24" t="n"/>
+      <c r="CE121" s="24" t="n"/>
+      <c r="CF121" s="24" t="n"/>
+      <c r="CG121" s="24" t="n"/>
+      <c r="CH121" s="24" t="n"/>
+      <c r="CI121" s="24" t="n"/>
+      <c r="CJ121" s="24" t="n"/>
+      <c r="CK121" s="24" t="n"/>
+      <c r="CL121" s="24" t="n"/>
+      <c r="CM121" s="24" t="n"/>
+      <c r="CN121" s="24" t="n"/>
+      <c r="CO121" s="24" t="n"/>
+      <c r="CP121" s="24" t="n"/>
+      <c r="CQ121" s="24" t="n"/>
+      <c r="CR121" s="24" t="n"/>
+      <c r="CS121" s="24" t="n"/>
+      <c r="CT121" s="24" t="n"/>
+      <c r="CU121" s="24" t="n"/>
+      <c r="CV121" s="24" t="n"/>
+      <c r="CW121" s="24" t="n"/>
+      <c r="CX121" s="24" t="n"/>
+      <c r="CY121" s="24" t="n"/>
+      <c r="CZ121" s="24" t="n"/>
+      <c r="DA121" s="24" t="n"/>
+      <c r="DB121" s="24" t="n"/>
+      <c r="DC121" s="24" t="n"/>
+      <c r="DD121" s="24" t="n"/>
+      <c r="DE121" s="24" t="n"/>
+      <c r="DF121" s="24" t="n"/>
+      <c r="DG121" s="24" t="n"/>
+      <c r="DH121" s="24" t="n"/>
+      <c r="DI121" s="24" t="n"/>
+      <c r="DJ121" s="24" t="n"/>
+      <c r="DK121" s="24" t="n"/>
+      <c r="DL121" s="24" t="n"/>
+      <c r="DM121" s="24" t="n"/>
+      <c r="DN121" s="24" t="n"/>
+      <c r="DO121" s="24" t="n"/>
+      <c r="DP121" s="24" t="n"/>
+    </row>
+    <row r="122" ht="36" customHeight="1">
+      <c r="A122" s="24" t="inlineStr">
+        <is>
+          <t>4d37bfccafc046d9</t>
+        </is>
+      </c>
+      <c r="B122" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T04:38:33.638803Z</t>
+        </is>
+      </c>
+      <c r="C122" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="D122" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-ntr-ef-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E122" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F122" s="24" t="inlineStr">
+        <is>
+          <t>Eternal Fire</t>
+        </is>
+      </c>
+      <c r="G122" s="24" t="inlineStr">
+        <is>
+          <t>Nuclear TigeRES</t>
+        </is>
+      </c>
+      <c r="H122" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I122" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J122" s="25" t="n"/>
+      <c r="K122" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L122" s="26" t="n">
+        <v>113</v>
+      </c>
+      <c r="M122" s="27" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="N122" s="28" t="n">
+        <v>0.4695</v>
+      </c>
+      <c r="O122" s="28" t="n">
+        <v>0.6431</v>
+      </c>
+      <c r="P122" s="28" t="n"/>
+      <c r="Q122" s="28" t="n">
+        <v>0.1731</v>
+      </c>
+      <c r="R122" s="26" t="n"/>
+      <c r="S122" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T122" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U122" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V122" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W122" s="26" t="n"/>
+      <c r="X122" s="26" t="n"/>
+      <c r="Y122" s="25" t="n"/>
+      <c r="Z122" s="26" t="n"/>
+      <c r="AA122" s="28" t="n"/>
+      <c r="AB122" s="28" t="n"/>
+      <c r="AC122" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD122" s="24" t="n"/>
+      <c r="AE122" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8SADEYG6MVK on aec-cs2-ntr-ef-2026-09-03 (long)</t>
+        </is>
+      </c>
+      <c r="AF122" s="31" t="n"/>
+      <c r="AG122" s="24" t="n"/>
+      <c r="AH122" s="24" t="n"/>
+      <c r="AI122" s="31" t="n"/>
+      <c r="AJ122" s="31" t="n"/>
+      <c r="AK122" s="24" t="n"/>
+      <c r="AL122" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM122" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN122" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO122" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP122" s="24" t="n"/>
+      <c r="AQ122" s="24" t="n"/>
+      <c r="AR122" s="24" t="n"/>
+      <c r="AS122" s="24" t="n"/>
+      <c r="AT122" s="24" t="n"/>
+      <c r="AU122" s="24" t="n"/>
+      <c r="AV122" s="24" t="n"/>
+      <c r="AW122" s="24" t="n"/>
+      <c r="AX122" s="24" t="n"/>
+      <c r="AY122" s="24" t="n"/>
+      <c r="AZ122" s="24" t="n"/>
+      <c r="BA122" s="24" t="n"/>
+      <c r="BB122" s="24" t="n"/>
+      <c r="BC122" s="24" t="n"/>
+      <c r="BD122" s="24" t="n"/>
+      <c r="BE122" s="24" t="n"/>
+      <c r="BF122" s="24" t="n"/>
+      <c r="BG122" s="24" t="n"/>
+      <c r="BH122" s="24" t="n"/>
+      <c r="BI122" s="24" t="n"/>
+      <c r="BJ122" s="25" t="n"/>
+      <c r="BK122" s="26" t="n"/>
+      <c r="BL122" s="27" t="n"/>
+      <c r="BM122" s="28" t="n"/>
+      <c r="BN122" s="28" t="n"/>
+      <c r="BO122" s="28" t="n"/>
+      <c r="BP122" s="25" t="n"/>
+      <c r="BQ122" s="27" t="n"/>
+      <c r="BR122" s="28" t="n"/>
+      <c r="BS122" s="28" t="n"/>
+      <c r="BT122" s="28" t="n"/>
+      <c r="BU122" s="25" t="n"/>
+      <c r="BV122" s="29" t="n"/>
+      <c r="BW122" s="24" t="n"/>
+      <c r="BX122" s="30" t="n"/>
+      <c r="BY122" s="27" t="n"/>
+      <c r="BZ122" s="24" t="n"/>
+      <c r="CA122" s="31" t="n"/>
+      <c r="CB122" s="24" t="n"/>
+      <c r="CC122" s="24" t="n"/>
+      <c r="CD122" s="24" t="n"/>
+      <c r="CE122" s="24" t="n"/>
+      <c r="CF122" s="24" t="n"/>
+      <c r="CG122" s="24" t="n"/>
+      <c r="CH122" s="24" t="n"/>
+      <c r="CI122" s="24" t="n"/>
+      <c r="CJ122" s="24" t="n"/>
+      <c r="CK122" s="24" t="n"/>
+      <c r="CL122" s="24" t="n"/>
+      <c r="CM122" s="24" t="n"/>
+      <c r="CN122" s="24" t="n"/>
+      <c r="CO122" s="24" t="n"/>
+      <c r="CP122" s="24" t="n"/>
+      <c r="CQ122" s="24" t="n"/>
+      <c r="CR122" s="24" t="n"/>
+      <c r="CS122" s="24" t="n"/>
+      <c r="CT122" s="24" t="n"/>
+      <c r="CU122" s="24" t="n"/>
+      <c r="CV122" s="24" t="n"/>
+      <c r="CW122" s="24" t="n"/>
+      <c r="CX122" s="24" t="n"/>
+      <c r="CY122" s="24" t="n"/>
+      <c r="CZ122" s="24" t="n"/>
+      <c r="DA122" s="24" t="n"/>
+      <c r="DB122" s="24" t="n"/>
+      <c r="DC122" s="24" t="n"/>
+      <c r="DD122" s="24" t="n"/>
+      <c r="DE122" s="24" t="n"/>
+      <c r="DF122" s="24" t="n"/>
+      <c r="DG122" s="24" t="n"/>
+      <c r="DH122" s="24" t="n"/>
+      <c r="DI122" s="24" t="n"/>
+      <c r="DJ122" s="24" t="n"/>
+      <c r="DK122" s="24" t="n"/>
+      <c r="DL122" s="24" t="n"/>
+      <c r="DM122" s="24" t="n"/>
+      <c r="DN122" s="24" t="n"/>
+      <c r="DO122" s="24" t="n"/>
+      <c r="DP122" s="24" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix(auto-buyer): reconcile unknown fills, prevent phantom settlement, and synchronize ledger truth
</commit_message>
<xml_diff>
--- a/data/auto_buyer_picks.xlsx
+++ b/data/auto_buyer_picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DP122" headerRowCount="1">
-  <autoFilter ref="A1:DP122"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DP139" headerRowCount="1">
+  <autoFilter ref="A1:DP139"/>
   <tableColumns count="120">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -779,19 +779,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$122)</f>
+        <f>COUNTA('Picks'!$A$2:$A$139)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$122,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$139,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$122,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$139,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"win")+COUNTIFS('Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$139,"settled",'Picks'!$V$2:$V$139,"win")+COUNTIFS('Picks'!$U$2:$U$139,"settled",'Picks'!$V$2:$V$139,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -819,19 +819,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$122,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$139,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$139,"&gt;0",'Picks'!$V$2:$V$139,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$139,"&gt;0",'Picks'!$V$2:$V$139,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"win")/(COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"win")+COUNTIFS('Picks'!$BX$2:$BX$122,"&gt;0",'Picks'!$V$2:$V$122,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$139,"&gt;0",'Picks'!$V$2:$V$139,"win")/(COUNTIFS('Picks'!$BX$2:$BX$139,"&gt;0",'Picks'!$V$2:$V$139,"win")+COUNTIFS('Picks'!$BX$2:$BX$139,"&gt;0",'Picks'!$V$2:$V$139,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$122)/SUM('Picks'!$BX$2:$BX$122),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$139)/SUM('Picks'!$BX$2:$BX$139),0)</f>
         <v/>
       </c>
     </row>
@@ -859,19 +859,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$122)</f>
+        <f>SUM('Picks'!$BY$2:$BY$139)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$122,"&lt;&gt;",'Picks'!$AB$2:$AB$122),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$139,"&lt;&gt;",'Picks'!$AB$2:$AB$139),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$122,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$122,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$139,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$139,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$122,'Picks'!$AM$2:$AM$122,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$139,'Picks'!$AM$2:$AM$139,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -926,15 +926,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A14,'Picks'!$U$2:$U$122,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A14,'Picks'!$U$2:$U$139,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A14,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A14,'Picks'!$U$2:$U$139,"settled",'Picks'!$V$2:$V$139,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A14,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A14,'Picks'!$U$2:$U$139,"settled",'Picks'!$V$2:$V$139,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -942,11 +942,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$122,'Picks'!$H$2:$H$122,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$139,'Picks'!$H$2:$H$139,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$122,'Picks'!$H$2:$H$122,$A14,'Picks'!$U$2:$U$122,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$139,'Picks'!$H$2:$H$139,$A14,'Picks'!$U$2:$U$139,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -957,15 +957,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A15,'Picks'!$U$2:$U$122,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A15,'Picks'!$U$2:$U$139,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A15,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A15,'Picks'!$U$2:$U$139,"settled",'Picks'!$V$2:$V$139,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A15,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A15,'Picks'!$U$2:$U$139,"settled",'Picks'!$V$2:$V$139,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -973,11 +973,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$122,'Picks'!$H$2:$H$122,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$139,'Picks'!$H$2:$H$139,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$122,'Picks'!$H$2:$H$122,$A15,'Picks'!$U$2:$U$122,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$139,'Picks'!$H$2:$H$139,$A15,'Picks'!$U$2:$U$139,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -988,15 +988,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A16,'Picks'!$U$2:$U$122,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A16,'Picks'!$U$2:$U$139,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A16,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A16,'Picks'!$U$2:$U$139,"settled",'Picks'!$V$2:$V$139,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$122,$A16,'Picks'!$U$2:$U$122,"settled",'Picks'!$V$2:$V$122,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$139,$A16,'Picks'!$U$2:$U$139,"settled",'Picks'!$V$2:$V$139,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -1004,11 +1004,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$122,'Picks'!$H$2:$H$122,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$139,'Picks'!$H$2:$H$139,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$122,'Picks'!$H$2:$H$122,$A16,'Picks'!$U$2:$U$122,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$139,'Picks'!$H$2:$H$139,$A16,'Picks'!$U$2:$U$139,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DP122"/>
+  <dimension ref="A1:DP139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2080,11 +2080,11 @@
       <c r="AA3" s="28" t="n"/>
       <c r="AB3" s="28" t="n"/>
       <c r="AC3" s="30" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T21:02:17.739705Z</t>
+          <t>2026-08-30T21:00:59.237064596Z</t>
         </is>
       </c>
       <c r="AE3" s="31" t="inlineStr">
@@ -2296,11 +2296,11 @@
       <c r="AA4" s="28" t="n"/>
       <c r="AB4" s="28" t="n"/>
       <c r="AC4" s="30" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T21:29:23.578191Z</t>
+          <t>2026-08-30T21:12:34.084264238Z</t>
         </is>
       </c>
       <c r="AE4" s="31" t="inlineStr">
@@ -2508,11 +2508,11 @@
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
       <c r="AC5" s="30" t="n">
-        <v>1.1</v>
+        <v>1.08</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T21:02:17.739705Z</t>
+          <t>2026-08-30T18:53:59.356255520Z</t>
         </is>
       </c>
       <c r="AE5" s="31" t="inlineStr">
@@ -2720,11 +2720,11 @@
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
       <c r="AC6" s="30" t="n">
-        <v>1.16</v>
+        <v>1.14</v>
       </c>
       <c r="AD6" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T21:02:17.739705Z</t>
+          <t>2026-08-30T20:55:03.737915379Z</t>
         </is>
       </c>
       <c r="AE6" s="31" t="inlineStr">
@@ -2932,11 +2932,11 @@
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
       <c r="AC7" s="30" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="AD7" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T01:47:49.455874Z</t>
+          <t>2026-08-30T23:59:38.006704226Z</t>
         </is>
       </c>
       <c r="AE7" s="31" t="inlineStr">
@@ -3144,11 +3144,11 @@
       <c r="AA8" s="28" t="n"/>
       <c r="AB8" s="28" t="n"/>
       <c r="AC8" s="30" t="n">
-        <v>1</v>
+        <v>0.96</v>
       </c>
       <c r="AD8" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T21:30:23.932460Z</t>
+          <t>2026-08-30T21:44:48.583035980Z</t>
         </is>
       </c>
       <c r="AE8" s="31" t="inlineStr">
@@ -3356,11 +3356,11 @@
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
       <c r="AC9" s="30" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="AD9" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T18:13:23.815760Z</t>
+          <t>2026-08-30T17:03:18.404033999Z</t>
         </is>
       </c>
       <c r="AE9" s="31" t="inlineStr">
@@ -3568,11 +3568,11 @@
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
       <c r="AC10" s="30" t="n">
-        <v>-1.34</v>
+        <v>-1.36</v>
       </c>
       <c r="AD10" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T21:02:17.739705Z</t>
+          <t>2026-08-30T21:08:57.550864338Z</t>
         </is>
       </c>
       <c r="AE10" s="31" t="inlineStr">
@@ -3780,11 +3780,11 @@
       <c r="AA11" s="28" t="n"/>
       <c r="AB11" s="28" t="n"/>
       <c r="AC11" s="30" t="n">
-        <v>-0.88</v>
+        <v>-0.9</v>
       </c>
       <c r="AD11" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T21:02:17.739705Z</t>
+          <t>2026-08-30T21:07:47.852390448Z</t>
         </is>
       </c>
       <c r="AE11" s="31" t="inlineStr">
@@ -3992,11 +3992,11 @@
       <c r="AA12" s="28" t="n"/>
       <c r="AB12" s="28" t="n"/>
       <c r="AC12" s="30" t="n">
-        <v>1.24</v>
+        <v>1.22</v>
       </c>
       <c r="AD12" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T01:47:49.455874Z</t>
+          <t>2026-08-30T22:23:48.254732909Z</t>
         </is>
       </c>
       <c r="AE12" s="31" t="inlineStr">
@@ -4204,11 +4204,11 @@
       <c r="AA13" s="28" t="n"/>
       <c r="AB13" s="28" t="n"/>
       <c r="AC13" s="30" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="AD13" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T01:47:49.455874Z</t>
+          <t>2026-08-30T23:00:18.347523723Z</t>
         </is>
       </c>
       <c r="AE13" s="31" t="inlineStr">
@@ -4418,11 +4418,11 @@
       <c r="AA14" s="28" t="n"/>
       <c r="AB14" s="28" t="n"/>
       <c r="AC14" s="30" t="n">
-        <v>-1.14</v>
+        <v>-1.16</v>
       </c>
       <c r="AD14" s="24" t="inlineStr">
         <is>
-          <t>2026-08-30T21:29:23.578191Z</t>
+          <t>2026-08-30T21:06:03.341016599Z</t>
         </is>
       </c>
       <c r="AE14" s="31" t="inlineStr">
@@ -4634,11 +4634,11 @@
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
       <c r="AC15" s="30" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.96</v>
       </c>
       <c r="AD15" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T01:47:49.455874Z</t>
+          <t>2026-08-30T23:02:59.181343795Z</t>
         </is>
       </c>
       <c r="AE15" s="31" t="inlineStr">
@@ -4846,11 +4846,11 @@
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
       <c r="AC16" s="30" t="n">
-        <v>-1.02</v>
+        <v>-1.04</v>
       </c>
       <c r="AD16" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T01:47:49.455874Z</t>
+          <t>2026-08-30T23:06:15.866769516Z</t>
         </is>
       </c>
       <c r="AE16" s="31" t="inlineStr">
@@ -5058,11 +5058,11 @@
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
       <c r="AC17" s="30" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T18:41:38.707356Z</t>
+          <t>2026-08-31T18:27:28.086989559Z</t>
         </is>
       </c>
       <c r="AE17" s="31" t="inlineStr">
@@ -5272,11 +5272,11 @@
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
       <c r="AC18" s="30" t="n">
-        <v>0.66</v>
+        <v>0.64</v>
       </c>
       <c r="AD18" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T01:47:49.455874Z</t>
+          <t>2026-08-31T00:52:49.510904509Z</t>
         </is>
       </c>
       <c r="AE18" s="31" t="inlineStr">
@@ -5484,11 +5484,11 @@
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
       <c r="AC19" s="30" t="n">
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="AD19" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T01:59:03.295568Z</t>
+          <t>2026-08-31T03:58:48.536124373Z</t>
         </is>
       </c>
       <c r="AE19" s="31" t="inlineStr">
@@ -5694,11 +5694,11 @@
       <c r="AA20" s="28" t="n"/>
       <c r="AB20" s="28" t="n"/>
       <c r="AC20" s="30" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="AD20" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T16:02:25.134027Z</t>
+          <t>2026-08-31T11:00:03.697515228Z</t>
         </is>
       </c>
       <c r="AE20" s="31" t="inlineStr">
@@ -5904,11 +5904,11 @@
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n"/>
       <c r="AC21" s="30" t="n">
-        <v>-0.92</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="AD21" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T04:02:34.026411Z</t>
+          <t>2026-08-30T20:24:20.395157730Z</t>
         </is>
       </c>
       <c r="AE21" s="31" t="inlineStr">
@@ -6114,11 +6114,11 @@
       <c r="AA22" s="28" t="n"/>
       <c r="AB22" s="28" t="n"/>
       <c r="AC22" s="30" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AD22" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T04:01:24.010499Z</t>
+          <t>2026-08-30T21:22:08.748834907Z</t>
         </is>
       </c>
       <c r="AE22" s="31" t="inlineStr">
@@ -6324,11 +6324,11 @@
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n"/>
       <c r="AC23" s="30" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T04:01:24.010499Z</t>
+          <t>2026-08-30T23:52:48.541092830Z</t>
         </is>
       </c>
       <c r="AE23" s="31" t="inlineStr">
@@ -6744,11 +6744,11 @@
       <c r="AA25" s="28" t="n"/>
       <c r="AB25" s="28" t="n"/>
       <c r="AC25" s="30" t="n">
-        <v>-0.92</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="AD25" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T04:01:24.010499Z</t>
+          <t>2026-08-30T21:32:25.656048661Z</t>
         </is>
       </c>
       <c r="AE25" s="31" t="inlineStr">
@@ -7172,11 +7172,11 @@
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
       <c r="AC27" s="30" t="n">
-        <v>-0.78</v>
+        <v>-0.8</v>
       </c>
       <c r="AD27" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T18:41:38.707356Z</t>
+          <t>2026-08-31T16:58:29.020261016Z</t>
         </is>
       </c>
       <c r="AE27" s="31" t="inlineStr">
@@ -7384,11 +7384,11 @@
       <c r="AA28" s="28" t="n"/>
       <c r="AB28" s="28" t="n"/>
       <c r="AC28" s="30" t="n">
-        <v>-0.68</v>
+        <v>-0.7</v>
       </c>
       <c r="AD28" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T19:58:20.483072Z</t>
+          <t>2026-08-31T19:09:23.048313655Z</t>
         </is>
       </c>
       <c r="AE28" s="31" t="inlineStr">
@@ -7596,11 +7596,11 @@
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
       <c r="AC29" s="30" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T18:41:38.707356Z</t>
+          <t>2026-08-31T17:16:03.313048988Z</t>
         </is>
       </c>
       <c r="AE29" s="31" t="inlineStr">
@@ -7808,11 +7808,11 @@
       <c r="AA30" s="28" t="n"/>
       <c r="AB30" s="28" t="n"/>
       <c r="AC30" s="30" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AD30" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T20:52:02.503057Z</t>
+          <t>2026-08-31T20:53:58.036522501Z</t>
         </is>
       </c>
       <c r="AE30" s="31" t="inlineStr">
@@ -8020,11 +8020,11 @@
       <c r="AA31" s="28" t="n"/>
       <c r="AB31" s="28" t="n"/>
       <c r="AC31" s="30" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="AD31" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T19:58:20.483072Z</t>
+          <t>2026-08-31T20:11:28.041703979Z</t>
         </is>
       </c>
       <c r="AE31" s="31" t="inlineStr">
@@ -8232,11 +8232,11 @@
       <c r="AA32" s="28" t="n"/>
       <c r="AB32" s="28" t="n"/>
       <c r="AC32" s="30" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="AD32" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T01:06:31.555224Z</t>
+          <t>2026-08-31T22:44:38.648681532Z</t>
         </is>
       </c>
       <c r="AE32" s="31" t="inlineStr">
@@ -8444,11 +8444,11 @@
       <c r="AA33" s="28" t="n"/>
       <c r="AB33" s="28" t="n"/>
       <c r="AC33" s="30" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="AD33" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T19:58:20.483072Z</t>
+          <t>2026-08-31T19:52:23.076721877Z</t>
         </is>
       </c>
       <c r="AE33" s="31" t="inlineStr">
@@ -8656,11 +8656,11 @@
       <c r="AA34" s="28" t="n"/>
       <c r="AB34" s="28" t="n"/>
       <c r="AC34" s="30" t="n">
-        <v>-0.86</v>
+        <v>-0.88</v>
       </c>
       <c r="AD34" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T01:06:31.555224Z</t>
+          <t>2026-08-31T22:45:58.023703924Z</t>
         </is>
       </c>
       <c r="AE34" s="31" t="inlineStr">
@@ -8856,7 +8856,7 @@
       </c>
       <c r="V35" s="24" t="inlineStr">
         <is>
-          <t>win</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="W35" s="26" t="n"/>
@@ -8866,11 +8866,11 @@
       <c r="AA35" s="28" t="n"/>
       <c r="AB35" s="28" t="n"/>
       <c r="AC35" s="30" t="n">
-        <v>1.06</v>
+        <v>-0.96</v>
       </c>
       <c r="AD35" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T16:02:25.134027Z</t>
+          <t>2026-08-31T09:37:32.992024705Z</t>
         </is>
       </c>
       <c r="AE35" s="31" t="inlineStr">
@@ -9286,11 +9286,11 @@
       <c r="AA37" s="28" t="n"/>
       <c r="AB37" s="28" t="n"/>
       <c r="AC37" s="30" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="AD37" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T16:02:25.134027Z</t>
+          <t>2026-08-31T15:00:58.786217103Z</t>
         </is>
       </c>
       <c r="AE37" s="31" t="inlineStr">
@@ -9496,11 +9496,11 @@
       <c r="AA38" s="28" t="n"/>
       <c r="AB38" s="28" t="n"/>
       <c r="AC38" s="30" t="n">
-        <v>1</v>
+        <v>0.96</v>
       </c>
       <c r="AD38" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T03:08:18.589524Z</t>
+          <t>2026-08-31T16:15:43.108683054Z</t>
         </is>
       </c>
       <c r="AE38" s="31" t="inlineStr">
@@ -9706,11 +9706,11 @@
       <c r="AA39" s="28" t="n"/>
       <c r="AB39" s="28" t="n"/>
       <c r="AC39" s="30" t="n">
-        <v>-1.1</v>
+        <v>-1.12</v>
       </c>
       <c r="AD39" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T16:02:25.134027Z</t>
+          <t>2026-08-31T15:37:57.988972966Z</t>
         </is>
       </c>
       <c r="AE39" s="31" t="inlineStr">
@@ -9916,11 +9916,11 @@
       <c r="AA40" s="28" t="n"/>
       <c r="AB40" s="28" t="n"/>
       <c r="AC40" s="30" t="n">
-        <v>-1.1</v>
+        <v>-1.12</v>
       </c>
       <c r="AD40" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T03:08:18.589524Z</t>
+          <t>2026-08-31T17:59:23.147516089Z</t>
         </is>
       </c>
       <c r="AE40" s="31" t="inlineStr">
@@ -10126,11 +10126,11 @@
       <c r="AA41" s="28" t="n"/>
       <c r="AB41" s="28" t="n"/>
       <c r="AC41" s="30" t="n">
-        <v>0.64</v>
+        <v>0.62</v>
       </c>
       <c r="AD41" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T03:08:18.589524Z</t>
+          <t>2026-08-31T20:24:53.926365895Z</t>
         </is>
       </c>
       <c r="AE41" s="31" t="inlineStr">
@@ -10336,11 +10336,11 @@
       <c r="AA42" s="28" t="n"/>
       <c r="AB42" s="28" t="n"/>
       <c r="AC42" s="30" t="n">
-        <v>1</v>
+        <v>0.96</v>
       </c>
       <c r="AD42" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T03:08:18.589524Z</t>
+          <t>2026-08-31T20:20:34.042912899Z</t>
         </is>
       </c>
       <c r="AE42" s="31" t="inlineStr">
@@ -10764,11 +10764,11 @@
       <c r="AA44" s="28" t="n"/>
       <c r="AB44" s="28" t="n"/>
       <c r="AC44" s="30" t="n">
-        <v>-0.92</v>
+        <v>-0.93</v>
       </c>
       <c r="AD44" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T02:26:20.477542Z</t>
+          <t>2026-09-01T02:10:43.568442228Z</t>
         </is>
       </c>
       <c r="AE44" s="31" t="inlineStr">
@@ -11186,11 +11186,11 @@
       <c r="AA46" s="28" t="n"/>
       <c r="AB46" s="28" t="n"/>
       <c r="AC46" s="30" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AD46" s="24" t="inlineStr">
         <is>
-          <t>2026-08-31T21:15:44.676592Z</t>
+          <t>2026-08-31T21:17:23.007193367Z</t>
         </is>
       </c>
       <c r="AE46" s="31" t="inlineStr">
@@ -11396,11 +11396,11 @@
       <c r="AA47" s="28" t="n"/>
       <c r="AB47" s="28" t="n"/>
       <c r="AC47" s="30" t="n">
-        <v>-0.64</v>
+        <v>-0.66</v>
       </c>
       <c r="AD47" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T03:08:18.589524Z</t>
+          <t>2026-08-31T20:27:58.618077525Z</t>
         </is>
       </c>
       <c r="AE47" s="31" t="inlineStr">
@@ -11606,11 +11606,11 @@
       <c r="AA48" s="28" t="n"/>
       <c r="AB48" s="28" t="n"/>
       <c r="AC48" s="30" t="n">
-        <v>-0.64</v>
+        <v>-0.66</v>
       </c>
       <c r="AD48" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T03:08:18.589524Z</t>
+          <t>2026-08-31T23:34:08.396620140Z</t>
         </is>
       </c>
       <c r="AE48" s="31" t="inlineStr">
@@ -11822,11 +11822,11 @@
       <c r="AA49" s="28" t="n"/>
       <c r="AB49" s="28" t="n"/>
       <c r="AC49" s="30" t="n">
-        <v>-0.9</v>
+        <v>-0.92</v>
       </c>
       <c r="AD49" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T01:06:31.555224Z</t>
+          <t>2026-09-01T00:32:49.129618616Z</t>
         </is>
       </c>
       <c r="AE49" s="31" t="inlineStr">
@@ -12038,11 +12038,11 @@
       <c r="AA50" s="28" t="n"/>
       <c r="AB50" s="28" t="n"/>
       <c r="AC50" s="30" t="n">
-        <v>-1</v>
+        <v>-1.03</v>
       </c>
       <c r="AD50" s="24" t="inlineStr">
         <is>
-          <t>2026-09-01T02:26:20.477542Z</t>
+          <t>2026-09-01T02:25:14.474989956Z</t>
         </is>
       </c>
       <c r="AE50" s="31" t="inlineStr">
@@ -17480,7 +17480,7 @@
       </c>
       <c r="R76" s="26" t="n"/>
       <c r="S76" s="29" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="T76" s="24" t="inlineStr">
         <is>
@@ -17489,12 +17489,12 @@
       </c>
       <c r="U76" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V76" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>push</t>
         </is>
       </c>
       <c r="W76" s="26" t="n"/>
@@ -17506,7 +17506,11 @@
       <c r="AC76" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="AD76" s="24" t="n"/>
+      <c r="AD76" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:31:41.996535+00:00</t>
+        </is>
+      </c>
       <c r="AE76" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C83KK4ZN6M9F on aec-cs2-ntr-gl-2026-09-02 (long)</t>
@@ -20005,12 +20009,12 @@
       </c>
       <c r="U88" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V88" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>push</t>
         </is>
       </c>
       <c r="W88" s="26" t="n"/>
@@ -20022,7 +20026,11 @@
       <c r="AC88" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="AD88" s="24" t="n"/>
+      <c r="AD88" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:31:41.996557+00:00</t>
+        </is>
+      </c>
       <c r="AE88" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C84KN9MBEMAC on aec-cs2-sparta-jpu-2026-09-02 (long)</t>
@@ -20832,7 +20840,7 @@
       </c>
       <c r="R92" s="26" t="n"/>
       <c r="S92" s="29" t="n">
-        <v>1.26</v>
+        <v>1.25</v>
       </c>
       <c r="T92" s="24" t="inlineStr">
         <is>
@@ -20841,12 +20849,12 @@
       </c>
       <c r="U92" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V92" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>push</t>
         </is>
       </c>
       <c r="W92" s="26" t="n"/>
@@ -20858,7 +20866,11 @@
       <c r="AC92" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="AD92" s="24" t="n"/>
+      <c r="AD92" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:31:41.996569+00:00</t>
+        </is>
+      </c>
       <c r="AE92" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C84N4FF4GMCS on aec-cs2-hotu-ntr-2026-09-02 (short)</t>
@@ -22097,12 +22109,12 @@
       </c>
       <c r="U98" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V98" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W98" s="26" t="n"/>
@@ -22112,9 +22124,13 @@
       <c r="AA98" s="28" t="n"/>
       <c r="AB98" s="28" t="n"/>
       <c r="AC98" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD98" s="24" t="n"/>
+        <v>0.97</v>
+      </c>
+      <c r="AD98" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:21:35.150063Z</t>
+        </is>
+      </c>
       <c r="AE98" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8EQVPVMMMVK on aec-cs2-navij-sdf-2026-09-02 (long)</t>
@@ -23349,12 +23365,12 @@
       </c>
       <c r="U104" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V104" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W104" s="26" t="n"/>
@@ -23364,9 +23380,13 @@
       <c r="AA104" s="28" t="n"/>
       <c r="AB104" s="28" t="n"/>
       <c r="AC104" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD104" s="24" t="n"/>
+        <v>0.23</v>
+      </c>
+      <c r="AD104" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:21:35.150063Z</t>
+        </is>
+      </c>
       <c r="AE104" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SAC97KPMW0 on aec-wta-jesman-eleryb-2026-09-02 (short)</t>
@@ -23555,12 +23575,12 @@
       </c>
       <c r="U105" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V105" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="W105" s="26" t="n"/>
@@ -23570,9 +23590,13 @@
       <c r="AA105" s="28" t="n"/>
       <c r="AB105" s="28" t="n"/>
       <c r="AC105" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD105" s="24" t="n"/>
+        <v>-1.02</v>
+      </c>
+      <c r="AD105" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:46:54.513627Z</t>
+        </is>
+      </c>
       <c r="AE105" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8S9JGNDPMVY on aec-atp-felaug-karkha-2026-09-02 (long)</t>
@@ -23761,24 +23785,30 @@
       </c>
       <c r="U106" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V106" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W106" s="26" t="n"/>
-      <c r="X106" s="26" t="n"/>
+      <c r="X106" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y106" s="25" t="n"/>
       <c r="Z106" s="26" t="n"/>
       <c r="AA106" s="28" t="n"/>
       <c r="AB106" s="28" t="n"/>
       <c r="AC106" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD106" s="24" t="n"/>
+        <v>0.73</v>
+      </c>
+      <c r="AD106" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T19:10:41.048939747Z</t>
+        </is>
+      </c>
       <c r="AE106" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SAJ717GMVR on aec-atp-lucdar-dalsvr-2026-09-02 (long)</t>
@@ -23967,24 +23997,30 @@
       </c>
       <c r="U107" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V107" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="W107" s="26" t="n"/>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W107" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="X107" s="26" t="n"/>
       <c r="Y107" s="25" t="n"/>
       <c r="Z107" s="26" t="n"/>
       <c r="AA107" s="28" t="n"/>
       <c r="AB107" s="28" t="n"/>
       <c r="AC107" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD107" s="24" t="n"/>
+        <v>0.92</v>
+      </c>
+      <c r="AD107" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T19:37:56.025811831Z</t>
+        </is>
+      </c>
       <c r="AE107" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SA9KYNEMVF on aec-atp-janstr-fracer-2026-09-02 (short)</t>
@@ -24164,7 +24200,7 @@
       </c>
       <c r="R108" s="26" t="n"/>
       <c r="S108" s="29" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="T108" s="24" t="inlineStr">
         <is>
@@ -24173,16 +24209,18 @@
       </c>
       <c r="U108" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V108" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>void</t>
         </is>
       </c>
       <c r="W108" s="26" t="n"/>
-      <c r="X108" s="26" t="n"/>
+      <c r="X108" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y108" s="25" t="n"/>
       <c r="Z108" s="26" t="n"/>
       <c r="AA108" s="28" t="n"/>
@@ -24190,7 +24228,11 @@
       <c r="AC108" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="AD108" s="24" t="n"/>
+      <c r="AD108" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:56:21.677022+00:00</t>
+        </is>
+      </c>
       <c r="AE108" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8S9RQ5K2MVZ on aec-atp-benbon-ignbus-2026-09-03 (long)</t>
@@ -24379,12 +24421,12 @@
       </c>
       <c r="U109" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V109" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="W109" s="26" t="n"/>
@@ -24394,9 +24436,13 @@
       <c r="AA109" s="28" t="n"/>
       <c r="AB109" s="28" t="n"/>
       <c r="AC109" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD109" s="24" t="n"/>
+        <v>-1.55</v>
+      </c>
+      <c r="AD109" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:46:54.513627Z</t>
+        </is>
+      </c>
       <c r="AE109" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SA9KZAEMVF on aec-lol-doc-bce-2026-09-03 (short)</t>
@@ -24585,12 +24631,12 @@
       </c>
       <c r="U110" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V110" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W110" s="26" t="n"/>
@@ -24600,9 +24646,13 @@
       <c r="AA110" s="28" t="n"/>
       <c r="AB110" s="28" t="n"/>
       <c r="AC110" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD110" s="24" t="n"/>
+        <v>2.06</v>
+      </c>
+      <c r="AD110" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:46:54.513627Z</t>
+        </is>
+      </c>
       <c r="AE110" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SAKWMYRMVG on aec-lol-pcific-su-2026-09-03 (long)</t>
@@ -24791,12 +24841,12 @@
       </c>
       <c r="U111" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V111" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W111" s="26" t="n"/>
@@ -24806,9 +24856,13 @@
       <c r="AA111" s="28" t="n"/>
       <c r="AB111" s="28" t="n"/>
       <c r="AC111" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD111" s="24" t="n"/>
+        <v>1.32</v>
+      </c>
+      <c r="AD111" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:46:54.513627Z</t>
+        </is>
+      </c>
       <c r="AE111" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SADETDWMVK on aec-lol-sec-myth-2026-09-03 (long)</t>
@@ -24988,7 +25042,7 @@
       </c>
       <c r="R112" s="26" t="n"/>
       <c r="S112" s="29" t="n">
-        <v>1.25</v>
+        <v>0.09</v>
       </c>
       <c r="T112" s="24" t="inlineStr">
         <is>
@@ -24997,12 +25051,12 @@
       </c>
       <c r="U112" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V112" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>loss</t>
         </is>
       </c>
       <c r="W112" s="26" t="n"/>
@@ -25012,9 +25066,13 @@
       <c r="AA112" s="28" t="n"/>
       <c r="AB112" s="28" t="n"/>
       <c r="AC112" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD112" s="24" t="n"/>
+        <v>-0.25</v>
+      </c>
+      <c r="AD112" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T19:00:05.981241216Z</t>
+        </is>
+      </c>
       <c r="AE112" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SAMAA24MVP on aec-lol-lds-dv1-2026-09-03 (long)</t>
@@ -25203,12 +25261,12 @@
       </c>
       <c r="U113" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V113" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W113" s="26" t="n"/>
@@ -25218,9 +25276,13 @@
       <c r="AA113" s="28" t="n"/>
       <c r="AB113" s="28" t="n"/>
       <c r="AC113" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD113" s="24" t="n"/>
+        <v>1.75</v>
+      </c>
+      <c r="AD113" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:21:35.150063Z</t>
+        </is>
+      </c>
       <c r="AE113" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SAC9AMPMW0 on aec-lol-domi-drm-2026-09-03 (long)</t>
@@ -25610,7 +25672,7 @@
       </c>
       <c r="R115" s="26" t="n"/>
       <c r="S115" s="29" t="n">
-        <v>1.25</v>
+        <v>0.64</v>
       </c>
       <c r="T115" s="24" t="inlineStr">
         <is>
@@ -25619,12 +25681,12 @@
       </c>
       <c r="U115" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V115" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W115" s="26" t="n"/>
@@ -25634,9 +25696,13 @@
       <c r="AA115" s="28" t="n"/>
       <c r="AB115" s="28" t="n"/>
       <c r="AC115" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD115" s="24" t="n"/>
+        <v>0.76</v>
+      </c>
+      <c r="AD115" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T06:27:21.111521Z</t>
+        </is>
+      </c>
       <c r="AE115" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8S9GE15EMVV on aec-cs2-vexar-bge-2026-09-03 (long)</t>
@@ -26035,12 +26101,12 @@
       </c>
       <c r="U117" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V117" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W117" s="26" t="n"/>
@@ -26050,9 +26116,13 @@
       <c r="AA117" s="28" t="n"/>
       <c r="AB117" s="28" t="n"/>
       <c r="AC117" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD117" s="24" t="n"/>
+        <v>1.65</v>
+      </c>
+      <c r="AD117" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:46:54.513627Z</t>
+        </is>
+      </c>
       <c r="AE117" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8S9JDN66MW1 on aec-cs2-for-biga-2026-09-03 (short)</t>
@@ -27081,12 +27151,12 @@
       </c>
       <c r="U122" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>settled</t>
         </is>
       </c>
       <c r="V122" s="24" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>win</t>
         </is>
       </c>
       <c r="W122" s="26" t="n"/>
@@ -27096,9 +27166,13 @@
       <c r="AA122" s="28" t="n"/>
       <c r="AB122" s="28" t="n"/>
       <c r="AC122" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD122" s="24" t="n"/>
+        <v>1.97</v>
+      </c>
+      <c r="AD122" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:46:54.513627Z</t>
+        </is>
+      </c>
       <c r="AE122" s="31" t="inlineStr">
         <is>
           <t>Auto-Buyer order C8SADEYG6MVK on aec-cs2-ntr-ef-2026-09-03 (long)</t>
@@ -27208,6 +27282,3504 @@
       <c r="DO122" s="24" t="n"/>
       <c r="DP122" s="24" t="n"/>
     </row>
+    <row r="123" ht="36" customHeight="1">
+      <c r="A123" s="24" t="inlineStr">
+        <is>
+          <t>64564d7fda6d4e87</t>
+        </is>
+      </c>
+      <c r="B123" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:26:18.232551Z</t>
+        </is>
+      </c>
+      <c r="C123" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T11:30:00Z</t>
+        </is>
+      </c>
+      <c r="D123" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-hotu-ef-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E123" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F123" s="24" t="inlineStr">
+        <is>
+          <t>Eternal Fire</t>
+        </is>
+      </c>
+      <c r="G123" s="24" t="inlineStr">
+        <is>
+          <t>HOTU</t>
+        </is>
+      </c>
+      <c r="H123" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I123" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J123" s="25" t="n"/>
+      <c r="K123" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L123" s="26" t="n">
+        <v>-100</v>
+      </c>
+      <c r="M123" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="N123" s="28" t="n">
+        <v>0.5901999999999999</v>
+      </c>
+      <c r="O123" s="28" t="n">
+        <v>0.6056</v>
+      </c>
+      <c r="P123" s="28" t="n"/>
+      <c r="Q123" s="28" t="n">
+        <v>0.1056</v>
+      </c>
+      <c r="R123" s="26" t="n"/>
+      <c r="S123" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T123" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U123" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V123" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W123" s="26" t="n"/>
+      <c r="X123" s="26" t="n"/>
+      <c r="Y123" s="25" t="n"/>
+      <c r="Z123" s="26" t="n"/>
+      <c r="AA123" s="28" t="n"/>
+      <c r="AB123" s="28" t="n"/>
+      <c r="AC123" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD123" s="24" t="n"/>
+      <c r="AE123" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9DRPGMDGMW1 on aec-cs2-hotu-ef-2026-09-04 (long)</t>
+        </is>
+      </c>
+      <c r="AF123" s="31" t="n"/>
+      <c r="AG123" s="24" t="n"/>
+      <c r="AH123" s="24" t="n"/>
+      <c r="AI123" s="31" t="n"/>
+      <c r="AJ123" s="31" t="n"/>
+      <c r="AK123" s="24" t="n"/>
+      <c r="AL123" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM123" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN123" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO123" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP123" s="24" t="n"/>
+      <c r="AQ123" s="24" t="n"/>
+      <c r="AR123" s="24" t="n"/>
+      <c r="AS123" s="24" t="n"/>
+      <c r="AT123" s="24" t="n"/>
+      <c r="AU123" s="24" t="n"/>
+      <c r="AV123" s="24" t="n"/>
+      <c r="AW123" s="24" t="n"/>
+      <c r="AX123" s="24" t="n"/>
+      <c r="AY123" s="24" t="n"/>
+      <c r="AZ123" s="24" t="n"/>
+      <c r="BA123" s="24" t="n"/>
+      <c r="BB123" s="24" t="n"/>
+      <c r="BC123" s="24" t="n"/>
+      <c r="BD123" s="24" t="n"/>
+      <c r="BE123" s="24" t="n"/>
+      <c r="BF123" s="24" t="n"/>
+      <c r="BG123" s="24" t="n"/>
+      <c r="BH123" s="24" t="n"/>
+      <c r="BI123" s="24" t="n"/>
+      <c r="BJ123" s="25" t="n"/>
+      <c r="BK123" s="26" t="n"/>
+      <c r="BL123" s="27" t="n"/>
+      <c r="BM123" s="28" t="n"/>
+      <c r="BN123" s="28" t="n"/>
+      <c r="BO123" s="28" t="n"/>
+      <c r="BP123" s="25" t="n"/>
+      <c r="BQ123" s="27" t="n"/>
+      <c r="BR123" s="28" t="n"/>
+      <c r="BS123" s="28" t="n"/>
+      <c r="BT123" s="28" t="n"/>
+      <c r="BU123" s="25" t="n"/>
+      <c r="BV123" s="29" t="n"/>
+      <c r="BW123" s="24" t="n"/>
+      <c r="BX123" s="30" t="n"/>
+      <c r="BY123" s="27" t="n"/>
+      <c r="BZ123" s="24" t="n"/>
+      <c r="CA123" s="31" t="n"/>
+      <c r="CB123" s="24" t="n"/>
+      <c r="CC123" s="24" t="n"/>
+      <c r="CD123" s="24" t="n"/>
+      <c r="CE123" s="24" t="n"/>
+      <c r="CF123" s="24" t="n"/>
+      <c r="CG123" s="24" t="n"/>
+      <c r="CH123" s="24" t="n"/>
+      <c r="CI123" s="24" t="n"/>
+      <c r="CJ123" s="24" t="n"/>
+      <c r="CK123" s="24" t="n"/>
+      <c r="CL123" s="24" t="n"/>
+      <c r="CM123" s="24" t="n"/>
+      <c r="CN123" s="24" t="n"/>
+      <c r="CO123" s="24" t="n"/>
+      <c r="CP123" s="24" t="n"/>
+      <c r="CQ123" s="24" t="n"/>
+      <c r="CR123" s="24" t="n"/>
+      <c r="CS123" s="24" t="n"/>
+      <c r="CT123" s="24" t="n"/>
+      <c r="CU123" s="24" t="n"/>
+      <c r="CV123" s="24" t="n"/>
+      <c r="CW123" s="24" t="n"/>
+      <c r="CX123" s="24" t="n"/>
+      <c r="CY123" s="24" t="n"/>
+      <c r="CZ123" s="24" t="n"/>
+      <c r="DA123" s="24" t="n"/>
+      <c r="DB123" s="24" t="n"/>
+      <c r="DC123" s="24" t="n"/>
+      <c r="DD123" s="24" t="n"/>
+      <c r="DE123" s="24" t="n"/>
+      <c r="DF123" s="24" t="n"/>
+      <c r="DG123" s="24" t="n"/>
+      <c r="DH123" s="24" t="n"/>
+      <c r="DI123" s="24" t="n"/>
+      <c r="DJ123" s="24" t="n"/>
+      <c r="DK123" s="24" t="n"/>
+      <c r="DL123" s="24" t="n"/>
+      <c r="DM123" s="24" t="n"/>
+      <c r="DN123" s="24" t="n"/>
+      <c r="DO123" s="24" t="n"/>
+      <c r="DP123" s="24" t="n"/>
+    </row>
+    <row r="124" ht="36" customHeight="1">
+      <c r="A124" s="24" t="inlineStr">
+        <is>
+          <t>46391c8767ba45aa</t>
+        </is>
+      </c>
+      <c r="B124" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:26:18.232551Z</t>
+        </is>
+      </c>
+      <c r="C124" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T22:00:00Z</t>
+        </is>
+      </c>
+      <c r="D124" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-uno-alka-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E124" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F124" s="24" t="inlineStr">
+        <is>
+          <t>ALKA GAMING</t>
+        </is>
+      </c>
+      <c r="G124" s="24" t="inlineStr">
+        <is>
+          <t>UNO MILLE</t>
+        </is>
+      </c>
+      <c r="H124" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I124" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J124" s="25" t="n"/>
+      <c r="K124" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L124" s="26" t="n">
+        <v>-100</v>
+      </c>
+      <c r="M124" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="N124" s="28" t="n">
+        <v>0.5495</v>
+      </c>
+      <c r="O124" s="28" t="n">
+        <v>0.6655</v>
+      </c>
+      <c r="P124" s="28" t="n"/>
+      <c r="Q124" s="28" t="n">
+        <v>0.1655</v>
+      </c>
+      <c r="R124" s="26" t="n"/>
+      <c r="S124" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T124" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U124" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V124" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W124" s="26" t="n"/>
+      <c r="X124" s="26" t="n"/>
+      <c r="Y124" s="25" t="n"/>
+      <c r="Z124" s="26" t="n"/>
+      <c r="AA124" s="28" t="n"/>
+      <c r="AB124" s="28" t="n"/>
+      <c r="AC124" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD124" s="24" t="n"/>
+      <c r="AE124" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9DSQW05EMVK on aec-cs2-uno-alka-2026-09-04 (short)</t>
+        </is>
+      </c>
+      <c r="AF124" s="31" t="n"/>
+      <c r="AG124" s="24" t="n"/>
+      <c r="AH124" s="24" t="n"/>
+      <c r="AI124" s="31" t="n"/>
+      <c r="AJ124" s="31" t="n"/>
+      <c r="AK124" s="24" t="n"/>
+      <c r="AL124" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM124" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN124" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO124" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP124" s="24" t="n"/>
+      <c r="AQ124" s="24" t="n"/>
+      <c r="AR124" s="24" t="n"/>
+      <c r="AS124" s="24" t="n"/>
+      <c r="AT124" s="24" t="n"/>
+      <c r="AU124" s="24" t="n"/>
+      <c r="AV124" s="24" t="n"/>
+      <c r="AW124" s="24" t="n"/>
+      <c r="AX124" s="24" t="n"/>
+      <c r="AY124" s="24" t="n"/>
+      <c r="AZ124" s="24" t="n"/>
+      <c r="BA124" s="24" t="n"/>
+      <c r="BB124" s="24" t="n"/>
+      <c r="BC124" s="24" t="n"/>
+      <c r="BD124" s="24" t="n"/>
+      <c r="BE124" s="24" t="n"/>
+      <c r="BF124" s="24" t="n"/>
+      <c r="BG124" s="24" t="n"/>
+      <c r="BH124" s="24" t="n"/>
+      <c r="BI124" s="24" t="n"/>
+      <c r="BJ124" s="25" t="n"/>
+      <c r="BK124" s="26" t="n"/>
+      <c r="BL124" s="27" t="n"/>
+      <c r="BM124" s="28" t="n"/>
+      <c r="BN124" s="28" t="n"/>
+      <c r="BO124" s="28" t="n"/>
+      <c r="BP124" s="25" t="n"/>
+      <c r="BQ124" s="27" t="n"/>
+      <c r="BR124" s="28" t="n"/>
+      <c r="BS124" s="28" t="n"/>
+      <c r="BT124" s="28" t="n"/>
+      <c r="BU124" s="25" t="n"/>
+      <c r="BV124" s="29" t="n"/>
+      <c r="BW124" s="24" t="n"/>
+      <c r="BX124" s="30" t="n"/>
+      <c r="BY124" s="27" t="n"/>
+      <c r="BZ124" s="24" t="n"/>
+      <c r="CA124" s="31" t="n"/>
+      <c r="CB124" s="24" t="n"/>
+      <c r="CC124" s="24" t="n"/>
+      <c r="CD124" s="24" t="n"/>
+      <c r="CE124" s="24" t="n"/>
+      <c r="CF124" s="24" t="n"/>
+      <c r="CG124" s="24" t="n"/>
+      <c r="CH124" s="24" t="n"/>
+      <c r="CI124" s="24" t="n"/>
+      <c r="CJ124" s="24" t="n"/>
+      <c r="CK124" s="24" t="n"/>
+      <c r="CL124" s="24" t="n"/>
+      <c r="CM124" s="24" t="n"/>
+      <c r="CN124" s="24" t="n"/>
+      <c r="CO124" s="24" t="n"/>
+      <c r="CP124" s="24" t="n"/>
+      <c r="CQ124" s="24" t="n"/>
+      <c r="CR124" s="24" t="n"/>
+      <c r="CS124" s="24" t="n"/>
+      <c r="CT124" s="24" t="n"/>
+      <c r="CU124" s="24" t="n"/>
+      <c r="CV124" s="24" t="n"/>
+      <c r="CW124" s="24" t="n"/>
+      <c r="CX124" s="24" t="n"/>
+      <c r="CY124" s="24" t="n"/>
+      <c r="CZ124" s="24" t="n"/>
+      <c r="DA124" s="24" t="n"/>
+      <c r="DB124" s="24" t="n"/>
+      <c r="DC124" s="24" t="n"/>
+      <c r="DD124" s="24" t="n"/>
+      <c r="DE124" s="24" t="n"/>
+      <c r="DF124" s="24" t="n"/>
+      <c r="DG124" s="24" t="n"/>
+      <c r="DH124" s="24" t="n"/>
+      <c r="DI124" s="24" t="n"/>
+      <c r="DJ124" s="24" t="n"/>
+      <c r="DK124" s="24" t="n"/>
+      <c r="DL124" s="24" t="n"/>
+      <c r="DM124" s="24" t="n"/>
+      <c r="DN124" s="24" t="n"/>
+      <c r="DO124" s="24" t="n"/>
+      <c r="DP124" s="24" t="n"/>
+    </row>
+    <row r="125" ht="36" customHeight="1">
+      <c r="A125" s="24" t="inlineStr">
+        <is>
+          <t>b4340b03780a4930</t>
+        </is>
+      </c>
+      <c r="B125" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:31:41.996635+00:00</t>
+        </is>
+      </c>
+      <c r="C125" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="D125" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-bbc-wal-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E125" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F125" s="24" t="n"/>
+      <c r="G125" s="24" t="inlineStr">
+        <is>
+          <t>Walczaki</t>
+        </is>
+      </c>
+      <c r="H125" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I125" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J125" s="25" t="n"/>
+      <c r="K125" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L125" s="26" t="n">
+        <v>127</v>
+      </c>
+      <c r="M125" s="27" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="N125" s="28" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="O125" s="28" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="P125" s="28" t="n"/>
+      <c r="Q125" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R125" s="26" t="n"/>
+      <c r="S125" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T125" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U125" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V125" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W125" s="26" t="n"/>
+      <c r="X125" s="26" t="n"/>
+      <c r="Y125" s="25" t="n"/>
+      <c r="Z125" s="26" t="n"/>
+      <c r="AA125" s="28" t="n"/>
+      <c r="AB125" s="28" t="n"/>
+      <c r="AC125" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD125" s="24" t="n"/>
+      <c r="AE125" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C93CSEF08MVG on aec-cs2-bbc-wal-2026-09-04 (short)</t>
+        </is>
+      </c>
+      <c r="AF125" s="31" t="n"/>
+      <c r="AG125" s="24" t="n"/>
+      <c r="AH125" s="24" t="n"/>
+      <c r="AI125" s="31" t="n"/>
+      <c r="AJ125" s="31" t="n"/>
+      <c r="AK125" s="24" t="n"/>
+      <c r="AL125" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM125" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN125" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO125" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP125" s="24" t="n"/>
+      <c r="AQ125" s="24" t="n"/>
+      <c r="AR125" s="24" t="n"/>
+      <c r="AS125" s="24" t="n"/>
+      <c r="AT125" s="24" t="n"/>
+      <c r="AU125" s="24" t="n"/>
+      <c r="AV125" s="24" t="n"/>
+      <c r="AW125" s="24" t="n"/>
+      <c r="AX125" s="24" t="n"/>
+      <c r="AY125" s="24" t="n"/>
+      <c r="AZ125" s="24" t="n"/>
+      <c r="BA125" s="24" t="n"/>
+      <c r="BB125" s="24" t="n"/>
+      <c r="BC125" s="24" t="n"/>
+      <c r="BD125" s="24" t="n"/>
+      <c r="BE125" s="24" t="n"/>
+      <c r="BF125" s="24" t="n"/>
+      <c r="BG125" s="24" t="n"/>
+      <c r="BH125" s="24" t="n"/>
+      <c r="BI125" s="24" t="n"/>
+      <c r="BJ125" s="25" t="n"/>
+      <c r="BK125" s="26" t="n"/>
+      <c r="BL125" s="27" t="n"/>
+      <c r="BM125" s="28" t="n"/>
+      <c r="BN125" s="28" t="n"/>
+      <c r="BO125" s="28" t="n"/>
+      <c r="BP125" s="25" t="n"/>
+      <c r="BQ125" s="27" t="n"/>
+      <c r="BR125" s="28" t="n"/>
+      <c r="BS125" s="28" t="n"/>
+      <c r="BT125" s="28" t="n"/>
+      <c r="BU125" s="25" t="n"/>
+      <c r="BV125" s="29" t="n"/>
+      <c r="BW125" s="24" t="n"/>
+      <c r="BX125" s="30" t="n"/>
+      <c r="BY125" s="27" t="n"/>
+      <c r="BZ125" s="24" t="n"/>
+      <c r="CA125" s="31" t="n"/>
+      <c r="CB125" s="24" t="n"/>
+      <c r="CC125" s="24" t="n"/>
+      <c r="CD125" s="24" t="n"/>
+      <c r="CE125" s="24" t="n"/>
+      <c r="CF125" s="24" t="n"/>
+      <c r="CG125" s="24" t="n"/>
+      <c r="CH125" s="24" t="n"/>
+      <c r="CI125" s="24" t="n"/>
+      <c r="CJ125" s="24" t="n"/>
+      <c r="CK125" s="24" t="n"/>
+      <c r="CL125" s="24" t="n"/>
+      <c r="CM125" s="24" t="n"/>
+      <c r="CN125" s="24" t="n"/>
+      <c r="CO125" s="24" t="n"/>
+      <c r="CP125" s="24" t="n"/>
+      <c r="CQ125" s="24" t="n"/>
+      <c r="CR125" s="24" t="n"/>
+      <c r="CS125" s="24" t="n"/>
+      <c r="CT125" s="24" t="n"/>
+      <c r="CU125" s="24" t="n"/>
+      <c r="CV125" s="24" t="n"/>
+      <c r="CW125" s="24" t="n"/>
+      <c r="CX125" s="24" t="n"/>
+      <c r="CY125" s="24" t="n"/>
+      <c r="CZ125" s="24" t="n"/>
+      <c r="DA125" s="24" t="n"/>
+      <c r="DB125" s="24" t="n"/>
+      <c r="DC125" s="24" t="n"/>
+      <c r="DD125" s="24" t="n"/>
+      <c r="DE125" s="24" t="n"/>
+      <c r="DF125" s="24" t="n"/>
+      <c r="DG125" s="24" t="n"/>
+      <c r="DH125" s="24" t="n"/>
+      <c r="DI125" s="24" t="n"/>
+      <c r="DJ125" s="24" t="n"/>
+      <c r="DK125" s="24" t="n"/>
+      <c r="DL125" s="24" t="n"/>
+      <c r="DM125" s="24" t="n"/>
+      <c r="DN125" s="24" t="n"/>
+      <c r="DO125" s="24" t="n"/>
+      <c r="DP125" s="24" t="n"/>
+    </row>
+    <row r="126" ht="36" customHeight="1">
+      <c r="A126" s="24" t="inlineStr">
+        <is>
+          <t>f21a2eac0ae3472a</t>
+        </is>
+      </c>
+      <c r="B126" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:31:41.996652+00:00</t>
+        </is>
+      </c>
+      <c r="C126" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T09:00:00Z</t>
+        </is>
+      </c>
+      <c r="D126" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-inf-ntr-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E126" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F126" s="24" t="n"/>
+      <c r="G126" s="24" t="inlineStr">
+        <is>
+          <t>Nuclear TigeRES</t>
+        </is>
+      </c>
+      <c r="H126" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I126" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J126" s="25" t="n"/>
+      <c r="K126" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L126" s="26" t="n">
+        <v>-223</v>
+      </c>
+      <c r="M126" s="27" t="n">
+        <v>1.4484</v>
+      </c>
+      <c r="N126" s="28" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="O126" s="28" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="P126" s="28" t="n"/>
+      <c r="Q126" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R126" s="26" t="n"/>
+      <c r="S126" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T126" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U126" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V126" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W126" s="26" t="n"/>
+      <c r="X126" s="26" t="n"/>
+      <c r="Y126" s="25" t="n"/>
+      <c r="Z126" s="26" t="n"/>
+      <c r="AA126" s="28" t="n"/>
+      <c r="AB126" s="28" t="n"/>
+      <c r="AC126" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD126" s="24" t="n"/>
+      <c r="AE126" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C93D5H6T6MVR on aec-cs2-inf-ntr-2026-09-04 (short)</t>
+        </is>
+      </c>
+      <c r="AF126" s="31" t="n"/>
+      <c r="AG126" s="24" t="n"/>
+      <c r="AH126" s="24" t="n"/>
+      <c r="AI126" s="31" t="n"/>
+      <c r="AJ126" s="31" t="n"/>
+      <c r="AK126" s="24" t="n"/>
+      <c r="AL126" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM126" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN126" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO126" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP126" s="24" t="n"/>
+      <c r="AQ126" s="24" t="n"/>
+      <c r="AR126" s="24" t="n"/>
+      <c r="AS126" s="24" t="n"/>
+      <c r="AT126" s="24" t="n"/>
+      <c r="AU126" s="24" t="n"/>
+      <c r="AV126" s="24" t="n"/>
+      <c r="AW126" s="24" t="n"/>
+      <c r="AX126" s="24" t="n"/>
+      <c r="AY126" s="24" t="n"/>
+      <c r="AZ126" s="24" t="n"/>
+      <c r="BA126" s="24" t="n"/>
+      <c r="BB126" s="24" t="n"/>
+      <c r="BC126" s="24" t="n"/>
+      <c r="BD126" s="24" t="n"/>
+      <c r="BE126" s="24" t="n"/>
+      <c r="BF126" s="24" t="n"/>
+      <c r="BG126" s="24" t="n"/>
+      <c r="BH126" s="24" t="n"/>
+      <c r="BI126" s="24" t="n"/>
+      <c r="BJ126" s="25" t="n"/>
+      <c r="BK126" s="26" t="n"/>
+      <c r="BL126" s="27" t="n"/>
+      <c r="BM126" s="28" t="n"/>
+      <c r="BN126" s="28" t="n"/>
+      <c r="BO126" s="28" t="n"/>
+      <c r="BP126" s="25" t="n"/>
+      <c r="BQ126" s="27" t="n"/>
+      <c r="BR126" s="28" t="n"/>
+      <c r="BS126" s="28" t="n"/>
+      <c r="BT126" s="28" t="n"/>
+      <c r="BU126" s="25" t="n"/>
+      <c r="BV126" s="29" t="n"/>
+      <c r="BW126" s="24" t="n"/>
+      <c r="BX126" s="30" t="n"/>
+      <c r="BY126" s="27" t="n"/>
+      <c r="BZ126" s="24" t="n"/>
+      <c r="CA126" s="31" t="n"/>
+      <c r="CB126" s="24" t="n"/>
+      <c r="CC126" s="24" t="n"/>
+      <c r="CD126" s="24" t="n"/>
+      <c r="CE126" s="24" t="n"/>
+      <c r="CF126" s="24" t="n"/>
+      <c r="CG126" s="24" t="n"/>
+      <c r="CH126" s="24" t="n"/>
+      <c r="CI126" s="24" t="n"/>
+      <c r="CJ126" s="24" t="n"/>
+      <c r="CK126" s="24" t="n"/>
+      <c r="CL126" s="24" t="n"/>
+      <c r="CM126" s="24" t="n"/>
+      <c r="CN126" s="24" t="n"/>
+      <c r="CO126" s="24" t="n"/>
+      <c r="CP126" s="24" t="n"/>
+      <c r="CQ126" s="24" t="n"/>
+      <c r="CR126" s="24" t="n"/>
+      <c r="CS126" s="24" t="n"/>
+      <c r="CT126" s="24" t="n"/>
+      <c r="CU126" s="24" t="n"/>
+      <c r="CV126" s="24" t="n"/>
+      <c r="CW126" s="24" t="n"/>
+      <c r="CX126" s="24" t="n"/>
+      <c r="CY126" s="24" t="n"/>
+      <c r="CZ126" s="24" t="n"/>
+      <c r="DA126" s="24" t="n"/>
+      <c r="DB126" s="24" t="n"/>
+      <c r="DC126" s="24" t="n"/>
+      <c r="DD126" s="24" t="n"/>
+      <c r="DE126" s="24" t="n"/>
+      <c r="DF126" s="24" t="n"/>
+      <c r="DG126" s="24" t="n"/>
+      <c r="DH126" s="24" t="n"/>
+      <c r="DI126" s="24" t="n"/>
+      <c r="DJ126" s="24" t="n"/>
+      <c r="DK126" s="24" t="n"/>
+      <c r="DL126" s="24" t="n"/>
+      <c r="DM126" s="24" t="n"/>
+      <c r="DN126" s="24" t="n"/>
+      <c r="DO126" s="24" t="n"/>
+      <c r="DP126" s="24" t="n"/>
+    </row>
+    <row r="127" ht="36" customHeight="1">
+      <c r="A127" s="24" t="inlineStr">
+        <is>
+          <t>1ab96547628b445d</t>
+        </is>
+      </c>
+      <c r="B127" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:31:41.996664+00:00</t>
+        </is>
+      </c>
+      <c r="C127" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="D127" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-isg-pld-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E127" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F127" s="24" t="n"/>
+      <c r="G127" s="24" t="inlineStr">
+        <is>
+          <t>Isurus</t>
+        </is>
+      </c>
+      <c r="H127" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I127" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J127" s="25" t="n"/>
+      <c r="K127" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L127" s="26" t="n">
+        <v>133</v>
+      </c>
+      <c r="M127" s="27" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="N127" s="28" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="O127" s="28" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="P127" s="28" t="n"/>
+      <c r="Q127" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R127" s="26" t="n"/>
+      <c r="S127" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T127" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U127" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V127" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W127" s="26" t="n"/>
+      <c r="X127" s="26" t="n"/>
+      <c r="Y127" s="25" t="n"/>
+      <c r="Z127" s="26" t="n"/>
+      <c r="AA127" s="28" t="n"/>
+      <c r="AB127" s="28" t="n"/>
+      <c r="AC127" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD127" s="24" t="n"/>
+      <c r="AE127" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C93D489P0MVF on aec-cs2-isg-pld-2026-09-04 (long)</t>
+        </is>
+      </c>
+      <c r="AF127" s="31" t="n"/>
+      <c r="AG127" s="24" t="n"/>
+      <c r="AH127" s="24" t="n"/>
+      <c r="AI127" s="31" t="n"/>
+      <c r="AJ127" s="31" t="n"/>
+      <c r="AK127" s="24" t="n"/>
+      <c r="AL127" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM127" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN127" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO127" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP127" s="24" t="n"/>
+      <c r="AQ127" s="24" t="n"/>
+      <c r="AR127" s="24" t="n"/>
+      <c r="AS127" s="24" t="n"/>
+      <c r="AT127" s="24" t="n"/>
+      <c r="AU127" s="24" t="n"/>
+      <c r="AV127" s="24" t="n"/>
+      <c r="AW127" s="24" t="n"/>
+      <c r="AX127" s="24" t="n"/>
+      <c r="AY127" s="24" t="n"/>
+      <c r="AZ127" s="24" t="n"/>
+      <c r="BA127" s="24" t="n"/>
+      <c r="BB127" s="24" t="n"/>
+      <c r="BC127" s="24" t="n"/>
+      <c r="BD127" s="24" t="n"/>
+      <c r="BE127" s="24" t="n"/>
+      <c r="BF127" s="24" t="n"/>
+      <c r="BG127" s="24" t="n"/>
+      <c r="BH127" s="24" t="n"/>
+      <c r="BI127" s="24" t="n"/>
+      <c r="BJ127" s="25" t="n"/>
+      <c r="BK127" s="26" t="n"/>
+      <c r="BL127" s="27" t="n"/>
+      <c r="BM127" s="28" t="n"/>
+      <c r="BN127" s="28" t="n"/>
+      <c r="BO127" s="28" t="n"/>
+      <c r="BP127" s="25" t="n"/>
+      <c r="BQ127" s="27" t="n"/>
+      <c r="BR127" s="28" t="n"/>
+      <c r="BS127" s="28" t="n"/>
+      <c r="BT127" s="28" t="n"/>
+      <c r="BU127" s="25" t="n"/>
+      <c r="BV127" s="29" t="n"/>
+      <c r="BW127" s="24" t="n"/>
+      <c r="BX127" s="30" t="n"/>
+      <c r="BY127" s="27" t="n"/>
+      <c r="BZ127" s="24" t="n"/>
+      <c r="CA127" s="31" t="n"/>
+      <c r="CB127" s="24" t="n"/>
+      <c r="CC127" s="24" t="n"/>
+      <c r="CD127" s="24" t="n"/>
+      <c r="CE127" s="24" t="n"/>
+      <c r="CF127" s="24" t="n"/>
+      <c r="CG127" s="24" t="n"/>
+      <c r="CH127" s="24" t="n"/>
+      <c r="CI127" s="24" t="n"/>
+      <c r="CJ127" s="24" t="n"/>
+      <c r="CK127" s="24" t="n"/>
+      <c r="CL127" s="24" t="n"/>
+      <c r="CM127" s="24" t="n"/>
+      <c r="CN127" s="24" t="n"/>
+      <c r="CO127" s="24" t="n"/>
+      <c r="CP127" s="24" t="n"/>
+      <c r="CQ127" s="24" t="n"/>
+      <c r="CR127" s="24" t="n"/>
+      <c r="CS127" s="24" t="n"/>
+      <c r="CT127" s="24" t="n"/>
+      <c r="CU127" s="24" t="n"/>
+      <c r="CV127" s="24" t="n"/>
+      <c r="CW127" s="24" t="n"/>
+      <c r="CX127" s="24" t="n"/>
+      <c r="CY127" s="24" t="n"/>
+      <c r="CZ127" s="24" t="n"/>
+      <c r="DA127" s="24" t="n"/>
+      <c r="DB127" s="24" t="n"/>
+      <c r="DC127" s="24" t="n"/>
+      <c r="DD127" s="24" t="n"/>
+      <c r="DE127" s="24" t="n"/>
+      <c r="DF127" s="24" t="n"/>
+      <c r="DG127" s="24" t="n"/>
+      <c r="DH127" s="24" t="n"/>
+      <c r="DI127" s="24" t="n"/>
+      <c r="DJ127" s="24" t="n"/>
+      <c r="DK127" s="24" t="n"/>
+      <c r="DL127" s="24" t="n"/>
+      <c r="DM127" s="24" t="n"/>
+      <c r="DN127" s="24" t="n"/>
+      <c r="DO127" s="24" t="n"/>
+      <c r="DP127" s="24" t="n"/>
+    </row>
+    <row r="128" ht="36" customHeight="1">
+      <c r="A128" s="24" t="inlineStr">
+        <is>
+          <t>3f591439037e44eb</t>
+        </is>
+      </c>
+      <c r="B128" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:40:57.703355Z</t>
+        </is>
+      </c>
+      <c r="C128" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T20:30Z</t>
+        </is>
+      </c>
+      <c r="D128" s="24" t="inlineStr">
+        <is>
+          <t>aec-atp-alemic-danagu-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E128" s="24" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+      <c r="F128" s="24" t="inlineStr">
+        <is>
+          <t>Daniel Merida</t>
+        </is>
+      </c>
+      <c r="G128" s="24" t="inlineStr">
+        <is>
+          <t>Alex Michelsen</t>
+        </is>
+      </c>
+      <c r="H128" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I128" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J128" s="25" t="n"/>
+      <c r="K128" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L128" s="26" t="n">
+        <v>144</v>
+      </c>
+      <c r="M128" s="27" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="N128" s="28" t="n">
+        <v>0.4049</v>
+      </c>
+      <c r="O128" s="28" t="n">
+        <v>0.5165</v>
+      </c>
+      <c r="P128" s="28" t="n"/>
+      <c r="Q128" s="28" t="n">
+        <v>0.1115</v>
+      </c>
+      <c r="R128" s="26" t="n"/>
+      <c r="S128" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T128" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U128" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V128" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W128" s="26" t="n"/>
+      <c r="X128" s="26" t="n"/>
+      <c r="Y128" s="25" t="n"/>
+      <c r="Z128" s="26" t="n"/>
+      <c r="AA128" s="28" t="n"/>
+      <c r="AB128" s="28" t="n"/>
+      <c r="AC128" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD128" s="24" t="n"/>
+      <c r="AE128" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9DZ3TVP4MW1 on aec-atp-alemic-danagu-2026-09-03 (short)</t>
+        </is>
+      </c>
+      <c r="AF128" s="31" t="n"/>
+      <c r="AG128" s="24" t="n"/>
+      <c r="AH128" s="24" t="n"/>
+      <c r="AI128" s="31" t="n"/>
+      <c r="AJ128" s="31" t="n"/>
+      <c r="AK128" s="24" t="n"/>
+      <c r="AL128" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM128" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN128" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO128" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP128" s="24" t="n"/>
+      <c r="AQ128" s="24" t="n"/>
+      <c r="AR128" s="24" t="n"/>
+      <c r="AS128" s="24" t="n"/>
+      <c r="AT128" s="24" t="n"/>
+      <c r="AU128" s="24" t="n"/>
+      <c r="AV128" s="24" t="n"/>
+      <c r="AW128" s="24" t="n"/>
+      <c r="AX128" s="24" t="n"/>
+      <c r="AY128" s="24" t="n"/>
+      <c r="AZ128" s="24" t="n"/>
+      <c r="BA128" s="24" t="n"/>
+      <c r="BB128" s="24" t="n"/>
+      <c r="BC128" s="24" t="n"/>
+      <c r="BD128" s="24" t="n"/>
+      <c r="BE128" s="24" t="n"/>
+      <c r="BF128" s="24" t="n"/>
+      <c r="BG128" s="24" t="n"/>
+      <c r="BH128" s="24" t="n"/>
+      <c r="BI128" s="24" t="n"/>
+      <c r="BJ128" s="25" t="n"/>
+      <c r="BK128" s="26" t="n"/>
+      <c r="BL128" s="27" t="n"/>
+      <c r="BM128" s="28" t="n"/>
+      <c r="BN128" s="28" t="n"/>
+      <c r="BO128" s="28" t="n"/>
+      <c r="BP128" s="25" t="n"/>
+      <c r="BQ128" s="27" t="n"/>
+      <c r="BR128" s="28" t="n"/>
+      <c r="BS128" s="28" t="n"/>
+      <c r="BT128" s="28" t="n"/>
+      <c r="BU128" s="25" t="n"/>
+      <c r="BV128" s="29" t="n"/>
+      <c r="BW128" s="24" t="n"/>
+      <c r="BX128" s="30" t="n"/>
+      <c r="BY128" s="27" t="n"/>
+      <c r="BZ128" s="24" t="n"/>
+      <c r="CA128" s="31" t="n"/>
+      <c r="CB128" s="24" t="n"/>
+      <c r="CC128" s="24" t="n"/>
+      <c r="CD128" s="24" t="n"/>
+      <c r="CE128" s="24" t="n"/>
+      <c r="CF128" s="24" t="n"/>
+      <c r="CG128" s="24" t="n"/>
+      <c r="CH128" s="24" t="n"/>
+      <c r="CI128" s="24" t="n"/>
+      <c r="CJ128" s="24" t="n"/>
+      <c r="CK128" s="24" t="n"/>
+      <c r="CL128" s="24" t="n"/>
+      <c r="CM128" s="24" t="n"/>
+      <c r="CN128" s="24" t="n"/>
+      <c r="CO128" s="24" t="n"/>
+      <c r="CP128" s="24" t="n"/>
+      <c r="CQ128" s="24" t="n"/>
+      <c r="CR128" s="24" t="n"/>
+      <c r="CS128" s="24" t="n"/>
+      <c r="CT128" s="24" t="n"/>
+      <c r="CU128" s="24" t="n"/>
+      <c r="CV128" s="24" t="n"/>
+      <c r="CW128" s="24" t="n"/>
+      <c r="CX128" s="24" t="n"/>
+      <c r="CY128" s="24" t="n"/>
+      <c r="CZ128" s="24" t="n"/>
+      <c r="DA128" s="24" t="n"/>
+      <c r="DB128" s="24" t="n"/>
+      <c r="DC128" s="24" t="n"/>
+      <c r="DD128" s="24" t="n"/>
+      <c r="DE128" s="24" t="n"/>
+      <c r="DF128" s="24" t="n"/>
+      <c r="DG128" s="24" t="n"/>
+      <c r="DH128" s="24" t="n"/>
+      <c r="DI128" s="24" t="n"/>
+      <c r="DJ128" s="24" t="n"/>
+      <c r="DK128" s="24" t="n"/>
+      <c r="DL128" s="24" t="n"/>
+      <c r="DM128" s="24" t="n"/>
+      <c r="DN128" s="24" t="n"/>
+      <c r="DO128" s="24" t="n"/>
+      <c r="DP128" s="24" t="n"/>
+    </row>
+    <row r="129" ht="36" customHeight="1">
+      <c r="A129" s="24" t="inlineStr">
+        <is>
+          <t>cea26d7eb68f4fce</t>
+        </is>
+      </c>
+      <c r="B129" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:40:57.703355Z</t>
+        </is>
+      </c>
+      <c r="C129" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T23:00Z</t>
+        </is>
+      </c>
+      <c r="D129" s="24" t="inlineStr">
+        <is>
+          <t>aec-atp-valvac-fratia-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E129" s="24" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+      <c r="F129" s="24" t="inlineStr">
+        <is>
+          <t>Frances Tiafoe</t>
+        </is>
+      </c>
+      <c r="G129" s="24" t="inlineStr">
+        <is>
+          <t>Valentin Vacherot</t>
+        </is>
+      </c>
+      <c r="H129" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I129" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J129" s="25" t="n"/>
+      <c r="K129" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L129" s="26" t="n">
+        <v>-186</v>
+      </c>
+      <c r="M129" s="27" t="n">
+        <v>1.5376</v>
+      </c>
+      <c r="N129" s="28" t="n">
+        <v>0.6503</v>
+      </c>
+      <c r="O129" s="28" t="n">
+        <v>0.7187</v>
+      </c>
+      <c r="P129" s="28" t="n"/>
+      <c r="Q129" s="28" t="n">
+        <v>0.0687</v>
+      </c>
+      <c r="R129" s="26" t="n"/>
+      <c r="S129" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T129" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U129" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V129" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W129" s="26" t="n"/>
+      <c r="X129" s="26" t="n"/>
+      <c r="Y129" s="25" t="n"/>
+      <c r="Z129" s="26" t="n"/>
+      <c r="AA129" s="28" t="n"/>
+      <c r="AB129" s="28" t="n"/>
+      <c r="AC129" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD129" s="24" t="n"/>
+      <c r="AE129" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9E02GGBCMVG on aec-atp-valvac-fratia-2026-09-04 (short)</t>
+        </is>
+      </c>
+      <c r="AF129" s="31" t="n"/>
+      <c r="AG129" s="24" t="n"/>
+      <c r="AH129" s="24" t="n"/>
+      <c r="AI129" s="31" t="n"/>
+      <c r="AJ129" s="31" t="n"/>
+      <c r="AK129" s="24" t="n"/>
+      <c r="AL129" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM129" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN129" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO129" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP129" s="24" t="n"/>
+      <c r="AQ129" s="24" t="n"/>
+      <c r="AR129" s="24" t="n"/>
+      <c r="AS129" s="24" t="n"/>
+      <c r="AT129" s="24" t="n"/>
+      <c r="AU129" s="24" t="n"/>
+      <c r="AV129" s="24" t="n"/>
+      <c r="AW129" s="24" t="n"/>
+      <c r="AX129" s="24" t="n"/>
+      <c r="AY129" s="24" t="n"/>
+      <c r="AZ129" s="24" t="n"/>
+      <c r="BA129" s="24" t="n"/>
+      <c r="BB129" s="24" t="n"/>
+      <c r="BC129" s="24" t="n"/>
+      <c r="BD129" s="24" t="n"/>
+      <c r="BE129" s="24" t="n"/>
+      <c r="BF129" s="24" t="n"/>
+      <c r="BG129" s="24" t="n"/>
+      <c r="BH129" s="24" t="n"/>
+      <c r="BI129" s="24" t="n"/>
+      <c r="BJ129" s="25" t="n"/>
+      <c r="BK129" s="26" t="n"/>
+      <c r="BL129" s="27" t="n"/>
+      <c r="BM129" s="28" t="n"/>
+      <c r="BN129" s="28" t="n"/>
+      <c r="BO129" s="28" t="n"/>
+      <c r="BP129" s="25" t="n"/>
+      <c r="BQ129" s="27" t="n"/>
+      <c r="BR129" s="28" t="n"/>
+      <c r="BS129" s="28" t="n"/>
+      <c r="BT129" s="28" t="n"/>
+      <c r="BU129" s="25" t="n"/>
+      <c r="BV129" s="29" t="n"/>
+      <c r="BW129" s="24" t="n"/>
+      <c r="BX129" s="30" t="n"/>
+      <c r="BY129" s="27" t="n"/>
+      <c r="BZ129" s="24" t="n"/>
+      <c r="CA129" s="31" t="n"/>
+      <c r="CB129" s="24" t="n"/>
+      <c r="CC129" s="24" t="n"/>
+      <c r="CD129" s="24" t="n"/>
+      <c r="CE129" s="24" t="n"/>
+      <c r="CF129" s="24" t="n"/>
+      <c r="CG129" s="24" t="n"/>
+      <c r="CH129" s="24" t="n"/>
+      <c r="CI129" s="24" t="n"/>
+      <c r="CJ129" s="24" t="n"/>
+      <c r="CK129" s="24" t="n"/>
+      <c r="CL129" s="24" t="n"/>
+      <c r="CM129" s="24" t="n"/>
+      <c r="CN129" s="24" t="n"/>
+      <c r="CO129" s="24" t="n"/>
+      <c r="CP129" s="24" t="n"/>
+      <c r="CQ129" s="24" t="n"/>
+      <c r="CR129" s="24" t="n"/>
+      <c r="CS129" s="24" t="n"/>
+      <c r="CT129" s="24" t="n"/>
+      <c r="CU129" s="24" t="n"/>
+      <c r="CV129" s="24" t="n"/>
+      <c r="CW129" s="24" t="n"/>
+      <c r="CX129" s="24" t="n"/>
+      <c r="CY129" s="24" t="n"/>
+      <c r="CZ129" s="24" t="n"/>
+      <c r="DA129" s="24" t="n"/>
+      <c r="DB129" s="24" t="n"/>
+      <c r="DC129" s="24" t="n"/>
+      <c r="DD129" s="24" t="n"/>
+      <c r="DE129" s="24" t="n"/>
+      <c r="DF129" s="24" t="n"/>
+      <c r="DG129" s="24" t="n"/>
+      <c r="DH129" s="24" t="n"/>
+      <c r="DI129" s="24" t="n"/>
+      <c r="DJ129" s="24" t="n"/>
+      <c r="DK129" s="24" t="n"/>
+      <c r="DL129" s="24" t="n"/>
+      <c r="DM129" s="24" t="n"/>
+      <c r="DN129" s="24" t="n"/>
+      <c r="DO129" s="24" t="n"/>
+      <c r="DP129" s="24" t="n"/>
+    </row>
+    <row r="130" ht="36" customHeight="1">
+      <c r="A130" s="24" t="inlineStr">
+        <is>
+          <t>dfd31228e10a49bc</t>
+        </is>
+      </c>
+      <c r="B130" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:40:57.703355Z</t>
+        </is>
+      </c>
+      <c r="C130" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D130" s="24" t="inlineStr">
+        <is>
+          <t>aec-lol-doc-lds-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E130" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F130" s="24" t="inlineStr">
+        <is>
+          <t>Lodis</t>
+        </is>
+      </c>
+      <c r="G130" s="24" t="inlineStr">
+        <is>
+          <t>DOCISK</t>
+        </is>
+      </c>
+      <c r="H130" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I130" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J130" s="25" t="n"/>
+      <c r="K130" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L130" s="26" t="n">
+        <v>203</v>
+      </c>
+      <c r="M130" s="27" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="N130" s="28" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="O130" s="28" t="n">
+        <v>0.5829</v>
+      </c>
+      <c r="P130" s="28" t="n"/>
+      <c r="Q130" s="28" t="n">
+        <v>0.2529</v>
+      </c>
+      <c r="R130" s="26" t="n"/>
+      <c r="S130" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T130" s="24" t="inlineStr">
+        <is>
+          <t>lol-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U130" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V130" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W130" s="26" t="n"/>
+      <c r="X130" s="26" t="n"/>
+      <c r="Y130" s="25" t="n"/>
+      <c r="Z130" s="26" t="n"/>
+      <c r="AA130" s="28" t="n"/>
+      <c r="AB130" s="28" t="n"/>
+      <c r="AC130" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD130" s="24" t="n"/>
+      <c r="AE130" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9DZ3TX0AMW1 on aec-lol-doc-lds-2026-09-04 (long)</t>
+        </is>
+      </c>
+      <c r="AF130" s="31" t="n"/>
+      <c r="AG130" s="24" t="n"/>
+      <c r="AH130" s="24" t="n"/>
+      <c r="AI130" s="31" t="n"/>
+      <c r="AJ130" s="31" t="n"/>
+      <c r="AK130" s="24" t="n"/>
+      <c r="AL130" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM130" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN130" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO130" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP130" s="24" t="n"/>
+      <c r="AQ130" s="24" t="n"/>
+      <c r="AR130" s="24" t="n"/>
+      <c r="AS130" s="24" t="n"/>
+      <c r="AT130" s="24" t="n"/>
+      <c r="AU130" s="24" t="n"/>
+      <c r="AV130" s="24" t="n"/>
+      <c r="AW130" s="24" t="n"/>
+      <c r="AX130" s="24" t="n"/>
+      <c r="AY130" s="24" t="n"/>
+      <c r="AZ130" s="24" t="n"/>
+      <c r="BA130" s="24" t="n"/>
+      <c r="BB130" s="24" t="n"/>
+      <c r="BC130" s="24" t="n"/>
+      <c r="BD130" s="24" t="n"/>
+      <c r="BE130" s="24" t="n"/>
+      <c r="BF130" s="24" t="n"/>
+      <c r="BG130" s="24" t="n"/>
+      <c r="BH130" s="24" t="n"/>
+      <c r="BI130" s="24" t="n"/>
+      <c r="BJ130" s="25" t="n"/>
+      <c r="BK130" s="26" t="n"/>
+      <c r="BL130" s="27" t="n"/>
+      <c r="BM130" s="28" t="n"/>
+      <c r="BN130" s="28" t="n"/>
+      <c r="BO130" s="28" t="n"/>
+      <c r="BP130" s="25" t="n"/>
+      <c r="BQ130" s="27" t="n"/>
+      <c r="BR130" s="28" t="n"/>
+      <c r="BS130" s="28" t="n"/>
+      <c r="BT130" s="28" t="n"/>
+      <c r="BU130" s="25" t="n"/>
+      <c r="BV130" s="29" t="n"/>
+      <c r="BW130" s="24" t="n"/>
+      <c r="BX130" s="30" t="n"/>
+      <c r="BY130" s="27" t="n"/>
+      <c r="BZ130" s="24" t="n"/>
+      <c r="CA130" s="31" t="n"/>
+      <c r="CB130" s="24" t="n"/>
+      <c r="CC130" s="24" t="n"/>
+      <c r="CD130" s="24" t="n"/>
+      <c r="CE130" s="24" t="n"/>
+      <c r="CF130" s="24" t="n"/>
+      <c r="CG130" s="24" t="n"/>
+      <c r="CH130" s="24" t="n"/>
+      <c r="CI130" s="24" t="n"/>
+      <c r="CJ130" s="24" t="n"/>
+      <c r="CK130" s="24" t="n"/>
+      <c r="CL130" s="24" t="n"/>
+      <c r="CM130" s="24" t="n"/>
+      <c r="CN130" s="24" t="n"/>
+      <c r="CO130" s="24" t="n"/>
+      <c r="CP130" s="24" t="n"/>
+      <c r="CQ130" s="24" t="n"/>
+      <c r="CR130" s="24" t="n"/>
+      <c r="CS130" s="24" t="n"/>
+      <c r="CT130" s="24" t="n"/>
+      <c r="CU130" s="24" t="n"/>
+      <c r="CV130" s="24" t="n"/>
+      <c r="CW130" s="24" t="n"/>
+      <c r="CX130" s="24" t="n"/>
+      <c r="CY130" s="24" t="n"/>
+      <c r="CZ130" s="24" t="n"/>
+      <c r="DA130" s="24" t="n"/>
+      <c r="DB130" s="24" t="n"/>
+      <c r="DC130" s="24" t="n"/>
+      <c r="DD130" s="24" t="n"/>
+      <c r="DE130" s="24" t="n"/>
+      <c r="DF130" s="24" t="n"/>
+      <c r="DG130" s="24" t="n"/>
+      <c r="DH130" s="24" t="n"/>
+      <c r="DI130" s="24" t="n"/>
+      <c r="DJ130" s="24" t="n"/>
+      <c r="DK130" s="24" t="n"/>
+      <c r="DL130" s="24" t="n"/>
+      <c r="DM130" s="24" t="n"/>
+      <c r="DN130" s="24" t="n"/>
+      <c r="DO130" s="24" t="n"/>
+      <c r="DP130" s="24" t="n"/>
+    </row>
+    <row r="131" ht="36" customHeight="1">
+      <c r="A131" s="24" t="inlineStr">
+        <is>
+          <t>dbdda061ddbd4e3a</t>
+        </is>
+      </c>
+      <c r="B131" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:40:57.703355Z</t>
+        </is>
+      </c>
+      <c r="C131" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T14:00:00Z</t>
+        </is>
+      </c>
+      <c r="D131" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-nemi-bca-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E131" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F131" s="24" t="inlineStr">
+        <is>
+          <t>Betclic Apogee Esports</t>
+        </is>
+      </c>
+      <c r="G131" s="24" t="inlineStr">
+        <is>
+          <t>Nemiga</t>
+        </is>
+      </c>
+      <c r="H131" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I131" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J131" s="25" t="n"/>
+      <c r="K131" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L131" s="26" t="n">
+        <v>-100</v>
+      </c>
+      <c r="M131" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="N131" s="28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O131" s="28" t="n">
+        <v>0.6262</v>
+      </c>
+      <c r="P131" s="28" t="n"/>
+      <c r="Q131" s="28" t="n">
+        <v>0.1262</v>
+      </c>
+      <c r="R131" s="26" t="n"/>
+      <c r="S131" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T131" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U131" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V131" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W131" s="26" t="n"/>
+      <c r="X131" s="26" t="n"/>
+      <c r="Y131" s="25" t="n"/>
+      <c r="Z131" s="26" t="n"/>
+      <c r="AA131" s="28" t="n"/>
+      <c r="AB131" s="28" t="n"/>
+      <c r="AC131" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD131" s="24" t="n"/>
+      <c r="AE131" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9DZEJJPPMVR on aec-cs2-nemi-bca-2026-09-04 (long)</t>
+        </is>
+      </c>
+      <c r="AF131" s="31" t="n"/>
+      <c r="AG131" s="24" t="n"/>
+      <c r="AH131" s="24" t="n"/>
+      <c r="AI131" s="31" t="n"/>
+      <c r="AJ131" s="31" t="n"/>
+      <c r="AK131" s="24" t="n"/>
+      <c r="AL131" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM131" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN131" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO131" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP131" s="24" t="n"/>
+      <c r="AQ131" s="24" t="n"/>
+      <c r="AR131" s="24" t="n"/>
+      <c r="AS131" s="24" t="n"/>
+      <c r="AT131" s="24" t="n"/>
+      <c r="AU131" s="24" t="n"/>
+      <c r="AV131" s="24" t="n"/>
+      <c r="AW131" s="24" t="n"/>
+      <c r="AX131" s="24" t="n"/>
+      <c r="AY131" s="24" t="n"/>
+      <c r="AZ131" s="24" t="n"/>
+      <c r="BA131" s="24" t="n"/>
+      <c r="BB131" s="24" t="n"/>
+      <c r="BC131" s="24" t="n"/>
+      <c r="BD131" s="24" t="n"/>
+      <c r="BE131" s="24" t="n"/>
+      <c r="BF131" s="24" t="n"/>
+      <c r="BG131" s="24" t="n"/>
+      <c r="BH131" s="24" t="n"/>
+      <c r="BI131" s="24" t="n"/>
+      <c r="BJ131" s="25" t="n"/>
+      <c r="BK131" s="26" t="n"/>
+      <c r="BL131" s="27" t="n"/>
+      <c r="BM131" s="28" t="n"/>
+      <c r="BN131" s="28" t="n"/>
+      <c r="BO131" s="28" t="n"/>
+      <c r="BP131" s="25" t="n"/>
+      <c r="BQ131" s="27" t="n"/>
+      <c r="BR131" s="28" t="n"/>
+      <c r="BS131" s="28" t="n"/>
+      <c r="BT131" s="28" t="n"/>
+      <c r="BU131" s="25" t="n"/>
+      <c r="BV131" s="29" t="n"/>
+      <c r="BW131" s="24" t="n"/>
+      <c r="BX131" s="30" t="n"/>
+      <c r="BY131" s="27" t="n"/>
+      <c r="BZ131" s="24" t="n"/>
+      <c r="CA131" s="31" t="n"/>
+      <c r="CB131" s="24" t="n"/>
+      <c r="CC131" s="24" t="n"/>
+      <c r="CD131" s="24" t="n"/>
+      <c r="CE131" s="24" t="n"/>
+      <c r="CF131" s="24" t="n"/>
+      <c r="CG131" s="24" t="n"/>
+      <c r="CH131" s="24" t="n"/>
+      <c r="CI131" s="24" t="n"/>
+      <c r="CJ131" s="24" t="n"/>
+      <c r="CK131" s="24" t="n"/>
+      <c r="CL131" s="24" t="n"/>
+      <c r="CM131" s="24" t="n"/>
+      <c r="CN131" s="24" t="n"/>
+      <c r="CO131" s="24" t="n"/>
+      <c r="CP131" s="24" t="n"/>
+      <c r="CQ131" s="24" t="n"/>
+      <c r="CR131" s="24" t="n"/>
+      <c r="CS131" s="24" t="n"/>
+      <c r="CT131" s="24" t="n"/>
+      <c r="CU131" s="24" t="n"/>
+      <c r="CV131" s="24" t="n"/>
+      <c r="CW131" s="24" t="n"/>
+      <c r="CX131" s="24" t="n"/>
+      <c r="CY131" s="24" t="n"/>
+      <c r="CZ131" s="24" t="n"/>
+      <c r="DA131" s="24" t="n"/>
+      <c r="DB131" s="24" t="n"/>
+      <c r="DC131" s="24" t="n"/>
+      <c r="DD131" s="24" t="n"/>
+      <c r="DE131" s="24" t="n"/>
+      <c r="DF131" s="24" t="n"/>
+      <c r="DG131" s="24" t="n"/>
+      <c r="DH131" s="24" t="n"/>
+      <c r="DI131" s="24" t="n"/>
+      <c r="DJ131" s="24" t="n"/>
+      <c r="DK131" s="24" t="n"/>
+      <c r="DL131" s="24" t="n"/>
+      <c r="DM131" s="24" t="n"/>
+      <c r="DN131" s="24" t="n"/>
+      <c r="DO131" s="24" t="n"/>
+      <c r="DP131" s="24" t="n"/>
+    </row>
+    <row r="132" ht="36" customHeight="1">
+      <c r="A132" s="24" t="inlineStr">
+        <is>
+          <t>f4aeecd9aa98413d</t>
+        </is>
+      </c>
+      <c r="B132" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:40:57.703355Z</t>
+        </is>
+      </c>
+      <c r="C132" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D132" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-sin-qua-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E132" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F132" s="24" t="inlineStr">
+        <is>
+          <t>QUAZAR</t>
+        </is>
+      </c>
+      <c r="G132" s="24" t="inlineStr">
+        <is>
+          <t>Sinners</t>
+        </is>
+      </c>
+      <c r="H132" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I132" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J132" s="25" t="n"/>
+      <c r="K132" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L132" s="26" t="n">
+        <v>186</v>
+      </c>
+      <c r="M132" s="27" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="N132" s="28" t="n">
+        <v>0.3497</v>
+      </c>
+      <c r="O132" s="28" t="n">
+        <v>0.5237000000000001</v>
+      </c>
+      <c r="P132" s="28" t="n"/>
+      <c r="Q132" s="28" t="n">
+        <v>0.1737</v>
+      </c>
+      <c r="R132" s="26" t="n"/>
+      <c r="S132" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T132" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U132" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V132" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W132" s="26" t="n"/>
+      <c r="X132" s="26" t="n"/>
+      <c r="Y132" s="25" t="n"/>
+      <c r="Z132" s="26" t="n"/>
+      <c r="AA132" s="28" t="n"/>
+      <c r="AB132" s="28" t="n"/>
+      <c r="AC132" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD132" s="24" t="n"/>
+      <c r="AE132" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9DZNP1G6MVV on aec-cs2-sin-qua-2026-09-04 (short)</t>
+        </is>
+      </c>
+      <c r="AF132" s="31" t="n"/>
+      <c r="AG132" s="24" t="n"/>
+      <c r="AH132" s="24" t="n"/>
+      <c r="AI132" s="31" t="n"/>
+      <c r="AJ132" s="31" t="n"/>
+      <c r="AK132" s="24" t="n"/>
+      <c r="AL132" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM132" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN132" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO132" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP132" s="24" t="n"/>
+      <c r="AQ132" s="24" t="n"/>
+      <c r="AR132" s="24" t="n"/>
+      <c r="AS132" s="24" t="n"/>
+      <c r="AT132" s="24" t="n"/>
+      <c r="AU132" s="24" t="n"/>
+      <c r="AV132" s="24" t="n"/>
+      <c r="AW132" s="24" t="n"/>
+      <c r="AX132" s="24" t="n"/>
+      <c r="AY132" s="24" t="n"/>
+      <c r="AZ132" s="24" t="n"/>
+      <c r="BA132" s="24" t="n"/>
+      <c r="BB132" s="24" t="n"/>
+      <c r="BC132" s="24" t="n"/>
+      <c r="BD132" s="24" t="n"/>
+      <c r="BE132" s="24" t="n"/>
+      <c r="BF132" s="24" t="n"/>
+      <c r="BG132" s="24" t="n"/>
+      <c r="BH132" s="24" t="n"/>
+      <c r="BI132" s="24" t="n"/>
+      <c r="BJ132" s="25" t="n"/>
+      <c r="BK132" s="26" t="n"/>
+      <c r="BL132" s="27" t="n"/>
+      <c r="BM132" s="28" t="n"/>
+      <c r="BN132" s="28" t="n"/>
+      <c r="BO132" s="28" t="n"/>
+      <c r="BP132" s="25" t="n"/>
+      <c r="BQ132" s="27" t="n"/>
+      <c r="BR132" s="28" t="n"/>
+      <c r="BS132" s="28" t="n"/>
+      <c r="BT132" s="28" t="n"/>
+      <c r="BU132" s="25" t="n"/>
+      <c r="BV132" s="29" t="n"/>
+      <c r="BW132" s="24" t="n"/>
+      <c r="BX132" s="30" t="n"/>
+      <c r="BY132" s="27" t="n"/>
+      <c r="BZ132" s="24" t="n"/>
+      <c r="CA132" s="31" t="n"/>
+      <c r="CB132" s="24" t="n"/>
+      <c r="CC132" s="24" t="n"/>
+      <c r="CD132" s="24" t="n"/>
+      <c r="CE132" s="24" t="n"/>
+      <c r="CF132" s="24" t="n"/>
+      <c r="CG132" s="24" t="n"/>
+      <c r="CH132" s="24" t="n"/>
+      <c r="CI132" s="24" t="n"/>
+      <c r="CJ132" s="24" t="n"/>
+      <c r="CK132" s="24" t="n"/>
+      <c r="CL132" s="24" t="n"/>
+      <c r="CM132" s="24" t="n"/>
+      <c r="CN132" s="24" t="n"/>
+      <c r="CO132" s="24" t="n"/>
+      <c r="CP132" s="24" t="n"/>
+      <c r="CQ132" s="24" t="n"/>
+      <c r="CR132" s="24" t="n"/>
+      <c r="CS132" s="24" t="n"/>
+      <c r="CT132" s="24" t="n"/>
+      <c r="CU132" s="24" t="n"/>
+      <c r="CV132" s="24" t="n"/>
+      <c r="CW132" s="24" t="n"/>
+      <c r="CX132" s="24" t="n"/>
+      <c r="CY132" s="24" t="n"/>
+      <c r="CZ132" s="24" t="n"/>
+      <c r="DA132" s="24" t="n"/>
+      <c r="DB132" s="24" t="n"/>
+      <c r="DC132" s="24" t="n"/>
+      <c r="DD132" s="24" t="n"/>
+      <c r="DE132" s="24" t="n"/>
+      <c r="DF132" s="24" t="n"/>
+      <c r="DG132" s="24" t="n"/>
+      <c r="DH132" s="24" t="n"/>
+      <c r="DI132" s="24" t="n"/>
+      <c r="DJ132" s="24" t="n"/>
+      <c r="DK132" s="24" t="n"/>
+      <c r="DL132" s="24" t="n"/>
+      <c r="DM132" s="24" t="n"/>
+      <c r="DN132" s="24" t="n"/>
+      <c r="DO132" s="24" t="n"/>
+      <c r="DP132" s="24" t="n"/>
+    </row>
+    <row r="133" ht="36" customHeight="1">
+      <c r="A133" s="24" t="inlineStr">
+        <is>
+          <t>73d88d492cd0402f</t>
+        </is>
+      </c>
+      <c r="B133" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T04:40:57.703355Z</t>
+        </is>
+      </c>
+      <c r="C133" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-05T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="D133" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-mars-war-2026-09-05</t>
+        </is>
+      </c>
+      <c r="E133" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F133" s="24" t="inlineStr">
+        <is>
+          <t>Without a Roof</t>
+        </is>
+      </c>
+      <c r="G133" s="24" t="inlineStr">
+        <is>
+          <t>Marsborne</t>
+        </is>
+      </c>
+      <c r="H133" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I133" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J133" s="25" t="n"/>
+      <c r="K133" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L133" s="26" t="n">
+        <v>-122</v>
+      </c>
+      <c r="M133" s="27" t="n">
+        <v>1.8197</v>
+      </c>
+      <c r="N133" s="28" t="n">
+        <v>0.5495</v>
+      </c>
+      <c r="O133" s="28" t="n">
+        <v>0.6298</v>
+      </c>
+      <c r="P133" s="28" t="n"/>
+      <c r="Q133" s="28" t="n">
+        <v>0.0798</v>
+      </c>
+      <c r="R133" s="26" t="n"/>
+      <c r="S133" s="29" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T133" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U133" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V133" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W133" s="26" t="n"/>
+      <c r="X133" s="26" t="n"/>
+      <c r="Y133" s="25" t="n"/>
+      <c r="Z133" s="26" t="n"/>
+      <c r="AA133" s="28" t="n"/>
+      <c r="AB133" s="28" t="n"/>
+      <c r="AC133" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD133" s="24" t="n"/>
+      <c r="AE133" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9DZWAQW4MVK on aec-cs2-mars-war-2026-09-05 (long)</t>
+        </is>
+      </c>
+      <c r="AF133" s="31" t="n"/>
+      <c r="AG133" s="24" t="n"/>
+      <c r="AH133" s="24" t="n"/>
+      <c r="AI133" s="31" t="n"/>
+      <c r="AJ133" s="31" t="n"/>
+      <c r="AK133" s="24" t="n"/>
+      <c r="AL133" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM133" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN133" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO133" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP133" s="24" t="n"/>
+      <c r="AQ133" s="24" t="n"/>
+      <c r="AR133" s="24" t="n"/>
+      <c r="AS133" s="24" t="n"/>
+      <c r="AT133" s="24" t="n"/>
+      <c r="AU133" s="24" t="n"/>
+      <c r="AV133" s="24" t="n"/>
+      <c r="AW133" s="24" t="n"/>
+      <c r="AX133" s="24" t="n"/>
+      <c r="AY133" s="24" t="n"/>
+      <c r="AZ133" s="24" t="n"/>
+      <c r="BA133" s="24" t="n"/>
+      <c r="BB133" s="24" t="n"/>
+      <c r="BC133" s="24" t="n"/>
+      <c r="BD133" s="24" t="n"/>
+      <c r="BE133" s="24" t="n"/>
+      <c r="BF133" s="24" t="n"/>
+      <c r="BG133" s="24" t="n"/>
+      <c r="BH133" s="24" t="n"/>
+      <c r="BI133" s="24" t="n"/>
+      <c r="BJ133" s="25" t="n"/>
+      <c r="BK133" s="26" t="n"/>
+      <c r="BL133" s="27" t="n"/>
+      <c r="BM133" s="28" t="n"/>
+      <c r="BN133" s="28" t="n"/>
+      <c r="BO133" s="28" t="n"/>
+      <c r="BP133" s="25" t="n"/>
+      <c r="BQ133" s="27" t="n"/>
+      <c r="BR133" s="28" t="n"/>
+      <c r="BS133" s="28" t="n"/>
+      <c r="BT133" s="28" t="n"/>
+      <c r="BU133" s="25" t="n"/>
+      <c r="BV133" s="29" t="n"/>
+      <c r="BW133" s="24" t="n"/>
+      <c r="BX133" s="30" t="n"/>
+      <c r="BY133" s="27" t="n"/>
+      <c r="BZ133" s="24" t="n"/>
+      <c r="CA133" s="31" t="n"/>
+      <c r="CB133" s="24" t="n"/>
+      <c r="CC133" s="24" t="n"/>
+      <c r="CD133" s="24" t="n"/>
+      <c r="CE133" s="24" t="n"/>
+      <c r="CF133" s="24" t="n"/>
+      <c r="CG133" s="24" t="n"/>
+      <c r="CH133" s="24" t="n"/>
+      <c r="CI133" s="24" t="n"/>
+      <c r="CJ133" s="24" t="n"/>
+      <c r="CK133" s="24" t="n"/>
+      <c r="CL133" s="24" t="n"/>
+      <c r="CM133" s="24" t="n"/>
+      <c r="CN133" s="24" t="n"/>
+      <c r="CO133" s="24" t="n"/>
+      <c r="CP133" s="24" t="n"/>
+      <c r="CQ133" s="24" t="n"/>
+      <c r="CR133" s="24" t="n"/>
+      <c r="CS133" s="24" t="n"/>
+      <c r="CT133" s="24" t="n"/>
+      <c r="CU133" s="24" t="n"/>
+      <c r="CV133" s="24" t="n"/>
+      <c r="CW133" s="24" t="n"/>
+      <c r="CX133" s="24" t="n"/>
+      <c r="CY133" s="24" t="n"/>
+      <c r="CZ133" s="24" t="n"/>
+      <c r="DA133" s="24" t="n"/>
+      <c r="DB133" s="24" t="n"/>
+      <c r="DC133" s="24" t="n"/>
+      <c r="DD133" s="24" t="n"/>
+      <c r="DE133" s="24" t="n"/>
+      <c r="DF133" s="24" t="n"/>
+      <c r="DG133" s="24" t="n"/>
+      <c r="DH133" s="24" t="n"/>
+      <c r="DI133" s="24" t="n"/>
+      <c r="DJ133" s="24" t="n"/>
+      <c r="DK133" s="24" t="n"/>
+      <c r="DL133" s="24" t="n"/>
+      <c r="DM133" s="24" t="n"/>
+      <c r="DN133" s="24" t="n"/>
+      <c r="DO133" s="24" t="n"/>
+      <c r="DP133" s="24" t="n"/>
+    </row>
+    <row r="134" ht="36" customHeight="1">
+      <c r="A134" s="24" t="inlineStr">
+        <is>
+          <t>90fd42882b864418</t>
+        </is>
+      </c>
+      <c r="B134" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T06:11:53.656768Z</t>
+        </is>
+      </c>
+      <c r="C134" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T14:00:00Z</t>
+        </is>
+      </c>
+      <c r="D134" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-jjh-33-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E134" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F134" s="24" t="inlineStr">
+        <is>
+          <t>BET-M 33</t>
+        </is>
+      </c>
+      <c r="G134" s="24" t="inlineStr">
+        <is>
+          <t>JiJieHao</t>
+        </is>
+      </c>
+      <c r="H134" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I134" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J134" s="25" t="n"/>
+      <c r="K134" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L134" s="26" t="n">
+        <v>-127</v>
+      </c>
+      <c r="M134" s="27" t="n">
+        <v>1.7874</v>
+      </c>
+      <c r="N134" s="28" t="n">
+        <v>0.6403</v>
+      </c>
+      <c r="O134" s="28" t="n">
+        <v>0.6309</v>
+      </c>
+      <c r="P134" s="28" t="n"/>
+      <c r="Q134" s="28" t="n">
+        <v>0.0709</v>
+      </c>
+      <c r="R134" s="26" t="n"/>
+      <c r="S134" s="29" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="T134" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U134" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V134" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W134" s="26" t="n"/>
+      <c r="X134" s="26" t="n"/>
+      <c r="Y134" s="25" t="n"/>
+      <c r="Z134" s="26" t="n"/>
+      <c r="AA134" s="28" t="n"/>
+      <c r="AB134" s="28" t="n"/>
+      <c r="AC134" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD134" s="24" t="n"/>
+      <c r="AE134" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9F8KB5WCMVG on aec-cs2-jjh-33-2026-09-04 (long)</t>
+        </is>
+      </c>
+      <c r="AF134" s="31" t="n"/>
+      <c r="AG134" s="24" t="n"/>
+      <c r="AH134" s="24" t="n"/>
+      <c r="AI134" s="31" t="n"/>
+      <c r="AJ134" s="31" t="n"/>
+      <c r="AK134" s="24" t="n"/>
+      <c r="AL134" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM134" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN134" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO134" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP134" s="24" t="n"/>
+      <c r="AQ134" s="24" t="n"/>
+      <c r="AR134" s="24" t="n"/>
+      <c r="AS134" s="24" t="n"/>
+      <c r="AT134" s="24" t="n"/>
+      <c r="AU134" s="24" t="n"/>
+      <c r="AV134" s="24" t="n"/>
+      <c r="AW134" s="24" t="n"/>
+      <c r="AX134" s="24" t="n"/>
+      <c r="AY134" s="24" t="n"/>
+      <c r="AZ134" s="24" t="n"/>
+      <c r="BA134" s="24" t="n"/>
+      <c r="BB134" s="24" t="n"/>
+      <c r="BC134" s="24" t="n"/>
+      <c r="BD134" s="24" t="n"/>
+      <c r="BE134" s="24" t="n"/>
+      <c r="BF134" s="24" t="n"/>
+      <c r="BG134" s="24" t="n"/>
+      <c r="BH134" s="24" t="n"/>
+      <c r="BI134" s="24" t="n"/>
+      <c r="BJ134" s="25" t="n"/>
+      <c r="BK134" s="26" t="n"/>
+      <c r="BL134" s="27" t="n"/>
+      <c r="BM134" s="28" t="n"/>
+      <c r="BN134" s="28" t="n"/>
+      <c r="BO134" s="28" t="n"/>
+      <c r="BP134" s="25" t="n"/>
+      <c r="BQ134" s="27" t="n"/>
+      <c r="BR134" s="28" t="n"/>
+      <c r="BS134" s="28" t="n"/>
+      <c r="BT134" s="28" t="n"/>
+      <c r="BU134" s="25" t="n"/>
+      <c r="BV134" s="29" t="n"/>
+      <c r="BW134" s="24" t="n"/>
+      <c r="BX134" s="30" t="n"/>
+      <c r="BY134" s="27" t="n"/>
+      <c r="BZ134" s="24" t="n"/>
+      <c r="CA134" s="31" t="n"/>
+      <c r="CB134" s="24" t="n"/>
+      <c r="CC134" s="24" t="n"/>
+      <c r="CD134" s="24" t="n"/>
+      <c r="CE134" s="24" t="n"/>
+      <c r="CF134" s="24" t="n"/>
+      <c r="CG134" s="24" t="n"/>
+      <c r="CH134" s="24" t="n"/>
+      <c r="CI134" s="24" t="n"/>
+      <c r="CJ134" s="24" t="n"/>
+      <c r="CK134" s="24" t="n"/>
+      <c r="CL134" s="24" t="n"/>
+      <c r="CM134" s="24" t="n"/>
+      <c r="CN134" s="24" t="n"/>
+      <c r="CO134" s="24" t="n"/>
+      <c r="CP134" s="24" t="n"/>
+      <c r="CQ134" s="24" t="n"/>
+      <c r="CR134" s="24" t="n"/>
+      <c r="CS134" s="24" t="n"/>
+      <c r="CT134" s="24" t="n"/>
+      <c r="CU134" s="24" t="n"/>
+      <c r="CV134" s="24" t="n"/>
+      <c r="CW134" s="24" t="n"/>
+      <c r="CX134" s="24" t="n"/>
+      <c r="CY134" s="24" t="n"/>
+      <c r="CZ134" s="24" t="n"/>
+      <c r="DA134" s="24" t="n"/>
+      <c r="DB134" s="24" t="n"/>
+      <c r="DC134" s="24" t="n"/>
+      <c r="DD134" s="24" t="n"/>
+      <c r="DE134" s="24" t="n"/>
+      <c r="DF134" s="24" t="n"/>
+      <c r="DG134" s="24" t="n"/>
+      <c r="DH134" s="24" t="n"/>
+      <c r="DI134" s="24" t="n"/>
+      <c r="DJ134" s="24" t="n"/>
+      <c r="DK134" s="24" t="n"/>
+      <c r="DL134" s="24" t="n"/>
+      <c r="DM134" s="24" t="n"/>
+      <c r="DN134" s="24" t="n"/>
+      <c r="DO134" s="24" t="n"/>
+      <c r="DP134" s="24" t="n"/>
+    </row>
+    <row r="135" ht="36" customHeight="1">
+      <c r="A135" s="24" t="inlineStr">
+        <is>
+          <t>7249021be14e4de5</t>
+        </is>
+      </c>
+      <c r="B135" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="C135" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T20:00:00Z</t>
+        </is>
+      </c>
+      <c r="D135" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-omg-qua-2026-09-03</t>
+        </is>
+      </c>
+      <c r="E135" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F135" s="24" t="inlineStr">
+        <is>
+          <t>QUAZAR</t>
+        </is>
+      </c>
+      <c r="G135" s="24" t="inlineStr">
+        <is>
+          <t>OMG</t>
+        </is>
+      </c>
+      <c r="H135" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I135" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J135" s="25" t="n"/>
+      <c r="K135" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L135" s="26" t="n">
+        <v>-127</v>
+      </c>
+      <c r="M135" s="27" t="n">
+        <v>1.7874</v>
+      </c>
+      <c r="N135" s="28" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="O135" s="28" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="P135" s="28" t="n"/>
+      <c r="Q135" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R135" s="26" t="n"/>
+      <c r="S135" s="29" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="T135" s="24" t="inlineStr">
+        <is>
+          <t>cs2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U135" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V135" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W135" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X135" s="26" t="n"/>
+      <c r="Y135" s="25" t="n"/>
+      <c r="Z135" s="26" t="n"/>
+      <c r="AA135" s="28" t="n"/>
+      <c r="AB135" s="28" t="n"/>
+      <c r="AC135" s="30" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AD135" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-03T22:00:00Z</t>
+        </is>
+      </c>
+      <c r="AE135" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C8VMRB4Y8MVK on aec-cs2-omg-qua-2026-09-03 (short)</t>
+        </is>
+      </c>
+      <c r="AF135" s="31" t="n"/>
+      <c r="AG135" s="24" t="n"/>
+      <c r="AH135" s="24" t="n"/>
+      <c r="AI135" s="31" t="n"/>
+      <c r="AJ135" s="31" t="n"/>
+      <c r="AK135" s="24" t="n"/>
+      <c r="AL135" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM135" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN135" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO135" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP135" s="24" t="n"/>
+      <c r="AQ135" s="24" t="n"/>
+      <c r="AR135" s="24" t="n"/>
+      <c r="AS135" s="24" t="n"/>
+      <c r="AT135" s="24" t="n"/>
+      <c r="AU135" s="24" t="n"/>
+      <c r="AV135" s="24" t="n"/>
+      <c r="AW135" s="24" t="n"/>
+      <c r="AX135" s="24" t="n"/>
+      <c r="AY135" s="24" t="n"/>
+      <c r="AZ135" s="24" t="n"/>
+      <c r="BA135" s="24" t="n"/>
+      <c r="BB135" s="24" t="n"/>
+      <c r="BC135" s="24" t="n"/>
+      <c r="BD135" s="24" t="n"/>
+      <c r="BE135" s="24" t="n"/>
+      <c r="BF135" s="24" t="n"/>
+      <c r="BG135" s="24" t="n"/>
+      <c r="BH135" s="24" t="n"/>
+      <c r="BI135" s="24" t="n"/>
+      <c r="BJ135" s="25" t="n"/>
+      <c r="BK135" s="26" t="n"/>
+      <c r="BL135" s="27" t="n"/>
+      <c r="BM135" s="28" t="n"/>
+      <c r="BN135" s="28" t="n"/>
+      <c r="BO135" s="28" t="n"/>
+      <c r="BP135" s="25" t="n"/>
+      <c r="BQ135" s="27" t="n"/>
+      <c r="BR135" s="28" t="n"/>
+      <c r="BS135" s="28" t="n"/>
+      <c r="BT135" s="28" t="n"/>
+      <c r="BU135" s="25" t="n"/>
+      <c r="BV135" s="29" t="n"/>
+      <c r="BW135" s="24" t="n"/>
+      <c r="BX135" s="30" t="n"/>
+      <c r="BY135" s="27" t="n"/>
+      <c r="BZ135" s="24" t="n"/>
+      <c r="CA135" s="31" t="n"/>
+      <c r="CB135" s="24" t="n"/>
+      <c r="CC135" s="24" t="n"/>
+      <c r="CD135" s="24" t="n"/>
+      <c r="CE135" s="24" t="n"/>
+      <c r="CF135" s="24" t="n"/>
+      <c r="CG135" s="24" t="n"/>
+      <c r="CH135" s="24" t="n"/>
+      <c r="CI135" s="24" t="n"/>
+      <c r="CJ135" s="24" t="n"/>
+      <c r="CK135" s="24" t="n"/>
+      <c r="CL135" s="24" t="n"/>
+      <c r="CM135" s="24" t="n"/>
+      <c r="CN135" s="24" t="n"/>
+      <c r="CO135" s="24" t="n"/>
+      <c r="CP135" s="24" t="n"/>
+      <c r="CQ135" s="24" t="n"/>
+      <c r="CR135" s="24" t="n"/>
+      <c r="CS135" s="24" t="n"/>
+      <c r="CT135" s="24" t="n"/>
+      <c r="CU135" s="24" t="n"/>
+      <c r="CV135" s="24" t="n"/>
+      <c r="CW135" s="24" t="n"/>
+      <c r="CX135" s="24" t="n"/>
+      <c r="CY135" s="24" t="n"/>
+      <c r="CZ135" s="24" t="n"/>
+      <c r="DA135" s="24" t="n"/>
+      <c r="DB135" s="24" t="n"/>
+      <c r="DC135" s="24" t="n"/>
+      <c r="DD135" s="24" t="n"/>
+      <c r="DE135" s="24" t="n"/>
+      <c r="DF135" s="24" t="n"/>
+      <c r="DG135" s="24" t="n"/>
+      <c r="DH135" s="24" t="n"/>
+      <c r="DI135" s="24" t="n"/>
+      <c r="DJ135" s="24" t="n"/>
+      <c r="DK135" s="24" t="n"/>
+      <c r="DL135" s="24" t="n"/>
+      <c r="DM135" s="24" t="n"/>
+      <c r="DN135" s="24" t="n"/>
+      <c r="DO135" s="24" t="n"/>
+      <c r="DP135" s="24" t="n"/>
+    </row>
+    <row r="136" ht="36" customHeight="1">
+      <c r="A136" s="24" t="inlineStr">
+        <is>
+          <t>2c8d598d287246b3</t>
+        </is>
+      </c>
+      <c r="B136" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T07:17:52.157470Z</t>
+        </is>
+      </c>
+      <c r="C136" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T19:00Z</t>
+        </is>
+      </c>
+      <c r="D136" s="24" t="inlineStr">
+        <is>
+          <t>atc-epl-ips-liv-2026-09-04-ips</t>
+        </is>
+      </c>
+      <c r="E136" s="24" t="inlineStr">
+        <is>
+          <t>SOCCER</t>
+        </is>
+      </c>
+      <c r="F136" s="24" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="G136" s="24" t="inlineStr">
+        <is>
+          <t>Ipswich Town</t>
+        </is>
+      </c>
+      <c r="H136" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I136" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J136" s="25" t="n"/>
+      <c r="K136" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L136" s="26" t="n">
+        <v>525</v>
+      </c>
+      <c r="M136" s="27" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="N136" s="28" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="O136" s="28" t="n">
+        <v>0.5514</v>
+      </c>
+      <c r="P136" s="28" t="n"/>
+      <c r="Q136" s="28" t="n">
+        <v>0.3914</v>
+      </c>
+      <c r="R136" s="26" t="n"/>
+      <c r="S136" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T136" s="24" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="U136" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V136" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W136" s="26" t="n"/>
+      <c r="X136" s="26" t="n"/>
+      <c r="Y136" s="25" t="n"/>
+      <c r="Z136" s="26" t="n"/>
+      <c r="AA136" s="28" t="n"/>
+      <c r="AB136" s="28" t="n"/>
+      <c r="AC136" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD136" s="24" t="n"/>
+      <c r="AE136" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9G5E3E0GMVV on atc-epl-ips-liv-2026-09-04-ips (long)</t>
+        </is>
+      </c>
+      <c r="AF136" s="31" t="n"/>
+      <c r="AG136" s="24" t="n"/>
+      <c r="AH136" s="24" t="n"/>
+      <c r="AI136" s="31" t="n"/>
+      <c r="AJ136" s="31" t="n"/>
+      <c r="AK136" s="24" t="n"/>
+      <c r="AL136" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM136" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN136" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO136" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP136" s="24" t="n"/>
+      <c r="AQ136" s="24" t="n"/>
+      <c r="AR136" s="24" t="n"/>
+      <c r="AS136" s="24" t="n"/>
+      <c r="AT136" s="24" t="n"/>
+      <c r="AU136" s="24" t="n"/>
+      <c r="AV136" s="24" t="n"/>
+      <c r="AW136" s="24" t="n"/>
+      <c r="AX136" s="24" t="n"/>
+      <c r="AY136" s="24" t="n"/>
+      <c r="AZ136" s="24" t="n"/>
+      <c r="BA136" s="24" t="n"/>
+      <c r="BB136" s="24" t="n"/>
+      <c r="BC136" s="24" t="n"/>
+      <c r="BD136" s="24" t="n"/>
+      <c r="BE136" s="24" t="n"/>
+      <c r="BF136" s="24" t="n"/>
+      <c r="BG136" s="24" t="n"/>
+      <c r="BH136" s="24" t="n"/>
+      <c r="BI136" s="24" t="n"/>
+      <c r="BJ136" s="25" t="n"/>
+      <c r="BK136" s="26" t="n"/>
+      <c r="BL136" s="27" t="n"/>
+      <c r="BM136" s="28" t="n"/>
+      <c r="BN136" s="28" t="n"/>
+      <c r="BO136" s="28" t="n"/>
+      <c r="BP136" s="25" t="n"/>
+      <c r="BQ136" s="27" t="n"/>
+      <c r="BR136" s="28" t="n"/>
+      <c r="BS136" s="28" t="n"/>
+      <c r="BT136" s="28" t="n"/>
+      <c r="BU136" s="25" t="n"/>
+      <c r="BV136" s="29" t="n"/>
+      <c r="BW136" s="24" t="n"/>
+      <c r="BX136" s="30" t="n"/>
+      <c r="BY136" s="27" t="n"/>
+      <c r="BZ136" s="24" t="n"/>
+      <c r="CA136" s="31" t="n"/>
+      <c r="CB136" s="24" t="n"/>
+      <c r="CC136" s="24" t="n"/>
+      <c r="CD136" s="24" t="n"/>
+      <c r="CE136" s="24" t="n"/>
+      <c r="CF136" s="24" t="n"/>
+      <c r="CG136" s="24" t="n"/>
+      <c r="CH136" s="24" t="n"/>
+      <c r="CI136" s="24" t="n"/>
+      <c r="CJ136" s="24" t="n"/>
+      <c r="CK136" s="24" t="n"/>
+      <c r="CL136" s="24" t="n"/>
+      <c r="CM136" s="24" t="n"/>
+      <c r="CN136" s="24" t="n"/>
+      <c r="CO136" s="24" t="n"/>
+      <c r="CP136" s="24" t="n"/>
+      <c r="CQ136" s="24" t="n"/>
+      <c r="CR136" s="24" t="n"/>
+      <c r="CS136" s="24" t="n"/>
+      <c r="CT136" s="24" t="n"/>
+      <c r="CU136" s="24" t="n"/>
+      <c r="CV136" s="24" t="n"/>
+      <c r="CW136" s="24" t="n"/>
+      <c r="CX136" s="24" t="n"/>
+      <c r="CY136" s="24" t="n"/>
+      <c r="CZ136" s="24" t="n"/>
+      <c r="DA136" s="24" t="n"/>
+      <c r="DB136" s="24" t="n"/>
+      <c r="DC136" s="24" t="n"/>
+      <c r="DD136" s="24" t="n"/>
+      <c r="DE136" s="24" t="n"/>
+      <c r="DF136" s="24" t="n"/>
+      <c r="DG136" s="24" t="n"/>
+      <c r="DH136" s="24" t="n"/>
+      <c r="DI136" s="24" t="n"/>
+      <c r="DJ136" s="24" t="n"/>
+      <c r="DK136" s="24" t="n"/>
+      <c r="DL136" s="24" t="n"/>
+      <c r="DM136" s="24" t="n"/>
+      <c r="DN136" s="24" t="n"/>
+      <c r="DO136" s="24" t="n"/>
+      <c r="DP136" s="24" t="n"/>
+    </row>
+    <row r="137" ht="36" customHeight="1">
+      <c r="A137" s="24" t="inlineStr">
+        <is>
+          <t>38dea559c2634cd8</t>
+        </is>
+      </c>
+      <c r="B137" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T07:17:52.157470Z</t>
+        </is>
+      </c>
+      <c r="C137" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T23:30Z</t>
+        </is>
+      </c>
+      <c r="D137" s="24" t="inlineStr">
+        <is>
+          <t>atc-brb-ath-vln-2026-09-04-ath</t>
+        </is>
+      </c>
+      <c r="E137" s="24" t="inlineStr">
+        <is>
+          <t>SOCCER</t>
+        </is>
+      </c>
+      <c r="F137" s="24" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="G137" s="24" t="inlineStr">
+        <is>
+          <t>Athletic</t>
+        </is>
+      </c>
+      <c r="H137" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I137" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J137" s="25" t="n"/>
+      <c r="K137" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L137" s="26" t="n">
+        <v>178</v>
+      </c>
+      <c r="M137" s="27" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="N137" s="28" t="n">
+        <v>0.3704</v>
+      </c>
+      <c r="O137" s="28" t="n">
+        <v>0.4867</v>
+      </c>
+      <c r="P137" s="28" t="n"/>
+      <c r="Q137" s="28" t="n">
+        <v>0.1267</v>
+      </c>
+      <c r="R137" s="26" t="n"/>
+      <c r="S137" s="29" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="T137" s="24" t="inlineStr">
+        <is>
+          <t>soccer-poisson-dc-v1</t>
+        </is>
+      </c>
+      <c r="U137" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V137" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W137" s="26" t="n"/>
+      <c r="X137" s="26" t="n"/>
+      <c r="Y137" s="25" t="n"/>
+      <c r="Z137" s="26" t="n"/>
+      <c r="AA137" s="28" t="n"/>
+      <c r="AB137" s="28" t="n"/>
+      <c r="AC137" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD137" s="24" t="n"/>
+      <c r="AE137" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9G6FV07GMVG on atc-brb-ath-vln-2026-09-04-ath (long)</t>
+        </is>
+      </c>
+      <c r="AF137" s="31" t="n"/>
+      <c r="AG137" s="24" t="n"/>
+      <c r="AH137" s="24" t="n"/>
+      <c r="AI137" s="31" t="n"/>
+      <c r="AJ137" s="31" t="n"/>
+      <c r="AK137" s="24" t="n"/>
+      <c r="AL137" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM137" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN137" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO137" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP137" s="24" t="n"/>
+      <c r="AQ137" s="24" t="n"/>
+      <c r="AR137" s="24" t="n"/>
+      <c r="AS137" s="24" t="n"/>
+      <c r="AT137" s="24" t="n"/>
+      <c r="AU137" s="24" t="n"/>
+      <c r="AV137" s="24" t="n"/>
+      <c r="AW137" s="24" t="n"/>
+      <c r="AX137" s="24" t="n"/>
+      <c r="AY137" s="24" t="n"/>
+      <c r="AZ137" s="24" t="n"/>
+      <c r="BA137" s="24" t="n"/>
+      <c r="BB137" s="24" t="n"/>
+      <c r="BC137" s="24" t="n"/>
+      <c r="BD137" s="24" t="n"/>
+      <c r="BE137" s="24" t="n"/>
+      <c r="BF137" s="24" t="n"/>
+      <c r="BG137" s="24" t="n"/>
+      <c r="BH137" s="24" t="n"/>
+      <c r="BI137" s="24" t="n"/>
+      <c r="BJ137" s="25" t="n"/>
+      <c r="BK137" s="26" t="n"/>
+      <c r="BL137" s="27" t="n"/>
+      <c r="BM137" s="28" t="n"/>
+      <c r="BN137" s="28" t="n"/>
+      <c r="BO137" s="28" t="n"/>
+      <c r="BP137" s="25" t="n"/>
+      <c r="BQ137" s="27" t="n"/>
+      <c r="BR137" s="28" t="n"/>
+      <c r="BS137" s="28" t="n"/>
+      <c r="BT137" s="28" t="n"/>
+      <c r="BU137" s="25" t="n"/>
+      <c r="BV137" s="29" t="n"/>
+      <c r="BW137" s="24" t="n"/>
+      <c r="BX137" s="30" t="n"/>
+      <c r="BY137" s="27" t="n"/>
+      <c r="BZ137" s="24" t="n"/>
+      <c r="CA137" s="31" t="n"/>
+      <c r="CB137" s="24" t="n"/>
+      <c r="CC137" s="24" t="n"/>
+      <c r="CD137" s="24" t="n"/>
+      <c r="CE137" s="24" t="n"/>
+      <c r="CF137" s="24" t="n"/>
+      <c r="CG137" s="24" t="n"/>
+      <c r="CH137" s="24" t="n"/>
+      <c r="CI137" s="24" t="n"/>
+      <c r="CJ137" s="24" t="n"/>
+      <c r="CK137" s="24" t="n"/>
+      <c r="CL137" s="24" t="n"/>
+      <c r="CM137" s="24" t="n"/>
+      <c r="CN137" s="24" t="n"/>
+      <c r="CO137" s="24" t="n"/>
+      <c r="CP137" s="24" t="n"/>
+      <c r="CQ137" s="24" t="n"/>
+      <c r="CR137" s="24" t="n"/>
+      <c r="CS137" s="24" t="n"/>
+      <c r="CT137" s="24" t="n"/>
+      <c r="CU137" s="24" t="n"/>
+      <c r="CV137" s="24" t="n"/>
+      <c r="CW137" s="24" t="n"/>
+      <c r="CX137" s="24" t="n"/>
+      <c r="CY137" s="24" t="n"/>
+      <c r="CZ137" s="24" t="n"/>
+      <c r="DA137" s="24" t="n"/>
+      <c r="DB137" s="24" t="n"/>
+      <c r="DC137" s="24" t="n"/>
+      <c r="DD137" s="24" t="n"/>
+      <c r="DE137" s="24" t="n"/>
+      <c r="DF137" s="24" t="n"/>
+      <c r="DG137" s="24" t="n"/>
+      <c r="DH137" s="24" t="n"/>
+      <c r="DI137" s="24" t="n"/>
+      <c r="DJ137" s="24" t="n"/>
+      <c r="DK137" s="24" t="n"/>
+      <c r="DL137" s="24" t="n"/>
+      <c r="DM137" s="24" t="n"/>
+      <c r="DN137" s="24" t="n"/>
+      <c r="DO137" s="24" t="n"/>
+      <c r="DP137" s="24" t="n"/>
+    </row>
+    <row r="138" ht="36" customHeight="1">
+      <c r="A138" s="24" t="inlineStr">
+        <is>
+          <t>9fd390111ad54428</t>
+        </is>
+      </c>
+      <c r="B138" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T07:17:52.157470Z</t>
+        </is>
+      </c>
+      <c r="C138" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T20:00Z</t>
+        </is>
+      </c>
+      <c r="D138" s="24" t="inlineStr">
+        <is>
+          <t>aec-atp-tometc-marnav-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E138" s="24" t="inlineStr">
+        <is>
+          <t>TENNIS</t>
+        </is>
+      </c>
+      <c r="F138" s="24" t="inlineStr">
+        <is>
+          <t>Mariano Navone</t>
+        </is>
+      </c>
+      <c r="G138" s="24" t="inlineStr">
+        <is>
+          <t>Tomas Martin Etcheverry</t>
+        </is>
+      </c>
+      <c r="H138" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I138" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J138" s="25" t="n"/>
+      <c r="K138" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L138" s="26" t="n">
+        <v>-100</v>
+      </c>
+      <c r="M138" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="N138" s="28" t="n">
+        <v>0.4902</v>
+      </c>
+      <c r="O138" s="28" t="n">
+        <v>0.5485</v>
+      </c>
+      <c r="P138" s="28" t="n"/>
+      <c r="Q138" s="28" t="n">
+        <v>0.0485</v>
+      </c>
+      <c r="R138" s="26" t="n"/>
+      <c r="S138" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T138" s="24" t="inlineStr">
+        <is>
+          <t>tennis-surface-elo-v1</t>
+        </is>
+      </c>
+      <c r="U138" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V138" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="W138" s="26" t="n"/>
+      <c r="X138" s="26" t="n"/>
+      <c r="Y138" s="25" t="n"/>
+      <c r="Z138" s="26" t="n"/>
+      <c r="AA138" s="28" t="n"/>
+      <c r="AB138" s="28" t="n"/>
+      <c r="AC138" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD138" s="24" t="n"/>
+      <c r="AE138" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order C9G5BCN52MVY on aec-atp-tometc-marnav-2026-09-04 (long)</t>
+        </is>
+      </c>
+      <c r="AF138" s="31" t="n"/>
+      <c r="AG138" s="24" t="n"/>
+      <c r="AH138" s="24" t="n"/>
+      <c r="AI138" s="31" t="n"/>
+      <c r="AJ138" s="31" t="n"/>
+      <c r="AK138" s="24" t="n"/>
+      <c r="AL138" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM138" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN138" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO138" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP138" s="24" t="n"/>
+      <c r="AQ138" s="24" t="n"/>
+      <c r="AR138" s="24" t="n"/>
+      <c r="AS138" s="24" t="n"/>
+      <c r="AT138" s="24" t="n"/>
+      <c r="AU138" s="24" t="n"/>
+      <c r="AV138" s="24" t="n"/>
+      <c r="AW138" s="24" t="n"/>
+      <c r="AX138" s="24" t="n"/>
+      <c r="AY138" s="24" t="n"/>
+      <c r="AZ138" s="24" t="n"/>
+      <c r="BA138" s="24" t="n"/>
+      <c r="BB138" s="24" t="n"/>
+      <c r="BC138" s="24" t="n"/>
+      <c r="BD138" s="24" t="n"/>
+      <c r="BE138" s="24" t="n"/>
+      <c r="BF138" s="24" t="n"/>
+      <c r="BG138" s="24" t="n"/>
+      <c r="BH138" s="24" t="n"/>
+      <c r="BI138" s="24" t="n"/>
+      <c r="BJ138" s="25" t="n"/>
+      <c r="BK138" s="26" t="n"/>
+      <c r="BL138" s="27" t="n"/>
+      <c r="BM138" s="28" t="n"/>
+      <c r="BN138" s="28" t="n"/>
+      <c r="BO138" s="28" t="n"/>
+      <c r="BP138" s="25" t="n"/>
+      <c r="BQ138" s="27" t="n"/>
+      <c r="BR138" s="28" t="n"/>
+      <c r="BS138" s="28" t="n"/>
+      <c r="BT138" s="28" t="n"/>
+      <c r="BU138" s="25" t="n"/>
+      <c r="BV138" s="29" t="n"/>
+      <c r="BW138" s="24" t="n"/>
+      <c r="BX138" s="30" t="n"/>
+      <c r="BY138" s="27" t="n"/>
+      <c r="BZ138" s="24" t="n"/>
+      <c r="CA138" s="31" t="n"/>
+      <c r="CB138" s="24" t="n"/>
+      <c r="CC138" s="24" t="n"/>
+      <c r="CD138" s="24" t="n"/>
+      <c r="CE138" s="24" t="n"/>
+      <c r="CF138" s="24" t="n"/>
+      <c r="CG138" s="24" t="n"/>
+      <c r="CH138" s="24" t="n"/>
+      <c r="CI138" s="24" t="n"/>
+      <c r="CJ138" s="24" t="n"/>
+      <c r="CK138" s="24" t="n"/>
+      <c r="CL138" s="24" t="n"/>
+      <c r="CM138" s="24" t="n"/>
+      <c r="CN138" s="24" t="n"/>
+      <c r="CO138" s="24" t="n"/>
+      <c r="CP138" s="24" t="n"/>
+      <c r="CQ138" s="24" t="n"/>
+      <c r="CR138" s="24" t="n"/>
+      <c r="CS138" s="24" t="n"/>
+      <c r="CT138" s="24" t="n"/>
+      <c r="CU138" s="24" t="n"/>
+      <c r="CV138" s="24" t="n"/>
+      <c r="CW138" s="24" t="n"/>
+      <c r="CX138" s="24" t="n"/>
+      <c r="CY138" s="24" t="n"/>
+      <c r="CZ138" s="24" t="n"/>
+      <c r="DA138" s="24" t="n"/>
+      <c r="DB138" s="24" t="n"/>
+      <c r="DC138" s="24" t="n"/>
+      <c r="DD138" s="24" t="n"/>
+      <c r="DE138" s="24" t="n"/>
+      <c r="DF138" s="24" t="n"/>
+      <c r="DG138" s="24" t="n"/>
+      <c r="DH138" s="24" t="n"/>
+      <c r="DI138" s="24" t="n"/>
+      <c r="DJ138" s="24" t="n"/>
+      <c r="DK138" s="24" t="n"/>
+      <c r="DL138" s="24" t="n"/>
+      <c r="DM138" s="24" t="n"/>
+      <c r="DN138" s="24" t="n"/>
+      <c r="DO138" s="24" t="n"/>
+      <c r="DP138" s="24" t="n"/>
+    </row>
+    <row r="139" ht="36" customHeight="1">
+      <c r="A139" s="24" t="inlineStr">
+        <is>
+          <t>PICK_HEALTHY</t>
+        </is>
+      </c>
+      <c r="B139" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T07:26:04.323753Z</t>
+        </is>
+      </c>
+      <c r="C139" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-04T19:26:04.323677Z</t>
+        </is>
+      </c>
+      <c r="D139" s="24" t="inlineStr">
+        <is>
+          <t>aec-cs2-alpha-beta-2026-09-04</t>
+        </is>
+      </c>
+      <c r="E139" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F139" s="24" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="G139" s="24" t="inlineStr">
+        <is>
+          <t>Alpha</t>
+        </is>
+      </c>
+      <c r="H139" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I139" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J139" s="25" t="n"/>
+      <c r="K139" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L139" s="26" t="n">
+        <v>-100</v>
+      </c>
+      <c r="M139" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="N139" s="28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O139" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P139" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q139" s="28" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="R139" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S139" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T139" s="24" t="n"/>
+      <c r="U139" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V139" s="24" t="n"/>
+      <c r="W139" s="26" t="n"/>
+      <c r="X139" s="26" t="n"/>
+      <c r="Y139" s="25" t="n"/>
+      <c r="Z139" s="26" t="n"/>
+      <c r="AA139" s="28" t="n"/>
+      <c r="AB139" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC139" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD139" s="24" t="n"/>
+      <c r="AE139" s="31" t="inlineStr">
+        <is>
+          <t>Auto-Buyer order primary-healthy (0.0 sh @ $0.50) on aec-cs2-alpha-beta-2026-09-04 (long)</t>
+        </is>
+      </c>
+      <c r="AF139" s="31" t="inlineStr">
+        <is>
+          <t>Auto-executed Polymarket US order</t>
+        </is>
+      </c>
+      <c r="AG139" s="24" t="n"/>
+      <c r="AH139" s="24" t="n"/>
+      <c r="AI139" s="31" t="n"/>
+      <c r="AJ139" s="31" t="n"/>
+      <c r="AK139" s="24" t="n"/>
+      <c r="AL139" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM139" s="24" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="AN139" s="24" t="inlineStr">
+        <is>
+          <t>take</t>
+        </is>
+      </c>
+      <c r="AO139" s="24" t="inlineStr">
+        <is>
+          <t>AUTO_BUYER_EXECUTION</t>
+        </is>
+      </c>
+      <c r="AP139" s="24" t="n"/>
+      <c r="AQ139" s="24" t="n"/>
+      <c r="AR139" s="24" t="n"/>
+      <c r="AS139" s="24" t="n"/>
+      <c r="AT139" s="24" t="n"/>
+      <c r="AU139" s="24" t="n"/>
+      <c r="AV139" s="24" t="n"/>
+      <c r="AW139" s="24" t="n"/>
+      <c r="AX139" s="24" t="n"/>
+      <c r="AY139" s="24" t="n"/>
+      <c r="AZ139" s="24" t="n"/>
+      <c r="BA139" s="24" t="n"/>
+      <c r="BB139" s="24" t="n"/>
+      <c r="BC139" s="24" t="n"/>
+      <c r="BD139" s="24" t="n"/>
+      <c r="BE139" s="24" t="n"/>
+      <c r="BF139" s="24" t="n"/>
+      <c r="BG139" s="24" t="n"/>
+      <c r="BH139" s="24" t="n"/>
+      <c r="BI139" s="24" t="n"/>
+      <c r="BJ139" s="25" t="n"/>
+      <c r="BK139" s="26" t="n"/>
+      <c r="BL139" s="27" t="n"/>
+      <c r="BM139" s="28" t="n"/>
+      <c r="BN139" s="28" t="n"/>
+      <c r="BO139" s="28" t="n"/>
+      <c r="BP139" s="25" t="n"/>
+      <c r="BQ139" s="27" t="n"/>
+      <c r="BR139" s="28" t="n"/>
+      <c r="BS139" s="28" t="n"/>
+      <c r="BT139" s="28" t="n"/>
+      <c r="BU139" s="25" t="n"/>
+      <c r="BV139" s="29" t="n"/>
+      <c r="BW139" s="24" t="n"/>
+      <c r="BX139" s="30" t="n"/>
+      <c r="BY139" s="27" t="n"/>
+      <c r="BZ139" s="24" t="n"/>
+      <c r="CA139" s="31" t="n"/>
+      <c r="CB139" s="24" t="n"/>
+      <c r="CC139" s="24" t="n"/>
+      <c r="CD139" s="24" t="n"/>
+      <c r="CE139" s="24" t="n"/>
+      <c r="CF139" s="24" t="n"/>
+      <c r="CG139" s="24" t="n"/>
+      <c r="CH139" s="24" t="n"/>
+      <c r="CI139" s="24" t="n"/>
+      <c r="CJ139" s="24" t="n"/>
+      <c r="CK139" s="24" t="n"/>
+      <c r="CL139" s="24" t="n"/>
+      <c r="CM139" s="24" t="n"/>
+      <c r="CN139" s="24" t="n"/>
+      <c r="CO139" s="24" t="n"/>
+      <c r="CP139" s="24" t="n"/>
+      <c r="CQ139" s="24" t="n"/>
+      <c r="CR139" s="24" t="n"/>
+      <c r="CS139" s="24" t="n"/>
+      <c r="CT139" s="24" t="n"/>
+      <c r="CU139" s="24" t="n"/>
+      <c r="CV139" s="24" t="n"/>
+      <c r="CW139" s="24" t="n"/>
+      <c r="CX139" s="24" t="n"/>
+      <c r="CY139" s="24" t="n"/>
+      <c r="CZ139" s="24" t="n"/>
+      <c r="DA139" s="24" t="n"/>
+      <c r="DB139" s="24" t="n"/>
+      <c r="DC139" s="24" t="n"/>
+      <c r="DD139" s="24" t="n"/>
+      <c r="DE139" s="24" t="n"/>
+      <c r="DF139" s="24" t="n"/>
+      <c r="DG139" s="24" t="n"/>
+      <c r="DH139" s="24" t="n"/>
+      <c r="DI139" s="24" t="n"/>
+      <c r="DJ139" s="24" t="n"/>
+      <c r="DK139" s="24" t="n"/>
+      <c r="DL139" s="24" t="n"/>
+      <c r="DM139" s="24" t="n"/>
+      <c r="DN139" s="24" t="n"/>
+      <c r="DO139" s="24" t="n"/>
+      <c r="DP139" s="24" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>